<commit_message>
docs: capture v2.6 next-branch requirements and roadmap
- DOCX: TZ_Retail_Media_Platform_v2_6_Next_Branch_2026-07-11.docx → docs/product/requirements/
- README: docs/product/requirements/README.md with v2.5/v2.6 context + roadmap ownership rules
- ADR-018: tenant model for next branch (Proposed) — single-retailer vs multi-retailer
- stabilization-tracker: S-024 row + Tenant model ADR gap
- release-versioning: Future branch v2.6 section
- roadmap xlsx: +12 tech rows +10 biz rows for v2.6 (2 sheets preserved, format unchanged)
- No code/schema changes
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1718,6 +1718,318 @@
       <c r="E48" s="3" t="inlineStr">
         <is>
           <t>Prometheus + Grafana after compose → production deploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>SECTION</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>v2.6 Next Branch</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Tenant Model ADR (ADR-018)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>🟡 Decision needed</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ADR-018 proposed 2026-07-11. P0 before v2.6 implementation.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Single-retailer vs multi-retailer decision.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Without decision: rewrite attribution, finance, competitive separation, RLS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Attribution &amp; Sales Lift</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>After tenant model ADR.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Requires PoP pipeline + receipt data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Self-Service Advertiser Cabinet</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>🟠 Foundation only</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>S-023 design gate: backend API ready, tenant isolation proven. apps/advertiser-web planned.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Seed fix: advertiser role, scaffold, campaign list.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Not v2.6 feature. This is TZ v2.5 portal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Competitive Separation</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>After tenant model ADR.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Blocking competitor brands on same screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Store-Level Audience Targeting</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>After tenant model ADR + inventory.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Campaign-to-store-profile targeting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Finance Contract/Invoicing Integration</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>After tenant model ADR.</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1C/ERP API integration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Programmatic Extension Point</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>TZ v2.6. OpenRTB stub.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>After production pilot.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>External DSP/SSP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Dynamic Creative MVP</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>TZ v2.6. HTML5 canvas/video templating.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>After KSO player stable.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Creative personalization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Mobile Field Ops MVP</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Mobile app for field operators.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>After KSO player stable.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Screen checks, content swap in field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>A/B Lift Metrics</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>After attribution.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>A/B testing of creatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Third-Party DOOH Measurement/Accreditation</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Design stub only.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>After production pilot.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Independent impression audit.</t>
         </is>
       </c>
     </row>
@@ -1733,7 +2045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2466,6 +2778,264 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SECTION</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>v2.6 Next Branch</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Self-service advertiser cabinet</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Foundation exists: backend API ready, tenant isolation proven (S-023 design gate). apps/advertiser-web planned.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No separate portal. Admin-web has no role-based routing. No self-service campaign creation.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>S-023a: scaffold advertiser-web + seed fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Sales Lift / Attribution proof</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>No attribution pipeline. No receipt data integration.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>After tenant model ADR + PoP pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Competitor blocking</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>No competitive separation model.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>After tenant model ADR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Store/audience targeting</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>No store profiles. No audience targeting.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>After tenant model ADR + inventory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Financial docs / reconciliation / integration</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>No 1C/ERP API. No invoicing.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>After tenant model ADR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Programmatic inventory sales</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TZ v2.6. OpenRTB stub.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>No DSP/SSP integration.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>After production pilot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Dynamic creatives</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TZ v2.6. HTML5 canvas/video templating.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>No creative templating.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>After KSO player stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Mobile field ops</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Mobile app.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>No mobile client.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>After KSO player stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Independent DOOH measurement</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Design stub only.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>No external impression audit.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>After production pilot.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: harden advertiser portal foundation guards
- test_seed_insert_count: 83→91 (+8 advertiser role INSERTs in S-023a)
- CampaignListPage: typed ApiError (e.status===401/403) instead of message string matching
- ProtectedRoute: add campaigns.read permission guard + AccessDenied component
- vitest: +2 permission guard tests (auth.test.tsx), fix campaign-list 401/403 tests to use mock ApiError class for instanceof
- stabilization-tracker: S-023a row added (seed RBAC + scaffold done)
- roadmap xlsx: advertiser portal → pilot foundation, self-service cabinet → pilot foundation
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1306,17 +1306,17 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟠 Pilot foundation</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.5 requires advertiser self-service portal with read-only campaign/report access.</t>
+          <t>S-023a: seed advertiser role (6 perms), advertiser-web scaffold (React+TS), read-only campaign list. 40 seed tests + 12 vitest.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>After admin-web campaign UI stable (S-009c+)</t>
+          <t>S-023b: campaign detail page</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1732,9 +1732,6 @@
           <t>v2.6 Next Branch</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2789,9 +2786,6 @@
           <t>v2.6 Next Branch</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2801,22 +2795,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🟠 Pilot foundation</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Foundation exists: backend API ready, tenant isolation proven (S-023 design gate). apps/advertiser-web planned.</t>
+          <t>S-023a: scaffold + auth shell + read-only campaign list. Advertiser-web (React+TS, port 3001) exists. Seed: advertiser role with 6 permissions.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>No separate portal. Admin-web has no role-based routing. No self-service campaign creation.</t>
+          <t>Full advertiser portal not done. Campaign detail (S-023b), creative library (S-023c), PoP reporting (S-023d) pending.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>S-023a: scaffold advertiser-web + seed fix.</t>
+          <t>S-023a foundation done. Next: S-023b campaign detail.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add advertiser campaign detail view
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1306,17 +1306,17 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>🟠 Pilot foundation</t>
+          <t>🟡 Pilot read-only detail</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a: seed advertiser role (6 perms), advertiser-web scaffold (React+TS), read-only campaign list. 40 seed tests + 12 vitest.</t>
+          <t>S-023a: seed advertiser role + scaffold. S-023b: CampaignDetailPage — 5 sections (overview, flights, placements, creatives, approvals), 7 API endpoints. Clickable list rows. 17 vitest tests. CI covered.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>S-023b: campaign detail page</t>
+          <t>S-023c: campaign create (advertiser)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>🟠 Foundation only</t>
+          <t>🟡 Pilot read-only</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023 design gate: backend API ready, tenant isolation proven. apps/advertiser-web planned.</t>
+          <t>S-023a/b: seed RBAC + scaffold + read-only campaign detail. 17 vitest + 40 seed tests. Advertiser-web CI covered.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Seed fix: advertiser role, scaffold, campaign list.</t>
+          <t>Campaign create, creative upload, PoP reporting</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">

</xml_diff>

<commit_message>
feat: add advertiser creative library upload
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1306,17 +1306,17 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>🟡 Pilot read-only detail</t>
+          <t>🟡 Pilot creative library/upload</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a: seed advertiser role + scaffold. S-023b: CampaignDetailPage — 5 sections (overview, flights, placements, creatives, approvals), 7 API endpoints. Clickable list rows. 17 vitest tests. CI covered.</t>
+          <t>S-023a: seed + scaffold. S-023b: campaign detail. S-023c: creative library (POST+upload flow), 26 vitest tests. Layout: nav updated.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>S-023c: campaign create (advertiser)</t>
+          <t>S-023d: attach creative to campaign, campaign create</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>🟡 Pilot read-only</t>
+          <t>🟡 Pilot creative library</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023a/b: seed RBAC + scaffold + read-only campaign detail. 17 vitest + 40 seed tests. Advertiser-web CI covered.</t>
+          <t>S-023a-c: RBAC + campaign detail + creative library/upload. 26 vitest + 40 seed tests.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Campaign create, creative upload, PoP reporting</t>
+          <t>Campaign create, attach creative, PoP reporting</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">

</xml_diff>

<commit_message>
feat: add advertiser pop reporting view
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1306,17 +1306,17 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>🟡 Pilot creative library/upload</t>
+          <t>🟡 Pilot reporting / PoP</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a: seed + scaffold. S-023b: campaign detail. S-023c: creative library (POST+upload flow), 26 vitest tests. Layout: nav updated.</t>
+          <t>S-023a-d: RBAC + scaffold + campaign detail + creative library/upload + PoP reporting (summary/by-day/by-surface). 32 vitest + 40 seed tests. Build green.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>S-023d: attach creative to campaign, campaign create</t>
+          <t>S-023e: campaign create (advertiser)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>🟡 Pilot creative library</t>
+          <t>🟡 Pilot PoP reporting</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023a-c: RBAC + campaign detail + creative library/upload. 26 vitest + 40 seed tests.</t>
+          <t>S-023a-d: full advertiser portal — campaigns, creatives, PoP. 32 vitest + 40 seed tests.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Campaign create, attach creative, PoP reporting</t>
+          <t>Campaign create, attach creative</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">

</xml_diff>

<commit_message>
docs: prepare advertiser portal foundation release
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1306,22 +1306,22 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>🟡 Pilot reporting / PoP</t>
+          <t>🟡 Pilot-ready / foundation</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a-d: RBAC + scaffold + campaign detail + creative library/upload + PoP reporting (summary/by-day/by-surface). 32 vitest + 40 seed tests. Build green.</t>
+          <t>S-023a-d: RBAC + scaffold + campaign list/detail + creative library/upload + PoP reporting. 32 vitest + 40 seed tests. CI #29159995308 green.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>S-023e: campaign create (advertiser)</t>
+          <t>Tag v0.3-advertiser-portal-foundation pending approval</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Separate React app or route group.</t>
+          <t>Not yet: campaign create/edit, attach creative, submit approval, profile page, password change.</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023a-d: full advertiser portal — campaigns, creatives, PoP. 32 vitest + 40 seed tests.</t>
+          <t>S-023a-d: full advertiser portal — campaigns list/detail, creatives library/upload, PoP reporting. 32 vitest + 40 seed tests. CI #29159995308.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Not v2.6 feature. This is TZ v2.5 portal.</t>
+          <t>Not v2.6 feature. This is TZ v2.5 portal. Next: campaign create (S-023e).</t>
         </is>
       </c>
     </row>
@@ -2163,23 +2163,22 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟡 Pilot-ready / foundation</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Advertiser-web: вход, список кампаний, деталь кампании, библиотека креативов, загрузка медиа, PoP отчёты. Только local_advertiser (bcrypt).</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Фронтенд рекламодателя отсутствует полностью.
-ТЗ требует: read-only доступ к своим кампаниям и отчётам.</t>
+          <t>Создание/редактирование кампаний, отправка на согласование, профиль организации, смена пароля. LDAPS не подключён.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>После стабилизации admin-web (S-009c+).</t>
+          <t>S-023e: campaign create (advertiser). После: attach creative, submit approval, profile page.</t>
         </is>
       </c>
     </row>
@@ -2421,16 +2420,14 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Backend API: GET pop/{summary,by-day,by-surface}.
-Admin-web UI: вкладка «PoP-отчёт» на странице кампании — сводка, график по дням, таблица по поверхностям.
-Scoped: рекламодатель видит только свои кампании.</t>
+          <t>Backend API: GET pop/{summary,by-day,by-surface}. Admin-web: вкладка «PoP-отчёты». Advertiser-web: секция Отчётность в детали кампании.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Нет UI для отчётов.
-Нет экспорта PDF/XLSX/CSV.
-Нет дашборда сети (ТЗ §15.1).</t>
+          <t>Нет экспорта PDF/XLSX/CSV.
+Нет дашборда сети (ТЗ §15.1).
+Нет ClickHouse / materialized views.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -2795,22 +2792,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>🟠 Pilot foundation</t>
+          <t>🟡 Pilot-ready / foundation</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>S-023a: scaffold + auth shell + read-only campaign list. Advertiser-web (React+TS, port 3001) exists. Seed: advertiser role with 6 permissions.</t>
+          <t>S-023a-d: advertiser-web — campaign list/detail, creative library/upload, PoP reporting. 32 vitest tests. CI green.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Full advertiser portal not done. Campaign detail (S-023b), creative library (S-023c), PoP reporting (S-023d) pending.</t>
+          <t>Campaign create/edit from advertiser portal. Attach creative to campaign. Submit approval. Profile page. Password change.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>S-023a foundation done. Next: S-023b campaign detail.</t>
+          <t>Next: S-023e campaign create. Then attach creative, submit approval, profile page, password change.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: track S-023e profile/password change
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1311,17 +1311,17 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a-d: RBAC + scaffold + campaign list/detail + creative library/upload + PoP reporting. 32 vitest + 40 seed tests. CI #29159995308 green.</t>
+          <t>S-023a-e: RBAC + scaffold + campaign list/detail + creative library/upload + PoP reporting + profile/password change. 45 vitest + 40 seed + 5 backend auth tests. CI #29161617184 green.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Tag v0.3-advertiser-portal-foundation pending approval</t>
+          <t>S-023f: campaign create (advertiser)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Not yet: campaign create/edit, attach creative, submit approval, profile page, password change.</t>
+          <t>Not yet: campaign create/edit, attach creative, submit approval.</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023a-d: full advertiser portal — campaigns list/detail, creatives library/upload, PoP reporting. 32 vitest + 40 seed tests. CI #29159995308.</t>
+          <t>S-023a-e: advertiser-web — login, campaigns, creatives, PoP, profile, password change. 45 vitest tests. CI #29161617184.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Not v2.6 feature. This is TZ v2.5 portal. Next: campaign create (S-023e).</t>
+          <t>Next: campaign create (S-023f). Then attach creative, submit approval.</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Advertiser-web: вход, список кампаний, деталь кампании, библиотека креативов, загрузка медиа, PoP отчёты. Только local_advertiser (bcrypt).</t>
+          <t>Advertiser-web: вход, список/деталь кампаний, библиотека креативов, загрузка медиа, PoP отчёты, профиль организации, смена пароля.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>S-023e: campaign create (advertiser). После: attach creative, submit approval, profile page.</t>
+          <t>S-023f: campaign create. После: attach creative, submit approval.</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>S-023a-d: advertiser-web — campaign list/detail, creative library/upload, PoP reporting. 32 vitest tests. CI green.</t>
+          <t>S-023a-e: advertiser-web — login, campaign list/detail, creative library/upload, PoP reporting, profile/password change. 45 vitest tests.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Next: S-023e campaign create. Then attach creative, submit approval, profile page, password change.</t>
+          <t>Next: S-023f campaign create.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: track S-023f campaign create/edit
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1311,17 +1311,17 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a-e: RBAC + scaffold + campaign list/detail + creative library/upload + PoP reporting + profile/password change. 45 vitest + 40 seed + 5 backend auth tests. CI #29161617184 green.</t>
+          <t>S-023a-f: RBAC + scaffold + campaign list/detail + creative library/upload + PoP + profile/password + create/edit drafts. 53 vitest + 40 seed + 5 backend. CI #29162245072.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>S-023f: campaign create (advertiser)</t>
+          <t>S-023g: attach creative + submit approval</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Not yet: campaign create/edit, attach creative, submit approval.</t>
+          <t>Not yet: attach creative, submit approval.</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023a-e: advertiser-web — login, campaigns, creatives, PoP, profile, password change. 45 vitest tests. CI #29161617184.</t>
+          <t>S-023a-f: advertiser-web — login, campaigns CRUD, creatives, PoP, profile, password. 53 vitest tests. CI #29162245072.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Next: campaign create (S-023f). Then attach creative, submit approval.</t>
+          <t>Next: attach creative + submit approval (S-023g).</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Advertiser-web: вход, список/деталь кампаний, библиотека креативов, загрузка медиа, PoP отчёты, профиль организации, смена пароля.</t>
+          <t>Advertiser-web: вход, кампании (список, деталь, создание, редактирование черновиков), библиотека креативов, загрузка, PoP, профиль, смена пароля.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>S-023f: campaign create. После: attach creative, submit approval.</t>
+          <t>S-023g: attach creative + submit approval.</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>S-023a-e: advertiser-web — login, campaign list/detail, creative library/upload, PoP reporting, profile/password change. 45 vitest tests.</t>
+          <t>S-023a-f: advertiser-web — login, campaign list/detail/create/edit drafts, creative library/upload, PoP, profile/password change. 53 vitest tests.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Next: S-023f campaign create.</t>
+          <t>Next: S-023g attach creative + submit approval.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: track S-023g attach creative and submit approval
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1306,22 +1306,22 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / foundation</t>
+          <t>🟡 Core pilot flow complete</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a-f: RBAC + scaffold + campaign list/detail + creative library/upload + PoP + profile/password + create/edit drafts. 53 vitest + 40 seed + 5 backend. CI #29162245072.</t>
+          <t>S-023a-g: RBAC + scaffold + campaign list/detail + creative library/upload + PoP + profile/password + create/edit drafts + attach creative + submit approval. 66 vitest + 40 seed + 5 backend. CI #29162925840 (core pilot flow complete).</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>S-023g: attach creative + submit approval</t>
+          <t>Production UX/accessibility polish, browser E2E</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Not yet: attach creative, submit approval.</t>
+          <t>Advertiser self-service MVP: login → create campaign → upload creative → attach to campaign → submit for approval. Not production-complete (no UX polish, no admin approval UI for advertiser).</t>
         </is>
       </c>
     </row>
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>🟡 Pilot PoP reporting</t>
+          <t>🟡 Core pilot flow complete</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023a-f: advertiser-web — login, campaigns CRUD, creatives, PoP, profile, password. 53 vitest tests. CI #29162245072.</t>
+          <t>S-023a-g: advertiser-web — login, campaigns CRUD, creatives, PoP, profile, password, attach creative, submit approval. 66 vitest tests. CI #29162925840.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Campaign create, attach creative</t>
+          <t>Production UX, browser E2E, admin approval UI for advertiser</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">

</xml_diff>

<commit_message>
docs: refresh roadmap and release status after advertiser self-service pilot
- stabilization-tracker: add S-023e/h/i rows, update header, remaining gaps
- release-versioning: add v0.4-advertiser-self-service-pilot (proposed, tag not created)
- roadmap xlsx: update Advertiser Portal, Creative Upload, Личный кабинет, etc.
- Roadmap: add Local Preview row (S-026b), preserve 2-sheet structure
- No code changes
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -925,7 +925,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Pilot: CREATIVE_AUTO_APPROVE_UPLOADS=true. Approval gate requires real upload.</t>
+          <t>Advertiser-web upload UI shipped (S-023c). Admin-web upload UI already shipped (S-017).</t>
         </is>
       </c>
     </row>
@@ -1306,22 +1306,22 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>🟡 Core pilot flow complete</t>
+          <t>🟡 Pilot-ready / self-service pilot</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>S-023a-g: RBAC + scaffold + campaign list/detail + creative library/upload + PoP + profile/password + create/edit drafts + attach creative + submit approval. 66 vitest + 40 seed + 5 backend. CI #29162925840 (core pilot flow complete).</t>
+          <t>S-023a-i (login, campaigns CRUD, creatives, upload, attach, submit, PoP, profile/password, responsive layout). CI #29166816518. 66 vitest tests. Live LAN preview at http://192.168.110.77:3001.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Production UX/accessibility polish, browser E2E</t>
+          <t>Production UX/accessibility, browser E2E</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Advertiser self-service MVP: login → create campaign → upload creative → attach to campaign → submit for approval. Not production-complete (no UX polish, no admin approval UI for advertiser).</t>
+          <t>Advertiser self-service pilot: login → create campaign → upload creative → attach → submit for approval. No admin approval UI for advertiser. No billing/attribution.</t>
         </is>
       </c>
     </row>
@@ -1724,127 +1724,127 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SECTION</t>
+          <t>Local Preview (S-026b)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>v2.6 Next Branch</t>
+          <t>✅ Done / LAN preview</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>docker-compose.preview.yml override. Runbook: docs/runbook/local-preview.md. Preview URLs: admin-web :3000, advertiser-web :3001, control-api :8000, device-gateway :8001.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>systemd/pm2 persistence for preview processes</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LAN-only preview (192.168.110.77). Not public internet. Dev credentials from seed.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tenant Model ADR (ADR-018)</t>
+          <t>SECTION</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>🟡 Decision needed</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>ADR-018 proposed 2026-07-11. P0 before v2.6 implementation.</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Single-retailer vs multi-retailer decision.</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Without decision: rewrite attribution, finance, competitive separation, RLS.</t>
+          <t>v2.6 Next Branch</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Attribution &amp; Sales Lift</t>
+          <t>Tenant Model ADR (ADR-018)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🟡 Decision needed</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>ADR-018 proposed 2026-07-11. P0 before v2.6 implementation.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>Single-retailer vs multi-retailer decision.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Requires PoP pipeline + receipt data.</t>
+          <t>Without decision: rewrite attribution, finance, competitive separation, RLS.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Self-Service Advertiser Cabinet</t>
+          <t>Attribution &amp; Sales Lift</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>🟡 Core pilot flow complete</t>
+          <t>⚪ Not started</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S-023a-g: advertiser-web — login, campaigns CRUD, creatives, PoP, profile, password, attach creative, submit approval. 66 vitest tests. CI #29162925840.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Production UX, browser E2E, admin approval UI for advertiser</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Next: attach creative + submit approval (S-023g).</t>
+          <t>Requires PoP pipeline + receipt data.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Competitive Separation</t>
+          <t>Self-Service Advertiser Cabinet</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🟡 Core pilot flow complete</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>S-023a-g: advertiser-web — login, campaigns CRUD, creatives, PoP, profile, password, attach creative, submit approval. 66 vitest tests. CI #29162925840.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>Production UX, browser E2E, admin approval UI for advertiser</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Blocking competitor brands on same screen.</t>
+          <t>Next: attach creative + submit approval (S-023g).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Store-Level Audience Targeting</t>
+          <t>Competitive Separation</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1859,19 +1859,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>After tenant model ADR + inventory.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Campaign-to-store-profile targeting.</t>
+          <t>Blocking competitor brands on same screen.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Finance Contract/Invoicing Integration</t>
+          <t>Store-Level Audience Targeting</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1886,46 +1886,46 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>After tenant model ADR + inventory.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1C/ERP API integration.</t>
+          <t>Campaign-to-store-profile targeting.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Programmatic Extension Point</t>
+          <t>Finance Contract/Invoicing Integration</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>⚪ Not started</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>TZ v2.6. OpenRTB stub.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>After production pilot.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>External DSP/SSP.</t>
+          <t>1C/ERP API integration.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Dynamic Creative MVP</t>
+          <t>Programmatic Extension Point</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1935,24 +1935,24 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>TZ v2.6. HTML5 canvas/video templating.</t>
+          <t>TZ v2.6. OpenRTB stub.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>After KSO player stable.</t>
+          <t>After production pilot.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Creative personalization.</t>
+          <t>External DSP/SSP.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Mobile Field Ops MVP</t>
+          <t>Dynamic Creative MVP</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>TZ v2.6. Mobile app for field operators.</t>
+          <t>TZ v2.6. HTML5 canvas/video templating.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1972,59 +1972,86 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Screen checks, content swap in field.</t>
+          <t>Creative personalization.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>A/B Lift Metrics</t>
+          <t>Mobile Field Ops MVP</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚫 Deferred</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>TZ v2.6. Mobile app for field operators.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>After attribution.</t>
+          <t>After KSO player stable.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>A/B testing of creatives.</t>
+          <t>Screen checks, content swap in field.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>A/B Lift Metrics</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Future v2.6.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>After attribution.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>A/B testing of creatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>Third-Party DOOH Measurement/Accreditation</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>🚫 Deferred</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>TZ v2.6. Design stub only.</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Independent impression audit.</t>
         </is>
@@ -2163,22 +2190,22 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / foundation</t>
+          <t>🟡 Pilot-ready / self-service pilot</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Advertiser-web: вход, кампании (список, деталь, создание, редактирование черновиков), библиотека креативов, загрузка, PoP, профиль, смена пароля.</t>
+          <t>Advertiser-web: вход, кампании (список, деталь, создание/редактирование черновиков), библиотека креативов + загрузка, привязка креативов, отправка на согласование, PoP-отчётность, профиль организации, смена пароля. Responsive layout (desktop + планшет). 66 vitest тестов. Live LAN preview.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Создание/редактирование кампаний, отправка на согласование, профиль организации, смена пароля. LDAPS не подключён.</t>
+          <t>Нет кнопок approve/reject (только admin). Нет биллинга/атрибуции. Нет production UX-аудита. Нет мобильной версии. Нет LDAPS.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>S-023g: attach creative + submit approval.</t>
+          <t>S-023a-i завершены. Pilot-ready для демо заказчику в LAN.</t>
         </is>
       </c>
     </row>
@@ -2211,13 +2238,8 @@
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Backend API: полный CRUD кампаний (7 endpoints).
-Admin-web UI: список кампаний с фильтром по статусу, мастер создания (выбор рекламодателя/бренда/контракта, часовой пояс), страница кампании с 5 вкладками:
-• Пролёты — создание и редактирование
-• Размещения — привязка к display surfaces
-• Креативы — привязка + загрузка файлов
-• Согласование — request/approve/reject
-• PoP-отчёты — summary, по дням, по поверхностям
-64 vitest теста.</t>
+Admin-web UI: список кампаний с фильтром, мастер создания, страница с 5 вкладками.
+Advertiser-web: создание/редактирование черновиков через отдельный порт.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -2231,7 +2253,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>S-009c: подключить campaign list/detail к реальным API.</t>
+          <t>Advertiser self-service create/edit работает (S-023f).</t>
         </is>
       </c>
     </row>
@@ -2248,13 +2270,14 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Backend: request-approval → approve/reject. Полный audit trail.
-Admin-web UI: вкладка «Согласование» на странице кампании — кнопки «Отправить», «Утвердить», «Отклонить» с модальным окном.Лог статусов с датами и причинами.</t>
+          <t>Backend: request-approval → approve/reject с audit trail.
+Admin-web: approve/reject UI.
+Advertiser-web: отправка на согласование (S-023g). Advertiser не может approve/reject.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>UI approval не реализован (нет кнопок «Отправить на согласование» / «Утвердить» / «Отклонить»).</t>
+          <t>Advertiser может только отправить; утверждает/отклоняет admin.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2276,18 +2299,14 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Backend: presigned URL (MinIO/S3) с серверной проверкой SHA-256.
-Admin-web UI: кнопка «Загрузить файл», прогресс-бар.
-Безопасность: storage_bucket/key не экспозятся.
-Пилотное авто-одобрение (CREATIVE_AUTO_APPROVE_UPLOADS=true).</t>
+          <t>Backend: presigned URL (MinIO/S3) + SHA-256.
+Admin-web UI: загрузка с прогресс-баром.
+Advertiser-web: библиотека + загрузка + привязка к кампании (S-023c, S-023g).</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Нет проверки на вирусы (malware scan).
-Нет ручной модерации креативов.
-Нет транскодирования и CDN.
-Файлы загружаются только через admin-web (нет рекламодательского портала).</t>
+          <t>Malware scan, transcoding, CDN — отложены.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -2420,7 +2439,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Backend API: GET pop/{summary,by-day,by-surface}. Admin-web: вкладка «PoP-отчёты». Advertiser-web: секция Отчётность в детали кампании.</t>
+          <t>Backend: GET pop/{summary,by-day,by-surface}. Admin-web: вкладка PoP-отчёты. Advertiser-web: секция Отчётность в детали кампании.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -2792,22 +2811,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / foundation</t>
+          <t>🟡 Pilot-ready / self-service pilot</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>S-023a-f: advertiser-web — login, campaign list/detail/create/edit drafts, creative library/upload, PoP, profile/password change. 53 vitest tests.</t>
+          <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Campaign create/edit from advertiser portal. Attach creative to campaign. Submit approval. Profile page. Password change.</t>
+          <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Next: S-023g attach creative + submit approval.</t>
+          <t>S-023a-i completed. Pilot-ready for demo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: triage production gaps after v0.4 pilot (S-029)
- New: docs/product/production-gaps-triage.md — 8 categories, 35+ gaps, P0–P3
- Recommended milestones: v0.5 (P0 ops) → v0.6 (identity) → v0.7 (moderation)
- Roadmap xlsx: +11 production gap rows (CI, backups, secrets, LDAPS, etc.)
- stabilization-tracker: +S-029 entry (docs/triage done)
- No code changes. Branch: develop.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>⚪ Not started (triaged)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>No Prometheus metrics. No alert rules. No Grafana dashboards.</t>
+          <t>v0.5 P0 gates: Prometheus + Grafana + AlertManager</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -2054,6 +2054,303 @@
       <c r="E61" t="inlineStr">
         <is>
           <t>Independent impression audit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Production Gaps Triage (S-029)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>✅ Docs/triage done</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>docs/product/production-gaps-triage.md. 8 categories, 35+ gaps prioritised. develop branch.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Start v0.5 P0 gates (CI, secrets, backups, monitoring)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>No code changes. Docs-only triage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Production CI Gate</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CI exists (33 jobs). Production config validation missing.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Add ENVIRONMENT=production validation, fail on weak secrets</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>P0 — blocks all further releases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Backup / Restore / DR</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>No automated PostgreSQL backups. No MinIO mirroring. No DR plan.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>pg_dump cron + restore runbook + test drill</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>P0 — data safety.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Secrets Management</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>.env.example exists. Production secrets not enforced.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>SECRET_* validation in production mode. Rotation runbook.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>P0 — security baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Identity Hardening (LDAPS)</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>AD stub returns 503. No real LDAPS integration.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Wire real AD adapter. Replace stub.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>P1 — blocks real admin access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Password Reset / Advertiser Invite</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>No self-service password reset. No invite flow.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Email-based reset token. Admin invite → set password.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>P1 — blocks advertiser self-onboarding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Creative Moderation (Manual)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CREATIVE_AUTO_APPROVE_UPLOADS=true. No human review.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Admin-web moderation queue. Approve/reject with reason.</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>P1 — quality control before live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Malware Scan</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Uploaded files unverified.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ClamAV on upload complete. Quarantine on detection.</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>P1 — security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Reporting Export (CSV/XLSX)</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>PoP data API-only. No offline export.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Export endpoints: GET /api/v1/identity/campaigns/{id}/pop/export</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>P1 — customer-facing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ClickHouse Foundation</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ADR-007: deferred to Phase 4+. Container exists, not wired.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ClickHouse deployment + PoP data replication</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>P1 — analytical performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Device / Player Readiness</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Manifest endpoint ready. Simulator proven. No real player.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Real KSO player. Manifest verification on device. Offline fail-closed.</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>P1 — first channel live.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: replace admin advertisers stub with real organization page
Backend:
- 6 new endpoints: org detail, filtered brands/contracts/contacts by org, user memberships
- Auth: advertisers.read/contacts.read + RLS on all endpoints
- Repository: 4 new functions filtered by org_id, memberships join with User+LocalCredential
- Schemas: AdvertiserUserMembershipOut, AdvertiserOrganizationDetailOut

Frontend (admin-web):
- AdvertisersPage: replaces stub with real page
- Org list: table with search, brand/contract/contact counts
- Detail panel: 5 tabs (Overview, Brands, Contracts, Contacts, Users)
- Types: AdvertiserContactOut, AdvertiserUserMembershipOut, AdvertiserOrganizationDetailOut
- Labels: contactTypeLabel, authProviderLabel

Tests: 17 backend + 7 admin-web vitest
All regression green. Import boundaries clean.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1289,7 +1289,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Advertisers page (placeholder → real). Polish/UX/accessibility. Browser E2E.</t>
+          <t>Polish/UX/accessibility. Browser E2E.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -2742,8 +2742,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Нет страницы рекламодателей (заглушка).
-Нет календаря планирования.
+          <t>Нет календаря планирования.
 Нет drag-and-drop.
 UX/accessibility не завершены.
 Нет браузерных E2E-тестов.</t>

</xml_diff>

<commit_message>
docs: prepare v0.5 business portal release
- release-versioning.md: add v0.5-business-portal-complete section
  with full capabilities, technical summary, known limitations,
  rollback notes, and proposed tag SHA (5c41a6a — last code baseline)
- production-gaps-triage.md: update baseline to v0.5 (SHA, test
  counts, CI status), mark v0.5 P0 gates closed (S-030/S-031),
  refresh recommendation section
- roadmap-s020.xlsx: update v0.5 milestone rows — admin user
  management, AD settings, creative moderation, inventory UI,
  campaign approval, advertiser cabinet, PoP CSV export,
  KSO blocker cleared. 2 sheets preserved.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1348,17 +1348,17 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>⚪ Не начато (v0.7)</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ADR-013: edge safety architecture locked. Runtime simulator: 41 safety proofs. Device Gateway ready.</t>
+          <t>ADR-013: edge safety architecture locked. Runtime simulator: 41 safety proofs. Device-gateway: GET /manifest/latest. ✅ v0.5 Business Portal Complete — blocker cleared.</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Real KSO player binary/wrapper. Hardware integration (ServPlus Sherman-J 5.1 + СуперМаг УКМ 4). ⛔ AFTER v0.5 Business Portal Complete.</t>
+          <t>Real KSO player binary. Hardware (ServPlus Sherman-J 5.1 + СуперМаг УКМ 4). Player is v0.7 milestone.</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1552,17 +1552,17 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟡 CSV done (S-040), XLSX deferred</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>TZ requires export for reports.</t>
+          <t>CSV export endpoint: GET /api/v1/identity/campaigns/{id}/pop/export. UTF-8 BOM, Russian headers. Admin + advertiser download buttons.</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Real KSO player binary/wrapper. Hardware integration (ServPlus Sherman-J 5.1 + СуперМаг УКМ 4). AFTER v0.5 Business Portal Complete.</t>
+          <t>XLSX export deferred (openpyxl dependency). PDF deferred.</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -1756,7 +1756,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Milestone: v0.5 Business Portal Complete (before KSO/Player)</t>
+          <t>✅ v0.5 complete (2026-07-13)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>S-042 readiness review: CONDITIONAL GO. S-042a tracker refreshed. S-043 release prep docs.</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1773,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>✅ S-033 done</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>No admin UI for user CRUD. Users only via seed/API. No lock/deactivate. No operator/scopes management.</t>
+          <t>Admin-web UsersPage: create/deactivate/reset. Backend: 5 user management endpoints with users.read/manage permissions. users.manage for activation/deactivation.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Manual account CRUD. Lock/deactivate/reset password. Roles/permissions/scopes assignment UI. Operational audit log view.</t>
+          <t>Production: real LDAPS, password reset invite/email (v0.6)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1795,17 +1800,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>🟡 AD stub only (honest 503)</t>
+          <t>✅ S-034 done (honest stub)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AD stub returns honest 503. No settings screen. No connection test. No status display.</t>
+          <t>Admin-web ADSettingsPage. GET/POST /auth/ad-settings with users.manage. Honest stub/disabled/configured status reporting. No secrets in responses.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Admin settings screen: AD config (without secrets), connection test button, current status. Honest current-state display.</t>
+          <t>Real LDAPS wiring deferred to v0.6+.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1822,17 +1827,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>✅ S-036 done</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Backend: CREATIVE_AUTO_APPROVE_UPLOADS=true. No human review. Uploaded creatives auto-approved.</t>
+          <t>Backend: GET moderation-queue, POST approve/reject with creatives.moderate permission. Admin-web: CreativeModerationPage. Advertiser-web: moderation status display. creative_auto_approve_uploads=False.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Admin moderation queue. Approve/reject with reason. Moderation history. Resubmit/re-upload after rejection. Pending/rejected creatives blocked from campaign approval.</t>
+          <t>Malware scan deferred to v0.7.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1849,17 +1854,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>✅ S-037 done</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>display_surfaces, stores, clusters exist in DB via seed only. No admin UI. Placements use manual UUID entry.</t>
+          <t>Backend: stores/surfaces endpoints with inventory.read/inventory.manage. Admin-web: InventoryPage — stores/surfaces tabs, search, active/inactive toggle.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Admin UI: stores list, zones, display surfaces, ad placements. Active/inactive status. Dimensions/capabilities. Campaign placements reference real inventory, not manual UUIDs.</t>
+          <t>Real inventory/forecasting calculation deferred.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1876,17 +1881,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready</t>
+          <t>✅ S-038 done</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Backend: request-approval/approve/reject with audit. Admin-web: approve/reject buttons. Advertiser: submit only.</t>
+          <t>Backend: GET /campaigns/approval-queue with readiness summary. Admin-web: ApprovalInboxPage — approve/reject with readiness checklist + creative moderation gate.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Advertiser resubmit after rejection. Rejection reason visible in advertiser UI. Role-based approve/reject. Approval history with comments.</t>
+          <t>Advertiser resubmit after rejection (v0.6).</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -1903,17 +1908,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready</t>
+          <t>✅ Done (S-039, S-023h-i)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>S-023a-i: login, campaigns CRUD, creatives, upload, attach, submit, PoP, profile, password. 66 tests. Responsive 768px.</t>
+          <t>Admin-web: AdvertisersPage — org list + 5-tab detail panel. Advertiser-web: Russian localization, responsive layout, CSS modules, hamburger sidebar. S-042 readiness review: CONDITIONAL GO.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Production UX audit. Browser E2E tests (Playwright). 390px mobile validation. Accessibility baseline (WCAG AA lite). Date/time picker localization.</t>
+          <t>Production UX audit deferred.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -1930,17 +1935,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>✅ CSV done, XLSX deferred (S-040)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>PoP data via API only. No offline export. No PDF/XLSX/CSV download.</t>
+          <t>Backend: GET /campaigns/{id}/pop/export — CSV UTF-8 BOM, Russian headers. Admin-web + advertiser-web: «Скачать CSV» buttons. Same auth/RBAC/RLS as JSON endpoints.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Export endpoints: campaign PoP as CSV/XLSX. Report templating. Note: real impressions depend on player (v0.7).</t>
+          <t>XLSX export deferred (no openpyxl in project).</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2688,22 +2693,22 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / self-service pilot</t>
+          <t>✅ Done / v0.5 Ready for RC</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Advertiser-web: вход, кампании (список, деталь, создание/редактирование черновиков), библиотека креативов + загрузка, привязка креативов, отправка на согласование, PoP-отчётность, профиль организации, смена пароля. Responsive layout (desktop + планшет). 66 vitest тестов. Live LAN preview.</t>
+          <t>Advertiser-web: вход, кампании (список, деталь, создание/редактирование черновиков), креативы (библиотека, загрузка, прикрепление), отправка на согласование, видимость статуса/причины отклонения, PoP-отчёты + CSV экспорт, профиль/смена пароля. Admin-web: полное управление. S-042 CONDITIONAL GO.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Нет кнопок approve/reject (только admin). Нет биллинга/атрибуции. Нет production UX-аудита. Нет мобильной версии. Нет LDAPS.</t>
+          <t>Нет кнопок approve/reject (только admin). Нет биллинга/атрибуции. Production UX audit deferred.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>S-023a-i завершены. Pilot-ready для демо заказчику в LAN.</t>
+          <t>Production UX audit (deferred). Browser E2E (deferred).</t>
         </is>
       </c>
     </row>
@@ -2974,22 +2979,22 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>⚪ Не начато (v0.7, ✅ v0.5 Business Portal done)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Архитектура зафиксирована (ADR-013, ADR-016). Симулятор: 41 тест доказывает безопасность. Manifest API готов. BACKEND-ПИЛОТ ЗАВЕРШЁН.</t>
+          <t>Архитектура зафиксирована (ADR-013, ADR-016). Симулятор: 41 тест. Device-gateway: GET /manifest/latest. ✅ v0.5 Business Portal Complete — blocker cleared. KSO/player — v0.7 milestone.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Реального KSO плеера нет. Нет интеграции с железом КСО (ServPlus Sherman-J 5.1 + СуперМаг УКМ 4). ⛔ ЗАБЛОКИРОВАНО до v0.5 Business Portal Complete.</t>
+          <t>Реального KSO плеера нет. Нет интеграции с железом КСО.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>KSO/Player — v0.7. После полного business portal (v0.5). Реальные показы недоступны до v0.7.</t>
+          <t>KSO после v0.6 production hardening.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: plan v0.6 production readiness milestone
- New: docs/product/v06-production-readiness-plan.md
  Scope: monitoring, LDAPS, MinIO/NATS backup, error boundaries,
  audit events, router decomposition, RLS test, XLSX decision.
  Out of scope: KSO/player, Emergency Mgmt, Feature Flags,
  Inventory Planning, ClickHouse, v2.6.
  S-ticket sequence: S-047 → S-048 → ... → S-055.
- release-versioning.md: mark v0.5 as Published, add v0.6
  Production Readiness Foundation section.
- stabilization-tracker.md: add S-042a..S-046 rows, refresh
  Remaining Gaps section for v0.6 planned items.
- roadmap-s020.xlsx: update existing rows (observability,
  DR/backup, LDAPS) + add v0.6 milestone section with 8 new
  rows in Технический Roadmap. Sheets preserved.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Real LDAPS wiring (not in pilot)</t>
+          <t>Real LDAPS wiring (v0.6, S-048)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟡 PostgreSQL: S-031 done. MinIO/NATS: 🚧 v0.6 planned (S-049/S-050)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>No automated PostgreSQL backups. No MinIO mirroring. No DR plan.</t>
+          <t>MinIO mirror + restore drill (S-049). NATS backup policy (S-050).</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>⚪ Not started (triaged)</t>
+          <t>🚧 v0.6 planned (S-047)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>v0.5 P0 gates: Prometheus + Grafana + AlertManager</t>
+          <t>Prometheus + Grafana + AlertManager (v0.6)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
@@ -1962,257 +1962,247 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>v2.6 Next Branch</t>
+          <t>Milestone: v0.6 Production Readiness (planned)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>S-046 plan: docs/product/v06-production-readiness-plan.md</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tenant Model ADR (ADR-018)</t>
+          <t>Monitoring / Observability</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>🟡 Decision needed</t>
+          <t>🚧 v0.6 planned (S-047)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ADR-018 proposed 2026-07-11. P0 before v2.6 implementation.</t>
+          <t>Prometheus metrics on control-api + device-gateway. Grafana: API, DB, NATS, outbox panels. AlertManager rules.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Single-retailer vs multi-retailer decision.</t>
+          <t>Implement S-047</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Without decision: rewrite attribution, finance, competitive separation, RLS.</t>
+          <t>P0 — blocks production deployment confidence.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Attribution &amp; Sales Lift</t>
+          <t>Real LDAPS Wiring</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚧 v0.6 planned (S-048)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>Replace AD stub with real LDAPS bind/search. AD_LDAP_URL/BIND_DN/SEARCH_BASE env vars. Fail-safe to local_break_glass.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>Implement S-048</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Requires PoP pipeline + receipt data.</t>
+          <t>P0 — blocks real admin access.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Self-Service Advertiser Cabinet</t>
+          <t>MinIO Backup (S3 Mirror)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>🟡 Core pilot flow complete</t>
+          <t>🚧 v0.6 planned (S-049)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>S-023a-g: advertiser-web — login, campaigns CRUD, creatives, PoP, profile, password, attach creative, submit approval. 66 vitest tests. CI #29162925840.</t>
+          <t>mc mirror cron for creative assets bucket. Restore drill + runbook update.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Production UX, browser E2E, admin approval UI for advertiser</t>
+          <t>Implement S-049</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Next: attach creative + submit approval (S-023g).</t>
+          <t>P0 — data safety for creative assets.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Competitive Separation</t>
+          <t>NATS Backup Policy</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚧 v0.6 planned (S-050)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>NATS state recoverable from outbox. Manual nats stream backup procedure.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>Document S-050</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Blocking competitor brands on same screen.</t>
+          <t>P1 — DR completeness.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Store-Level Audience Targeting</t>
+          <t>Portal Error Boundaries</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚧 v0.6 planned (S-051)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>React ErrorBoundary in admin-web + advertiser-web main.tsx. Graceful fallback UI.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>After tenant model ADR + inventory.</t>
+          <t>Implement S-051</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Campaign-to-store-profile targeting.</t>
+          <t>P2 — UX resilience.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Finance Contract/Invoicing Integration</t>
+          <t>Audit: Approval/Moderation</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚧 v0.6 planned (S-052)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>create_audit_event on campaign approve/reject + creative approve/reject. Behavioural proof.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>Implement S-052</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1C/ERP API integration.</t>
+          <t>P2 — audit trail completeness.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Programmatic Extension Point</t>
+          <t>Identity Router Decomposition</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚧 v0.6 planned (S-053)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>TZ v2.6. OpenRTB stub.</t>
+          <t>Plan: split identity.py (2036 lines) → domain routers. ADR or design doc.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>After production pilot.</t>
+          <t>Plan S-053</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>External DSP/SSP.</t>
+          <t>P2 — code maintainability.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Dynamic Creative MVP</t>
+          <t>SECTION</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>TZ v2.6. HTML5 canvas/video templating.</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>After KSO player stable.</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Creative personalization.</t>
+          <t>v2.6 Next Branch</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Mobile Field Ops MVP</t>
+          <t>Tenant Model ADR (ADR-018)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🟡 Decision needed</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>TZ v2.6. Mobile app for field operators.</t>
+          <t>ADR-018 proposed 2026-07-11. P0 before v2.6 implementation.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>After KSO player stable.</t>
+          <t>Single-retailer vs multi-retailer decision.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Screen checks, content swap in field.</t>
+          <t>Without decision: rewrite attribution, finance, competitive separation, RLS.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>A/B Lift Metrics</t>
+          <t>Attribution &amp; Sales Lift</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2227,208 +2217,208 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>After attribution.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>A/B testing of creatives.</t>
+          <t>Requires PoP pipeline + receipt data.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Third-Party DOOH Measurement/Accreditation</t>
+          <t>Self-Service Advertiser Cabinet</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🟡 Core pilot flow complete</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>TZ v2.6. Design stub only.</t>
+          <t>S-023a-g: advertiser-web — login, campaigns CRUD, creatives, PoP, profile, password, attach creative, submit approval. 66 vitest tests. CI #29162925840.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>After production pilot.</t>
+          <t>Production UX, browser E2E, admin approval UI for advertiser</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Independent impression audit.</t>
+          <t>Next: attach creative + submit approval (S-023g).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Production Gaps Triage (S-029)</t>
+          <t>Competitive Separation</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>✅ Docs/triage done</t>
+          <t>⚪ Not started</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>docs/product/production-gaps-triage.md. 8 categories, 35+ gaps prioritised. develop branch.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Start v0.5 P0 gates (CI, secrets, backups, monitoring)</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>No code changes. Docs-only triage.</t>
+          <t>Blocking competitor brands on same screen.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Production CI Gate</t>
+          <t>Store-Level Audience Targeting</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>✅ S-030 done</t>
+          <t>⚪ Not started</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CI: production-config-gate job in phase1-ci.yml. 24 gate tests. ENVIRONMENT=production fails on weak secrets.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Add ENVIRONMENT=production validation, fail on weak secrets</t>
+          <t>After tenant model ADR + inventory.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>P0 — blocks all further releases.</t>
+          <t>Campaign-to-store-profile targeting.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Backup / Restore / DR</t>
+          <t>Finance Contract/Invoicing Integration</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>✅ S-031 done</t>
+          <t>⚪ Not started</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>scripts/backup/, scripts/restore/. Integration drill test (5/5 passed). Runbook: docs/runbook/backup-restore-dr.md.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>pg_dump cron + restore runbook + test drill</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>P0 — data safety.</t>
+          <t>1C/ERP API integration.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Secrets Management</t>
+          <t>Programmatic Extension Point</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚫 Deferred</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>.env.example exists. Production secrets not enforced.</t>
+          <t>TZ v2.6. OpenRTB stub.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>SECRET_* validation in production mode. Rotation runbook.</t>
+          <t>After production pilot.</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>P0 — security baseline.</t>
+          <t>External DSP/SSP.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Identity Hardening (LDAPS)</t>
+          <t>Dynamic Creative MVP</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚫 Deferred</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>AD stub returns 503. No real LDAPS integration.</t>
+          <t>TZ v2.6. HTML5 canvas/video templating.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Wire real AD adapter. Replace stub.</t>
+          <t>After KSO player stable.</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>P1 — blocks real admin access.</t>
+          <t>Creative personalization.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Password Reset / Advertiser Invite</t>
+          <t>Mobile Field Ops MVP</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚫 Deferred</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>No self-service password reset. No invite flow.</t>
+          <t>TZ v2.6. Mobile app for field operators.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Email-based reset token. Admin invite → set password.</t>
+          <t>After KSO player stable.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>P1 — blocks advertiser self-onboarding.</t>
+          <t>Screen checks, content swap in field.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Creative Moderation (Manual)</t>
+          <t>A/B Lift Metrics</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2438,123 +2428,339 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CREATIVE_AUTO_APPROVE_UPLOADS=true. No human review.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Admin-web moderation queue. Approve/reject with reason.</t>
+          <t>After attribution.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>P1 — quality control before live.</t>
+          <t>A/B testing of creatives.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Malware Scan</t>
+          <t>Third-Party DOOH Measurement/Accreditation</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🚫 Deferred</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Uploaded files unverified.</t>
+          <t>TZ v2.6. Design stub only.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ClamAV on upload complete. Quarantine on detection.</t>
+          <t>After production pilot.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>P1 — security.</t>
+          <t>Independent impression audit.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Reporting Export (CSV/XLSX)</t>
+          <t>Production Gaps Triage (S-029)</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>✅ Docs/triage done</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PoP data API-only. No offline export.</t>
+          <t>docs/product/production-gaps-triage.md. 8 categories, 35+ gaps prioritised. develop branch.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Export endpoints: GET /api/v1/identity/campaigns/{id}/pop/export</t>
+          <t>v0.5 published. v0.6 Production Readiness planned (S-046).</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>P1 — customer-facing.</t>
+          <t>No code changes. Docs-only triage.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ClickHouse Foundation</t>
+          <t>Production CI Gate</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>✅ S-030 done</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ADR-007: deferred to Phase 4+. Container exists, not wired.</t>
+          <t>CI: production-config-gate job in phase1-ci.yml. 24 gate tests. ENVIRONMENT=production fails on weak secrets.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>ClickHouse deployment + PoP data replication</t>
+          <t>Add ENVIRONMENT=production validation, fail on weak secrets</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>P1 — analytical performance.</t>
+          <t>P0 — blocks all further releases.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
+          <t>Backup / Restore / DR</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>✅ S-031 done</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>scripts/backup/, scripts/restore/. Integration drill test (5/5 passed). Runbook: docs/runbook/backup-restore-dr.md.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>pg_dump cron + restore runbook + test drill</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>P0 — data safety.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Secrets Management</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>.env.example exists. Production secrets not enforced.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>SECRET_* validation in production mode. Rotation runbook.</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>P0 — security baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Identity Hardening (LDAPS)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>🚧 v0.6 planned (S-048)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>AD stub returns 503. No real LDAPS integration.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Wire real AD adapter. Replace stub.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>P1 — blocks real admin access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Password Reset / Advertiser Invite</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>No self-service password reset. No invite flow.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Email-based reset token. Admin invite → set password.</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>P1 — blocks advertiser self-onboarding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Creative Moderation (Manual)</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CREATIVE_AUTO_APPROVE_UPLOADS=true. No human review.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Admin-web moderation queue. Approve/reject with reason.</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>P1 — quality control before live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Malware Scan</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>⚪ Not started</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Uploaded files unverified.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>ClamAV on upload complete. Quarantine on detection.</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>P1 — security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Reporting Export (CSV/XLSX)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>🟡 CSV done (S-040). XLSX: 🚧 v0.6 decision (S-054a)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>PoP data API-only. No offline export.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Export endpoints: GET /api/v1/identity/campaigns/{id}/pop/export</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>P1 — customer-facing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ClickHouse Foundation</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ADR-007: deferred to Phase 4+. Container exists, not wired.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ClickHouse deployment + PoP data replication</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>P1 — analytical performance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>Device / Player Readiness</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>⚪ Not started</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Manifest endpoint ready. Simulator proven. No real player.</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>Real KSO player. Manifest verification on device. Offline fail-closed. AFTER v0.5 Business Portal Complete.</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>P1 — first channel live. BLOCKED until v0.5 Business Portal Complete.</t>
         </is>
@@ -2572,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2632,7 +2838,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready</t>
+          <t>🟡 Pilot-ready / 🚧 v0.6 LDAPS planned</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -2651,7 +2857,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Ждём provisioning LDAPS-контроллера. Пока: тестовые учётные записи для пилота.</t>
+          <t>Real LDAPS wiring planned for v0.6 (S-048).</t>
         </is>
       </c>
     </row>
@@ -3234,7 +3440,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟡 PostgreSQL: done (S-031). MinIO/NATS: 🚧 v0.6 planned</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -3252,29 +3458,56 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Перед production deployment.</t>
+          <t>MinIO mirror + NATS policy — v0.6 (S-049/S-050).</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Мониторинг и observability</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>🚧 v0.6 planned (S-047)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>HealthState counters на control-api + device-gateway.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Prometheus/Grafana/AlertManager не развёрнуты.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>v0.6: Prometheus metrics endpoint + Grafana dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Мониторинг и алерты</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>🟠 Частично</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Health endpoints: /health/live + /health/ready на всех сервисах.
 HealthState counters (published, failed, dead-letter, acked, nakd).
 Graceful shutdown (SIGTERM).</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Нет Prometheus metrics.
 Нет alert rules.
@@ -3282,82 +3515,55 @@
 Нет мониторинга инфраструктуры (CPU, RAM, диск).</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Deferred: Prometheus + Grafana после compose → production.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>v2.6 Next Branch</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Self-service advertiser cabinet</t>
+          <t>SECTION</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / self-service pilot</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>S-023a-i completed. Pilot-ready for demo.</t>
+          <t>v2.6 Next Branch</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sales Lift / Attribution proof</t>
+          <t>Self-service advertiser cabinet</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>🟡 Pilot-ready / self-service pilot</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>No attribution pipeline. No receipt data integration.</t>
+          <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>After tenant model ADR + PoP pipeline.</t>
+          <t>S-023a-i completed. Pilot-ready for demo.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Competitor blocking</t>
+          <t>Sales Lift / Attribution proof</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3372,19 +3578,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No competitive separation model.</t>
+          <t>No attribution pipeline. No receipt data integration.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>After tenant model ADR + PoP pipeline.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Store/audience targeting</t>
+          <t>Competitor blocking</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3399,19 +3605,19 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>No store profiles. No audience targeting.</t>
+          <t>No competitive separation model.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>After tenant model ADR + inventory.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Financial docs / reconciliation / integration</t>
+          <t>Store/audience targeting</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3426,46 +3632,46 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>No 1C/ERP API. No invoicing.</t>
+          <t>No store profiles. No audience targeting.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>After tenant model ADR + inventory.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Programmatic inventory sales</t>
+          <t>Financial docs / reconciliation / integration</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>⚪ Not started</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>TZ v2.6. OpenRTB stub.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>No DSP/SSP integration.</t>
+          <t>No 1C/ERP API. No invoicing.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>After production pilot.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Dynamic creatives</t>
+          <t>Programmatic inventory sales</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3475,24 +3681,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>TZ v2.6. HTML5 canvas/video templating.</t>
+          <t>TZ v2.6. OpenRTB stub.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>No creative templating.</t>
+          <t>No DSP/SSP integration.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>After KSO player stable.</t>
+          <t>After production pilot.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Mobile field ops</t>
+          <t>Dynamic creatives</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3502,12 +3708,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>TZ v2.6. Mobile app.</t>
+          <t>TZ v2.6. HTML5 canvas/video templating.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>No mobile client.</t>
+          <t>No creative templating.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3519,25 +3725,52 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Mobile field ops</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>🚫 Deferred</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Mobile app.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>No mobile client.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>After KSO player stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Independent DOOH measurement</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>🚫 Deferred</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>TZ v2.6. Design stub only.</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>No external impression audit.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>

</xml_diff>

<commit_message>
feat: add observability baseline with prometheus and grafana
S-047 — Production observability foundation for v0.6.

Metrics:
- packages/observability/metrics.py: 18 Prometheus metrics
  (HTTP, outbox, NATS, manifest, PoP, DB, auth) in text/plain
  format. No third-party dependency — pure Python stdlib.
- /metrics endpoint on control-api (port 8000) and
  device-gateway (port 8001). No auth required.
- HTTP metrics middleware records request count + 5xx.

Compose observability profile:
- docker-compose.observability.yml: Prometheus + Grafana
- prometheus.yml: scrape control-api + device-gateway
- alerts.yml: 8 alert rules (ServiceDown, High5xx, DB, NATS,
  outbox dead letters, manifest failures, PoP quarantine,
  NATS consumer failures)
- Grafana: RMP Overview dashboard (4 sections, 10 panels)

Runbook: docs/runbook/observability.md

Tests: tests/test_phase_observability.py — 9/9 pass

Docs: stabilization-tracker + roadmap updated for S-047 done
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1702,22 +1702,22 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-047)</t>
+          <t>✅ S-047 done (Prometheus + Grafana)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Foundation: HealthState counters (published, failed, dead-letter, acked, nakd). Periodic summary logger.</t>
+          <t>Prometheus metrics on control-api + device-gateway. Grafana dashboard RMP Overview (4 sections, 10 panels). Alert rules (8). Runbook. dev-only compose profile.</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Prometheus + Grafana + AlertManager (v0.6)</t>
+          <t>Production secret hardening for Grafana admin password.</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Prometheus + Grafana after compose → production deploy.</t>
+          <t>P0 — baseline production observability ready.</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-047)</t>
+          <t>✅ S-047 done</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">

</xml_diff>

<commit_message>
feat: add real LDAPS authentication provider
S-048 — Real LDAPS wiring for v0.6.

ad_provider.py:
- RealLDAPAuthProvider: ldap3 bind+search flow
- Service account or anonymous bind → search user DN →
  bind as user → verify password
- Safe filter escaping (ldap3.utils.conv.escape_filter_chars)
- Timeout on all operations (10s receive, 5s connect)
- Never logs passwords or bind credentials
- StubADAuthProvider preserved when AD_ENABLED=false
- get_ad_provider() factory selects real vs stub

AuthService: uses get_ad_provider() instead of hardcoded stub.

AD endpoints: updated to use real provider for settings + test.
Modes: disabled | misconfigured | configured | unavailable.
Test endpoint: service bind without user password.

Runbook: docs/runbook/ldaps-auth.md — env vars, modes,
failure matrix, production checklist, verification commands.

Docs: stabilization-tracker + roadmap updated for S-048.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -716,7 +716,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Real LDAPS wiring (v0.6, S-048)</t>
+          <t>Real LDAPS wired (S-048). Production deploy checklist pending.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -2006,17 +2006,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-048)</t>
+          <t>✅ S-048 done</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Replace AD stub with real LDAPS bind/search. AD_LDAP_URL/BIND_DN/SEARCH_BASE env vars. Fail-safe to local_break_glass.</t>
+          <t>RealLDAPAuthProvider with ldap3 bind+search. Safe filter escaping. Timeouts. No password logs. Stub preserved when AD_ENABLED=false.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Implement S-048</t>
+          <t>Production deploy: TLS cert validation + secrets management.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>✅ S-048 done (Real LDAPS provider)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">

</xml_diff>

<commit_message>
feat: add minio backup restore drill
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>🟡 PostgreSQL: S-031 done. MinIO/NATS: 🚧 v0.6 planned (S-049/S-050)</t>
+          <t>🟡 PostgreSQL: S-031 done. MinIO: S-049 done. NATS: 🚧 v0.6 planned (S-050)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>MinIO mirror + restore drill (S-049). NATS backup policy (S-050).</t>
+          <t>MinIO backup/restore done (S-049). NATS backup policy (S-050).</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -2033,22 +2033,22 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-049)</t>
+          <t>✅ S-049 done</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>mc mirror cron for creative assets bucket. Restore drill + runbook update.</t>
+          <t>Python SDK full-bucket backup + manifest + SHA-256. Restore with check/dry-run/confirm. Integration test (4 cases). Runbook: docs/runbook/minio-backup-restore.md.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Implement S-049</t>
+          <t>Merged to develop</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>P0 — data safety for creative assets.</t>
+          <t>P0 — complete. Deferred: offsite, lifecycle, monitoring, incremental.</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>🟡 PostgreSQL: done (S-031). MinIO/NATS: 🚧 v0.6 planned</t>
+          <t>🟡 PostgreSQL: done (S-031). MinIO: done (S-049). NATS: 🚧 v0.6 planned (S-050)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: add nats recovery policy and proof
- Policy: PostgreSQL outbox is source of truth; NATS JetStream is transport
- Recovery: provisioning + relay replay (dedup-safe: Nats-Msg-Id = event_id)
- Scripts/check/nats_recovery_check.py: diagnostics for stream/outbox health
- tests/integration/test_nats_recovery.py: 4 scenarios (provisioning, replay
  after reset, dedup safety, check script)
- docs/runbook/nats-backup-restore.md: full runbook with failure scenarios
- compose: named nats_jetstream volume for faster dev recovery
- backup-restore-dr.md: updated with 4-step recovery order (DB → MinIO → NATS)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>🟡 PostgreSQL: S-031 done. MinIO: S-049 done. NATS: 🚧 v0.6 planned (S-050)</t>
+          <t>🟡 PostgreSQL: S-031 done. MinIO: S-049 done. NATS: S-050 done.</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2060,22 +2060,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-050)</t>
+          <t>✅ S-050 done</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>NATS state recoverable from outbox. Manual nats stream backup procedure.</t>
+          <t>Policy: outbox source of truth. Recovery via provisioning + relay replay (dedup-safe: Nats-Msg-Id = event_id). Runbook: docs/runbook/nats-backup-restore.md. Integration test proves recovery cycle.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Document S-050</t>
+          <t>Documented</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>P1 — DR completeness.</t>
+          <t>P1 — complete. Outbox relay publishes with dedup. Compose named volume for faster recovery.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add portal error boundaries
- ErrorBoundary class component in admin-web and advertiser-web
- Top-level wrap + route errorElement for per-route isolation
- Russian fallback: 'Что-то пошло не так' + 'Обновить страницу'
- Secret redaction in dev mode (JWT/credential patterns)
- resetKey prop for route-change auto-reset
- Tests: 7 vitest per portal (fallback, refresh, reset, no secrets)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -2087,22 +2087,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-051)</t>
+          <t>✅ S-051 done</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>React ErrorBoundary in admin-web + advertiser-web main.tsx. Graceful fallback UI.</t>
+          <t>ErrorBoundary class component. Top-level wrap + route errorElement. Russian fallback, secret redaction. 7 vitest tests per portal.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Implement S-051</t>
+          <t>Merged to develop</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>P2 — UX resilience.</t>
+          <t>P2 — complete. Class component, route-level auto-reset, no secrets in UI.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add audit events for approval and moderation
- Campaign approve: writes campaign.approved audit event
- Campaign reject: writes campaign.rejected audit event (with reason)
- Creative approve: writes creative.approved audit event
- Creative reject: writes creative.rejected audit event (with reason)
- Same DB transaction as state change, before outbox enqueue
- Details: old/new status, rejection_reason (truncated 200)
- No secrets/storage fields in audit details
- Tests: 7 new unit tests (audit writes, no secrets, 403 skips)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -2114,22 +2114,22 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-052)</t>
+          <t>✅ S-052 done</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>create_audit_event on campaign approve/reject + creative approve/reject. Behavioural proof.</t>
+          <t>Campaign approve/reject + creative approve/reject write audit_events_operational. 4 actions: campaign.approved/rejected, creative.approved/rejected. Same tx. 7 new unit tests.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Implement S-052</t>
+          <t>Merged to develop</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>P2 — audit trail completeness.</t>
+          <t>P2 — complete. Follows S-035e user-management audit pattern.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: split identity api router by domain
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -2141,22 +2141,22 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-053)</t>
+          <t>✅ S-053 done</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Plan: split identity.py (2036 lines) → domain routers. ADR or design doc.</t>
+          <t>Split 2097-line identity.py into 8 domain routers: common (99), users (408), ad_settings (106), advertisers (147), campaigns (725), creatives (314), reporting (155), inventory (122). identity.py now 40-line aggregator. 66/66 tests, import boundaries clean.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Plan S-053</t>
+          <t>Merged to develop</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>P2 — code maintainability.</t>
+          <t>P2 — complete. Pure refactor, no API/business change.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record xlsx export decision for v0.6
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>🟡 CSV done (S-040), XLSX deferred</t>
+          <t>✅ CSV done (S-040). XLSX deferred to v0.7/v0.8.</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1562,12 +1562,12 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>XLSX export deferred (openpyxl dependency). PDF deferred.</t>
+          <t>CSV export: GET /api/v1/identity/campaigns/{id}/pop/export. UTF-8 BOM. XLSX deferred — no openpyxl dep added.</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>BLOCKED until v0.5 Business Portal Complete. Player is v0.7 milestone.</t>
+          <t>P1 — CSV complete. XLSX revisit with report snapshots (v0.8).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: fix v0.6 readiness status before release prep
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1962,7 +1962,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Milestone: v0.6 Production Readiness (planned)</t>
+          <t>Milestone: v0.6 Production Readiness (ready for release prep)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>v0.5 published. v0.6 Production Readiness planned (S-046).</t>
+          <t>v0.5 published. v0.6 Production Readiness ready for release prep (S-046…S-055 done).</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-048)</t>
+          <t>✅ S-048 done (Real LDAPS provider)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Wire real AD adapter. Replace stub.</t>
+          <t>real LDAPS bind+search via ldap3. Stub preserved for AD_ENABLED=false. local_advertiser + break_glass preserved.</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>🟡 CSV done (S-040). XLSX: 🚧 v0.6 decision (S-054a)</t>
+          <t>✅ CSV done (S-040). XLSX deferred (S-054a done)</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / 🚧 v0.6 LDAPS planned</t>
+          <t>🟡 Pilot-ready / ✅ Real LDAPS done (S-048)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -2850,9 +2850,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Реальный LDAPS (Active Directory) не подключён — возвращает честный 503.
-MFA не реализован.
-Нет саморегистрации рекламодателей.</t>
+          <t>Real LDAPS bind+search. local_advertiser + break_glass preserved. Stub when AD_ENABLED=false.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -3440,7 +3438,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>🟡 PostgreSQL: done (S-031). MinIO: done (S-049). NATS: 🚧 v0.6 planned (S-050)</t>
+          <t>🟡 PostgreSQL: done (S-031). MinIO: ✅ done (S-049). NATS: ✅ done (S-050)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -3470,7 +3468,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>🚧 v0.6 planned (S-047)</t>
+          <t>✅ S-047 done (Prometheus + Grafana)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3480,7 +3478,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Prometheus/Grafana/AlertManager не развёрнуты.</t>
+          <t>Prometheus metrics + Grafana dashboard + AlertManager rules (not provisioned). Осталось: Grafana развернуть на production стенде.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">

</xml_diff>

<commit_message>
docs: prepare v0.6 production readiness release
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1962,7 +1962,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Milestone: v0.6 Production Readiness (ready for release prep)</t>
+          <t>Milestone: v0.6 Production Readiness (ready for publish)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>v0.5 published. v0.6 Production Readiness ready for release prep (S-046…S-055 done).</t>
+          <t>v0.5 published. v0.6 Production Readiness ready for publish (S-047…S-056 done). Tag target: fd43791.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">

</xml_diff>

<commit_message>
docs: add audit v4 remediation plan
- New: docs/product/audit-v4-remediation-plan.md
  - P1/P2/P3 classified (8+11+7 findings)
  - Proposed S-062…S-074 sequence
  - Production blocker assessment
- Updated: stabilization-tracker (S-059/S-060/S-061 + backlog)
- Updated: production-gaps-triage (baseline→v0.6.1, audit v4)
- Updated: release-versioning (v0.6→Published, v0.6.1 section)
- Updated: roadmap-s020 (milestone→v0.6.1, auth row)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1962,7 +1962,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Milestone: v0.6 Production Readiness (ready for publish)</t>
+          <t>Milestone: v0.6.1 Critical Hotfix published; v0.6.2/v0.7 audit remediation planned</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / ✅ Real LDAPS done (S-048)</t>
+          <t>🟡 Pilot-ready / ✅ Real LDAPS done (S-048) / ✅ Critical hotfix v0.6.1</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: analyze inventory domain gap (S-072)
- New doc: docs/product/inventory-domain-gap-analysis.md (324 lines)
  - Current state: static catalog — stores, surfaces, is_active toggle
  - 10 ТЗ §6.3 gaps identified (airtime, forecast, conflicts, SOV, sold-out, rules, reports, emergency/offline impact)
  - Proposed phased plan: S-075 model → S-076 availability → S-077 booking → S-078 conflicts → S-079 integration → S-080 rules → S-081…S-086 visibility+runtime
  - Player/KSO assessment: blocked until S-079 (minimal inventory contract: availability + booking)
  - Data model candidates: InventorySlot, InventoryRule
  - API/UI candidates: calendar, forecast, conflict check, rules admin
- audit-v4-remediation-plan: S-072 marked done
- stabilization-tracker: S-072 marked done
- production-gaps-triage: fixed overclaim ('inventory UI' → 'inventory catalog UI')
- roadmap.xlsx: inventory rows updated — S-072 done, S-075+ planned
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1525,7 +1525,7 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟡 S-072 done (gap analysis). S-075+ planned.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>No inventory calculation. No forecasting engine.</t>
+          <t>S-072 done 2026-07-16: gap analysis approved. Phased plan: S-075 model → S-076 availability → S-077 booking → S-078 conflicts → S-079 campaign integration. Full inventory domain per ТЗ §6.3 deferred to S-075…S-086.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>✅ S-037 done</t>
+          <t>✅ S-037 done (catalog). S-072 done (gap analysis).</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Real inventory/forecasting calculation deferred.</t>
+          <t>Full inventory/forecasting calculation planned (S-075…S-086). Current: static catalog — stores, surfaces, is_active toggle. See docs/product/inventory-domain-gap-analysis.md.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟡 S-072 done (gap analysis). S-075+ planned.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Планирование после стабилизации campaign domain.</t>
+          <t>S-072 gap analysis approved 2026-07-16. Phased plan: S-075…S-086. MVP inventory contract (S-075…S-079) before player/KSO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: review audit v4 remediation readiness (S-074)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1621,12 +1621,12 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>✅ S-071 done (backend + UI + outbox)</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>ADR-013 kill-switch architecture proven by simulator (4 levels, fail-closed).</t>
+          <t>POST /emergency/activate|deactivate, GET /emergency/status. Admin-web EmergencyPage. Permissions emergency.read|manage. Outbox emergency.changed. Player-side enforcement deferred.</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SECTION</t>
+          <t>SECTION | Milestone: v0.6.1 Critical Hotfix published; v0.6.2 audit-remediation GO — tag proposed at 90e91cb; v0.7 deferred (inventory, WCAG, i18n)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3408,12 +3408,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>✅ S-071 done (backend + UI)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Архитектура kill-switch (ADR-013): 4 уровня, fail-closed — доказана симулятором (41 тест).</t>
+          <t>Аварийный режим через админ-портал: активация/деактивация с причиной, статус, аудит. Применение на устройствах — deferred (KSO runtime).</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: design inventory domain foundation (S-076)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1525,7 +1525,7 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>🟡 S-072 done (gap analysis). S-075+ planned.</t>
+          <t>🟡 S-076 design in progress (architecture model). S-077+ planned.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1854,12 +1854,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>✅ S-037 done (catalog). S-072 done (gap analysis).</t>
+          <t>✅ S-037 (catalog). S-072 (gap analysis). S-076 (architecture design in progress).</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Backend: stores/surfaces endpoints with inventory.read/inventory.manage. Admin-web: InventoryPage — stores/surfaces tabs, search, active/inactive toggle.</t>
+          <t>Backend: stores/surfaces endpoints. Inventory domain model: docs/architecture/inventory-domain-model.md. Implementation: S-077+.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1957,7 +1957,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SECTION | Milestone: v0.6.1 Critical Hotfix published; v0.6.2 audit-remediation GO — tag proposed at 90e91cb; v0.7 deferred (inventory, WCAG, i18n)</t>
+          <t>SECTION | Milestone: v0.6.2 published (tag at 90e91cb). v0.7 inventory foundation design in progress (S-076).</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3336,12 +3336,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>🟡 S-072 done (gap analysis). S-075+ planned.</t>
+          <t>🟡 S-076 design in progress. S-077+ implementation planned.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Архитектурный дизайн: InventorySlot, InventoryBooking, InventoryRule. API: availability, reservation, commit/release, conflicts, calendar, reports. Конфликт-детекция: 8 типов.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: add inventory domain schema foundation (S-077)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1525,12 +1525,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>🟡 S-076 design in progress (architecture model). S-077+ planned.</t>
+          <t>🟡 S-077 schema in progress. S-076 design done. S-078+ planned.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>TZ §6.3: availability grid, forecasting, prime-time rules, statuses.</t>
+          <t>S-076: architecture design. S-077: InventorySlot/Booking/Rule models, migration 015, Pydantic schemas, repository CRUD. 17 unit tests. 49 DB tables. RLS deferred (admin-only MVP).</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1854,12 +1854,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>✅ S-037 (catalog). S-072 (gap analysis). S-076 (architecture design in progress).</t>
+          <t>✅ S-037 (catalog). S-072 (gap). S-076 (design). S-077 (schema in progress).</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Backend: stores/surfaces endpoints. Inventory domain model: docs/architecture/inventory-domain-model.md. Implementation: S-077+.</t>
+          <t>Inventory domain schema foundation: 3 tables (inventory_slots, inventory_bookings, inventory_rules), repository skeleton.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3336,12 +3336,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>🟡 S-076 design in progress. S-077+ implementation planned.</t>
+          <t>🟡 S-077 schema in progress. S-076 design done.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Архитектурный дизайн: InventorySlot, InventoryBooking, InventoryRule. API: availability, reservation, commit/release, conflicts, calendar, reports. Конфликт-детекция: 8 типов.</t>
+          <t>Inventory DB schema: slots (per surface/date/hour), bookings (reserve/commit/release), rules (scoped business constraints). Migration 015. RLS deferred.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: normalize roadmap format and Russian business narrative
S-078b — Roadmap Format + Russian Business Narrative Repair

- Normalized all statuses to Russian dictionary (9 status types)
- Updated inventory rows: S-077 ✅, S-078 ✅, S-079+ planned
- Rewrote business roadmap in simple Russian with dependency explanations
- Fixed copy-paste error: Dynamic Creative MVP row had LDAPS status
- Removed duplicate monitoring row in business sheet
- Added KSO/player dependency explanation: blocked until minimum inventory contract
- Created docs/product/roadmap-maintenance-rules.md
- Updated stabilization-tracker.md and inventory-domain-gap-analysis.md
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / self-service pilot</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -1525,22 +1525,22 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>🟡 S-077 schema in progress. S-076 design done. S-078+ planned.</t>
+          <t>✅ Готово: S-077 schema/repo, S-078 availability calculator. S-079+ запланировано.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>S-076: architecture design. S-077: InventorySlot/Booking/Rule models, migration 015, Pydantic schemas, repository CRUD. 17 unit tests. 49 DB tables. RLS deferred (admin-only MVP).</t>
+          <t>S-076: architecture model (5 entities, 8 conflict types). S-077: InventorySlot/Booking/Rule models + migration 015 + Pydantic schemas + repository (17 unit). S-078: compute_inventory_availability() + POST /inventory/availability + 23 unit tests. 49 DB tables. RLS deferred (admin-only MVP).</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>S-072 done 2026-07-16: gap analysis approved. Phased plan: S-075 model → S-076 availability → S-077 booking → S-078 conflicts → S-079 campaign integration. Full inventory domain per ТЗ §6.3 deferred to S-075…S-086.</t>
+          <t>S-079 reservation lifecycle + campaign integration. S-080 conflict detection. S-081 UI календарь инвентаря.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Planning after campaign domain stable.</t>
+          <t>S-077+S-078 completed 2026-07-16. Minimum inventory contract: availability check ✅, booking ⏳, campaign integration ⏳. Player/KSO blocked until booking+campaign integration done.</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>✅ CSV done (S-040). XLSX deferred to v0.7/v0.8.</t>
+          <t>✅ CSV готово (S-040), XLSX 🚫 отложено</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>✅ S-071 done (backend + UI + outbox)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>🟡 PostgreSQL: S-031 done. MinIO: S-049 done. NATS: S-050 done.</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>✅ S-047 done (Prometheus + Grafana)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>✅ Done / LAN preview</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1854,17 +1854,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>✅ S-037 (catalog). S-072 (gap). S-076 (design). S-077 (schema in progress).</t>
+          <t>✅ S-037 catalog. S-072 gap analysis. S-076 design. S-077 schema. S-078 availability calculator.</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Inventory domain schema foundation: 3 tables (inventory_slots, inventory_bookings, inventory_rules), repository skeleton.</t>
+          <t>Inventory foundation: 3 tables (inventory_slots, inventory_bookings, inventory_rules), repository, availability calculator. 17+23=40 unit tests.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Full inventory/forecasting calculation planned (S-075…S-086). Current: static catalog — stores, surfaces, is_active toggle. See docs/product/inventory-domain-gap-analysis.md.</t>
+          <t>S-079 booking lifecycle + campaign integration. S-080 conflicts. S-081 UI calendar.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>✅ Done (S-039, S-023h-i)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>✅ CSV done, XLSX deferred (S-040)</t>
+          <t>✅ CSV готово (S-040), XLSX 🚫 отложено</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1957,12 +1957,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SECTION | Milestone: v0.6.2 published (tag at 90e91cb). v0.7 inventory foundation design in progress (S-076).</t>
+          <t>SECTION</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Milestone: v0.6.1 Critical Hotfix published; v0.6.2/v0.7 audit remediation planned</t>
+          <t>Milestone: v0.6.2 опубликован (тег 90e91cb). v0.7 inventory foundation: S-076 design ✅, S-077 schema ✅, S-078 availability ✅. S-079 booking запланирован.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>✅ S-049 done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>✅ S-050 done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>✅ S-051 done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>✅ S-052 done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>✅ S-053 done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>🟡 Decision needed</t>
+          <t>🧭 Требует решения</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>✅ S-048 done (Real LDAPS provider)</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>✅ Docs/triage done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>✅ S-030 done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>✅ S-031 done</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>✅ S-048 done (Real LDAPS provider)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>✅ CSV done (S-040). XLSX deferred (S-054a done)</t>
+          <t>✅ CSV готово (S-040), XLSX 🚫 отложено</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2747,7 +2747,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2838,19 +2838,22 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / ✅ Real LDAPS done (S-048) / ✅ Critical hotfix v0.6.1</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Тестовый вход через local_advertiser и local_break_glass (bcrypt).
-Admin-web: страница логина с выбором провайдера (Рекламодатель / Break-glass Admin / Сотрудник AD).
-JWT access + refresh токены, HttpOnly cookie. /me из БД.</t>
+          <t>✅ Вход через local_advertiser и local_break_glass (bcrypt).
+✅ Admin-web: страница логина с выбором провайдера (Рекламодатель / Break-glass Admin / Сотрудник AD).
+✅ JWT access + refresh токены, HttpOnly cookie.
+✅ Реальный LDAPS (S-048): ldap3 bind+search, safe filter escaping, таймауты. Stub preserved при AD_ENABLED=false.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Real LDAPS bind+search. local_advertiser + break_glass preserved. Stub when AD_ENABLED=false.</t>
+          <t>❌ Нет self-service сброса пароля.
+❌ Нет инвайт-писем для новых рекламодателей.
+Почему: базовый вход работает. Self-service onboarding — v0.8.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2897,17 +2900,21 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>✅ Done / v0.5 Ready for RC</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Advertiser-web: вход, кампании (список, деталь, создание/редактирование черновиков), креативы (библиотека, загрузка, прикрепление), отправка на согласование, видимость статуса/причины отклонения, PoP-отчёты + CSV экспорт, профиль/смена пароля. Admin-web: полное управление. S-042 CONDITIONAL GO.</t>
+          <t>✅ Advertiser-web (http://192.168.110.77:3001): вход, создание/редактирование кампаний, библиотека креативов, загрузка, прикрепление к кампании, отправка на согласование, PoP-отчёты + CSV экспорт, профиль/смена пароля.
+✅ Admin-web: полное управление рекламодателями.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Нет кнопок approve/reject (только admin). Нет биллинга/атрибуции. Production UX audit deferred.</t>
+          <t>❌ Рекламодатель не может сам утверждать кампании — только admin.
+❌ Нет биллинга/атрибуции.
+❌ Production UX audit отложен.
+Почему: self-service пилот работает. Полный production UX — после стабилизации backend.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -2939,22 +2946,22 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Backend API: полный CRUD кампаний (7 endpoints).
-Admin-web UI: список кампаний с фильтром, мастер создания, страница с 5 вкладками.
-Advertiser-web: создание/редактирование черновиков через отдельный порт.</t>
+          <t>✅ Backend: полный CRUD кампаний (7 endpoints), пролёты, размещения, креативы.
+✅ Admin-web: список с фильтром, мастер создания, 5 вкладок (пролёты, размещения, креативы+upload, согласование, PoP-отчёты).
+✅ Advertiser-web: создание/редактирование черновиков.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Нет календаря планирования.
-Нет drag-and-drop.
-UX/accessibility не завершены.
-Нет браузерных E2E-тестов.</t>
+          <t>❌ Нет календаря планирования.
+❌ Нет drag-and-drop.
+❌ UX/accessibility не завершены.
+❌ Нет браузерных E2E-тестов.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2971,19 +2978,20 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Backend: request-approval → approve/reject с audit trail.
-Admin-web: approve/reject UI.
-Advertiser-web: отправка на согласование (S-023g). Advertiser не может approve/reject.</t>
+          <t>✅ Backend: request-approval → approve/reject с audit trail.
+✅ Admin-web: очередь согласования, approve/reject с причиной.
+✅ Advertiser-web: отправка на согласование, видимость статуса/причины отклонения.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Advertiser может только отправить; утверждает/отклоняет admin.</t>
+          <t>❌ Рекламодатель не может сам утверждать — только отправляет.
+Почему: это осознанное ограничение безопасности.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -3000,7 +3008,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -3183,12 +3191,15 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>⚪ Не начато (v0.7, ✅ v0.5 Business Portal done)</t>
+          <t>⚪ Не начато (v0.7)</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Архитектура зафиксирована (ADR-013, ADR-016). Симулятор: 41 тест. Device-gateway: GET /manifest/latest. ✅ v0.5 Business Portal Complete — blocker cleared. KSO/player — v0.7 milestone.</t>
+          <t>✅ Архитектура зафиксирована (ADR-013, ADR-016). Симулятор: 41 тест безопасности.
+✅ Device-gateway: GET /manifest/latest.
+✅ v0.5 Business Portal — блокер снят. KSO/player — v0.7 milestone.
+Почему ждём: без inventory (слоты + бронирование) плеер может получить конфликтующие размещения. Minimum inventory contract (availability + booking) должен быть готов до интеграции с реальным плеером.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -3198,7 +3209,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>KSO после v0.6 production hardening.</t>
+          <t>После minimum inventory contract (S-079 booking + S-082 campaign integration).</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3221,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -3239,7 +3250,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -3266,7 +3277,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -3294,7 +3305,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -3336,24 +3347,29 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>🟡 S-077 schema in progress. S-076 design done.</t>
+          <t>✅ Готово: S-077 schema, S-078 availability. S-079+ запланировано.</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Inventory DB schema: slots (per surface/date/hour), bookings (reserve/commit/release), rules (scoped business constraints). Migration 015. RLS deferred.</t>
+          <t>✅ Inventory DB: слоты (surface × дата × час), бронирования (reserve/commit/release), бизнес-правила (scoped constraints). Migration 015.
+✅ Availability calculator: POST /inventory/availability — проверка свободных слотов по поверхности и временному диапазону, get-or-create слотов с default capacity, SOV → units конвертация, детекция конфликтов.
+Что можно: программно проверить доступность слота перед размещением.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Нет расчёта свободного/занятого/зарезервированного эфирного времени.
-Нет визуальной сетки инвентаря по филиалам/магазинам.
-Нет настройки правил (макс. нагрузка, prime-time, приоритеты).</t>
+          <t>❌ Нет бронирования (reserve/commit) — нельзя зафиксировать слот за кампанией.
+❌ Нет интеграции с campaign approval — слот не резервируется при submit.
+❌ Нет визуальной сетки инвентаря по магазинам.
+❌ Нет настройки правил (макс. нагрузка, prime-time, приоритеты).
+❌ Нет прогноза доступности.
+Почему идём так: без inventory нельзя гарантировать, что плеер не получит конфликтующие размещения. Поэтому inventory — обязательный контракт перед KSO/player.</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>S-072 gap analysis approved 2026-07-16. Phased plan: S-075…S-086. MVP inventory contract (S-075…S-079) before player/KSO.</t>
+          <t>S-079: reservation lifecycle (reserve → commit → release/expire). S-080: conflict detection. S-081: UI календарь. S-082: campaign integration (авто-бронирование при approval). S-083-086: rules, forecasting, reporting.</t>
         </is>
       </c>
     </row>
@@ -3408,20 +3424,22 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>✅ S-071 done (backend + UI)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Аварийный режим через админ-портал: активация/деактивация с причиной, статус, аудит. Применение на устройствах — deferred (KSO runtime).</t>
+          <t>✅ Backend: POST /emergency/activate|deactivate, GET /emergency/status.
+✅ Admin-web: EmergencyPage — активация/деактивация с причиной.
+✅ Аудит всех emergency-действий.
+✅ Outbox: emergency.changed события.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Нет emergency API endpoint'ов.
-Нет MFA для emergency-пользователей.
-Нет UI для отправки emergency-команд.
-Нет мониторинга прогресса применения команд по устройствам.</t>
+          <t>❌ Применение на устройствах — deferred (требуется KSO runtime).
+❌ Нет MFA для emergency-пользователей.
+Почему: backend готов. Применение на устройствах ждёт player/KSO (v0.9).</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -3438,20 +3456,22 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>🟡 PostgreSQL: done (S-031). MinIO: ✅ done (S-049). NATS: ✅ done (S-050)</t>
+          <t>✅ Готово: PostgreSQL (S-031), MinIO (S-049), NATS (S-050)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ PostgreSQL: pg_dump backup + restore, drill test (5/5), runbook.
+✅ MinIO: полный backup + manifest + SHA-256, restore с check/dry-run/confirm, runbook.
+✅ NATS: outbox как source of truth, recovery через provisioning + relay replay (dedup-safe), runbook.</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Нет автоматических бэкапов PostgreSQL.
-Нет зеркалирования MinIO.
-Нет DR-плана.
-Нет нагрузочных тестов (ТЗ требует 40 000 устройств).</t>
+          <t>❌ Нет автоматического расписания бэкапов.
+❌ Нет offsite-репликации.
+❌ Нет DR-плана.
+❌ Нет нагрузочных тестов (ТЗ: 40 000 устройств).</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -3468,17 +3488,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>✅ S-047 done (Prometheus + Grafana)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HealthState counters на control-api + device-gateway.</t>
+          <t>✅ Prometheus метрики на control-api + device-gateway.
+✅ Grafana дашборд «RMP Overview»: 4 секции, 10 панелей.
+✅ AlertManager: 8 правил.
+✅ Health endpoints: /health/live + /health/ready на всех сервисах.
+✅ Graceful shutdown (SIGTERM).</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Prometheus metrics + Grafana dashboard + AlertManager rules (not provisioned). Осталось: Grafana развернуть на production стенде.</t>
+          <t>❌ Нет мониторинга инфраструктуры (CPU, RAM, диск).
+❌ Grafana admin password не hardened для production.
+Почему: baseline observability готов. Инфраструктурный мониторинг — после production deploy.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3488,36 +3514,11 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Мониторинг и алерты</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>🟠 Частично</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Health endpoints: /health/live + /health/ready на всех сервисах.
-HealthState counters (published, failed, dead-letter, acked, nakd).
-Graceful shutdown (SIGTERM).</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Нет Prometheus metrics.
-Нет alert rules.
-Нет Grafana dashboards.
-Нет мониторинга инфраструктуры (CPU, RAM, диск).</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>Deferred: Prometheus + Grafana после compose → production.</t>
-        </is>
-      </c>
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3539,7 +3540,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>🟡 Pilot-ready / self-service pilot</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3566,7 +3567,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3593,7 +3594,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3620,7 +3621,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3647,7 +3648,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>⚪ Not started</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3674,7 +3675,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3701,7 +3702,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3728,7 +3729,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3755,7 +3756,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>🚫 Deferred</t>
+          <t>🚫 Отложено</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">

</xml_diff>

<commit_message>
docs: expand business roadmap with explanation columns
S-079b — Roadmap Business Columns Repair

- Expanded business sheet from 5 to 8 columns:
  1. Версия / этап
  2. Бизнес-функция
  3. Статус
  4. Для чего нужна (NEW)
  5. Что уже можно использовать
  6. Что ещё нельзя / ограничения
  7. Почему сейчас / зависимость (NEW)
  8. Следующий шаг
- Filled all 30+ business rows with Russian explanations
- Every function now has: what it's for, why it's at this stage,
  what depends on it
- Updated roadmap-maintenance-rules.md (v1.1)
- Updated stabilization-tracker.md
- Visual formatting: column widths, frozen headers, wrap text
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -55,7 +55,7 @@
       <color rgb="009C6500"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +104,12 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -131,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -156,6 +162,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -527,10 +539,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2778,70 +2790,121 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Версия / этап</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Бизнес-функция</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Что можно использовать сейчас</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Что нельзя использовать</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>План / Ближайший шаг</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>Для чего нужна</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Что уже можно использовать</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Что ещё нельзя / ограничения</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Почему сейчас / зависимость</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>Следующий шаг</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="10" t="inlineStr"/>
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Пользователи и доступ</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
           <t>Вход сотрудников / рекламодателей</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>🟡 Готово для пилота</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Чтобы сотрудники офиса и рекламодатели могли войти в систему безопасно, каждый под своей учётной записью, без передачи паролей в открытом виде.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>✅ Вход через local_advertiser и local_break_glass (bcrypt).
 ✅ Admin-web: страница логина с выбором провайдера (Рекламодатель / Break-glass Admin / Сотрудник AD).
@@ -2849,31 +2912,46 @@
 ✅ Реальный LDAPS (S-048): ldap3 bind+search, safe filter escaping, таймауты. Stub preserved при AD_ENABLED=false.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>❌ Нет self-service сброса пароля.
 ❌ Нет инвайт-писем для новых рекламодателей.
 Почему: базовый вход работает. Self-service onboarding — v0.8.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Real LDAPS wiring planned for v0.6 (S-048).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Самая первая функция — без входа нельзя построить ничего. Сделана в v0.1, улучшалась до v0.6 (реальный LDAPS).</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Готово (S-048). Self-service сброс пароля — v0.8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
           <t>Роли и права (RBAC)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Чтобы разные роли (админ, оператор, аналитик) видели только то, что им положено. Безопасность данных рекламодателей.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>4 системные роли (system_admin, security_admin, operator, analyst).
 16 permissions с backend-проверкой.
@@ -2881,35 +2959,50 @@
 Scoped-доступ: branch, cluster, store, advertiser.</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Нет UI для управления ролями и назначения прав (только API).</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Основа безопасности. Сделано до campaign-логики, потому что все эндпоинты зависят от проверки прав.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
           <t>Личный кабинет рекламодателя</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Чтобы рекламодатель мог сам создавать кампании, загружать креативы и смотреть отчёты — без помощи администратора.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>✅ Advertiser-web (http://192.168.110.77:3001): вход, создание/редактирование кампаний, библиотека креативов, загрузка, прикрепление к кампании, отправка на согласование, PoP-отчёты + CSV экспорт, профиль/смена пароля.
 ✅ Admin-web: полное управление рекламодателями.</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>❌ Рекламодатель не может сам утверждать кампании — только admin.
 ❌ Нет биллинга/атрибуции.
@@ -2917,46 +3010,84 @@
 Почему: self-service пилот работает. Полный production UX — после стабилизации backend.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Self-service снижает нагрузку на операторов. Сделано после RBAC и campaign API, потому что кабинет — это UI поверх готового backend.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Production UX audit (deferred). Browser E2E (deferred).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="10" t="inlineStr"/>
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Управление рекламными кампаниями</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
           <t>Создание и редактирование кампаний</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>🟡 Готово для пилота</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Основной рабочий инструмент: создание, настройка и управление рекламными кампаниями (бюджет, сроки, поверхности).</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: полный CRUD кампаний (7 endpoints), пролёты, размещения, креативы.
 ✅ Admin-web: список с фильтром, мастер создания, 5 вкладок (пролёты, размещения, креативы+upload, согласование, PoP-отчёты).
 ✅ Advertiser-web: создание/редактирование черновиков.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>❌ Нет календаря планирования.
 ❌ Нет drag-and-drop.
@@ -2964,130 +3095,213 @@
 ❌ Нет браузерных E2E-тестов.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Ядро продукта. Сделано первым после аутентификации, потому что все остальные функции (креативы, отчёты) привязаны к кампании.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Advertiser self-service create/edit работает (S-023f).</t>
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
           <t>Согласование кампаний (Approval)</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>🟡 Готово для пилота</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Чтобы ни одна кампания не пошла в показ без проверки администратором: правильные ли креативы, не нарушен ли бюджет.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: request-approval → approve/reject с audit trail.
 ✅ Admin-web: очередь согласования, approve/reject с причиной.
 ✅ Advertiser-web: отправка на согласование, видимость статуса/причины отклонения.</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>❌ Рекламодатель не может сам утверждать — только отправляет.
 Почему: это осознанное ограничение безопасности.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>После CRUD кампаний — чтобы цепочка «создал → отправил → проверили → запустили» работала полностью.</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>После campaign UI (S-009c).</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
           <t>Загрузка креативов (медиафайлы)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>🟡 Готово для пилота</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Чтобы рекламодатели могли загружать изображения и видео для показа на экранах. Хранение — в защищённом MinIO (S3).</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Backend: presigned URL (MinIO/S3) + SHA-256.
 Admin-web UI: загрузка с прогресс-баром.
 Advertiser-web: библиотека + загрузка + привязка к кампании (S-023c, S-023g).</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Malware scan, transcoding, CDN — отложены.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>После базового CRUD кампаний, потому что креатив привязывается к кампании. До модерации — потому что загруженный файл нужно проверить.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Malware scan, transcoding, manual moderation — отложены.
 Работает для пилота.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="10" t="inlineStr"/>
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Доставка контента на устройства</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
           <t>Формирование плейлистов (manifest)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Автоматически формирует плейлист для каждого устройства: какие креативы и в каком порядке показывать. Без этого плеер не знает, что играть.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Manifest JSON с полями: device_id, store_id, playlist[], media_files[], valid_from/to, offline_ttl_hours.
 ETag/304 — кэширование на устройстве.
 Автоматическая генерация при изменении кампании.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Верификация подписи на device-gateway (signing есть, verify deferred).
 Nested per-surface playlist — Manifest v2.
 Манифест доставляется только в тестах (нет реального плеера).</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>После campaign и creative API — manifest собирает утверждённые кампании в плейлист. Это «выход» платформы на устройство.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Production manifest signing (отдельная задача).</t>
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>Получение manifest устройством</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Единая точка получения manifest для всех устройств. Кэширование (ETag), чтобы не грузить сеть повторными запросами.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>GET /api/v1/device/manifest/latest.
 Аутентификация: device JWT (sub=device_id, auth_provider=device).
@@ -3095,7 +3309,7 @@
 ETag/If-None-Match для кэширования.</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Только HTTP (не HTTPS/mTLS).
 Верификация подписи manifest на устройстве (backend signing есть, verify deferred).
@@ -3103,98 +3317,166 @@
 Нет реального KSO плеера, принимающего manifest.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Нужен сразу после manifest — устройству нужен способ безопасно получить плейлист.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>mTLS после интеграции с KSO плеером.
 Production manifest signing.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>Proof-of-Play (подтверждение показов)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Принимает подтверждения показов от устройств: что, когда и сколько раз показали. Это основа для отчётности перед рекламодателем.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>POST /api/v1/pop/batch — приём PoP-событий от устройств.
 11-шаговая валидация: schema, device, dedup, duration, playback, clock drift, cross-entity.
 Карантин 72h. Billing-grade accepted события.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>PoP эмитится только симулятором (не реальным KSO плеером).
 Нет экспорта отчётов о показах.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>После device gateway — так как PoP-события приходят от устройств, получающих manifest.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Реальный KSO плеер — вне backend-пилота.</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>Отчёты по показам</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Чтобы рекламодатель и администратор видели: сколько показов было, по каким поверхностям, в какой день. Это «доказательство» для рекламодателя.</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Backend: GET pop/{summary,by-day,by-surface}. Admin-web: вкладка PoP-отчёты. Advertiser-web: секция Отчётность в детали кампании.</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Нет дашборда сети (ТЗ §15.1).
 Нет ClickHouse / materialized views.</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>После PoP ingestion — данные сначала нужно принять и сохранить, потом показывать.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>После campaign UI стабилизации.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="10" t="inlineStr"/>
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Каналы и устройства</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>v0.7</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>КСО (кассы самообслуживания)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>⚪ Не начато (v0.7)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Кассы самообслуживания — первый физический канал показа рекламы в магазинах сети «Верный». Основной носитель для розничной рекламы.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>✅ Архитектура зафиксирована (ADR-013, ADR-016). Симулятор: 41 тест безопасности.
 ✅ Device-gateway: GET /manifest/latest.
@@ -3202,155 +3484,253 @@
 Почему ждём: без inventory (слоты + бронирование) плеер может получить конфликтующие размещения. Minimum inventory contract (availability + booking) должен быть готов до интеграции с реальным плеером.</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Реального KSO плеера нет. Нет интеграции с железом КСО.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>После minimum inventory contract (S-079 booking + S-082 campaign integration).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Блокирован до минимального inventory-контракта (S-079). Без гарантии, что размещения не конфликтуют, плеер будет работать технически, но бизнес-правила будут неполными. Планируется на v0.9 после S-080/S-081.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>После S-080/S-081 (конфликты + календарь инвентаря), затем v0.9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
           <t>Android / Android TV</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Второй по важности канал после КСО — ТВ-приставки в магазинах. Расширяет охват аудитории.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Архитектура заложена: capability profiles в БД, manifest поддерживает несколько device_types.</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Нет Android плеера.
 Нет WebView kiosk режима.
 Нет ТВ-приставок.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>После пилота КСО — архитектура каналов позволяет подключать новые типы устройств без переписывания платформы.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Второй канал после KSO pilot.</t>
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
           <t>Price Checker (Android)</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Прайс-чекеры — дополнительные точки контакта с покупателем. Показ рекламы в режиме ожидания.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ (§6.8): показ рекламы только в idle/screen saver, без блокировки проверки цены.</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Нет реализации.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Низкий приоритет. После КСО и Android TV.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>После KSO + Android TV.</t>
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
           <t>ESL / Электронные ценники</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Электронные ценники — потенциально тысячи мини-экранов в магазине. Требуют интеграции с оборудованием вендоров.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ (§6.8): интеграция через шлюзы и vendor API.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Нет адаптеров к ESL-шлюзам.
 Нет поддержки протоколов вендоров.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Отдельный интеграционный проект. Зависит от доступности оборудования и API вендоров.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Отдельный проект интеграции.</t>
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>LED Shelf Banners</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>LED-панели на полках — дополнительный рекламный инвентарь. Схож с КСО по архитектуре.</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ.</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Нет реализации.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Самый низкий приоритет среди каналов.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Низкий приоритет.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="10" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Инвентарь и прогноз</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>v0.7</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
           <t>Инвентарь рекламных мест</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>✅ Готово: калькулятор + бронирование + интеграция с approval (S-079).</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Гарантирует, что два рекламодателя не получат один и тот же слот на одном экране в одно время. Управляет ёмкостью рекламных поверхностей.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>✅ Inventory DB: слоты (surface × дата × час), бронирования (reserve/commit/release/expire).
 ✅ Availability calculator: проверка свободных слотов.
@@ -3359,7 +3739,7 @@
 Что можно: размещения автоматически проверяются на доступность инвентаря. Нельзя согласовать кампанию, если инвентарь недоступен.</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>❌ Нет визуальной сетки/календаря инвентаря по магазинам.
 ❌ Нет настройки правил (макс. нагрузка, prime-time, приоритеты).
@@ -3368,67 +3748,120 @@
 Почему идём так: minimum inventory contract (availability + booking + campaign integration) готов. Дальше — конфликты (S-080) и календарь (S-081) перед KSO/player.</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>S-080: conflict detection engine. S-081: UI календарь инвентаря. S-082-086: campaign integration hardening, rules, forecasting, reporting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Критично до запуска плеера: без inventory плеер может получить конфликтующие размещения. Availability + reservation + campaign integration готовы (S-079). Дальше — конфликты (S-080) и календарь (S-081).</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>S-080: conflict detection. S-081: UI календарь. S-082: campaign integration hardening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>v0.7</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
           <t>Прогноз показов</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Позволяет планировать рекламные кампании на будущие периоды, оценивать доступность слотов и загрузку поверхностей.</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Нет данных для прогноза — нужен работающий PoP pipeline + статистика за период.
 Нет ML/статистической модели.</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>После production PoP pipeline — нужны реальные данные о показах за несколько месяцев для обучения модели.</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>После production PoP pipeline.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="10" t="inlineStr"/>
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Эксплуатация и безопасность</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
+          <t>v0.6</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
           <t>Emergency-управление</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Возможность мгновенно остановить показ всей рекламы при чрезвычайной ситуации. Кнопка «стоп» для всей сети.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: POST /emergency/activate|deactivate, GET /emergency/status.
 ✅ Admin-web: EmergencyPage — активация/деактивация с причиной.
@@ -3436,38 +3869,53 @@
 ✅ Outbox: emergency.changed события.</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>❌ Применение на устройствах — deferred (требуется KSO runtime).
 ❌ Нет MFA для emergency-пользователей.
 Почему: backend готов. Применение на устройствах ждёт player/KSO (v0.9).</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>После device gateway stable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Backend готов. Применение на устройствах ждёт KSO runtime (v0.9).</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Интеграция с KSO runtime (v0.9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>v0.6</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
           <t>Резервное копирование и DR</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>✅ Готово: PostgreSQL (S-031), MinIO (S-049), NATS (S-050)</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Защита от потери данных: база, медиафайлы, конфигурация. Возможность восстановления после сбоя.</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>✅ PostgreSQL: pg_dump backup + restore, drill test (5/5), runbook.
 ✅ MinIO: полный backup + manifest + SHA-256, restore с check/dry-run/confirm, runbook.
 ✅ NATS: outbox как source of truth, recovery через provisioning + relay replay (dedup-safe), runbook.</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>❌ Нет автоматического расписания бэкапов.
 ❌ Нет offsite-репликации.
@@ -3475,24 +3923,39 @@
 ❌ Нет нагрузочных тестов (ТЗ: 40 000 устройств).</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>До production-развёртывания. PostgreSQL, MinIO, NATS — все три компонента покрыты (S-031, S-049, S-050).</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>MinIO mirror + NATS policy — v0.6 (S-049/S-050).</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>v0.6</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Мониторинг и observability</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Чтобы видеть состояние платформы в реальном времени: жива ли, сколько запросов, есть ли ошибки. Prometheus + Grafana.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>✅ Prometheus метрики на control-api + device-gateway.
 ✅ Grafana дашборд «RMP Overview»: 4 секции, 10 панелей.
@@ -3501,276 +3964,449 @@
 ✅ Graceful shutdown (SIGTERM).</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>❌ Нет мониторинга инфраструктуры (CPU, RAM, диск).
 ❌ Grafana admin password не hardened для production.
 Почему: baseline observability готов. Инфраструктурный мониторинг — после production deploy.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>До масштабирования и до плееров — чтобы не строить runtime на непрозрачной платформе.</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>v0.6: Prometheus metrics endpoint + Grafana dashboard.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="n"/>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>v0.5–v0.6</t>
+        </is>
+      </c>
       <c r="B28" s="5" t="n"/>
       <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
+      <c r="D28" s="3" t="inlineStr"/>
       <c r="E28" s="3" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SECTION</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="10" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>v2.6 Next Branch</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Self-service advertiser cabinet</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>🟡 Готово для пилота</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Полноценный личный кабинет рекламодателя с самостоятельным управлением кампаниями, без участия оператора.</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>После стабилизации основного портала (v0.5). Сейчас pilot-ready — работает для демо.</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>S-023a-i completed. Pilot-ready for demo.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Sales Lift / Attribution proof</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Измерение влияния рекламы на продажи: какие показы привели к покупкам. Ключевая метрика для рекламодателя.</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>No attribution pipeline. No receipt data integration.</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>После tenant model ADR (ADR-018) и PoP pipeline. Требует интеграции с данными чеков.</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>After tenant model ADR + PoP pipeline.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Competitor blocking</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Запрет показа рекламы конкурентов на одном экране. Защита интересов рекламодателей.</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>No competitive separation model.</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>После tenant model ADR. Без разделения рекламодателей нельзя определить «конкурента».</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Store/audience targeting</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Таргетинг рекламы на конкретные магазины или профили магазинов. Повышает релевантность показов.</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>No store profiles. No audience targeting.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>После tenant model ADR и inventory — нужно знать, на каких поверхностях в каких магазинах есть свободные слоты.</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>After tenant model ADR + inventory.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Financial docs / reconciliation / integration</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Финансовые документы: счета, акты, сверки. Интеграция с 1С / ERP для биллинга рекламодателей.</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>No 1C/ERP API. No invoicing.</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>После tenant model ADR и production pilot — биллинг имеет смысл когда есть реальные показы и рекламодатели.</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Programmatic inventory sales</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Автоматизированная продажа рекламного инвентаря через внешние DSP/SSP платформы (OpenRTB).</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. OpenRTB stub.</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>No DSP/SSP integration.</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>После production pilot — нужен работающий инвентарь и стабильные показы для подключения внешних площадок.</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Dynamic creatives</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Креативы, которые меняются в реальном времени: цена, погода, остатки товара. Повышает вовлечённость.</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. HTML5 canvas/video templating.</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>No creative templating.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>После стабильного KSO плеера — требует HTML5-рендеринга на устройстве.</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>After KSO player stable.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Mobile field ops</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Мобильное приложение для полевых операторов: проверка экранов, замена контента на месте.</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Mobile app.</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>No mobile client.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>После KSO плеера — пока нет устройств в поле, нет потребности в полевых операциях.</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>After KSO player stable.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Independent DOOH measurement</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Независимый аудит показов по стандартам DOOH (Digital Out-of-Home). Доверие крупных рекламодателей.</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Design stub only.</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>No external impression audit.</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>После production pilot — нужно иметь стабильный поток показов для аудита.</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>

</xml_diff>

<commit_message>
feat: add inventory conflict detection rules
S-080 — Inventory Conflict Detection + Rules MVP

Conflict types (6):
- CAPACITY_OVERBOOKED — slot capacity exceeded
- SURFACE_INACTIVE — surface deleted or deactivated
- BLACKOUT_RULE — rule blocks time window
- INTERNAL_BLOCK — rule reserves internal capacity
- MAX_SOV_RULE — requested SOV exceeds rule max
- SOV_OVER_100 — total demand exceeds 100%

Rule engine:
- Scope precedence: surface > store > cluster > branch > global
- Priority breaks ties within same scope
- Time-window filter (starts_at/ends_at)
- Inactive rules excluded
- MVP: surface and global scopes fully supported

Integration:
- reserve_inventory_for_placement pre-checks conflicts
- request_approval fails if inventory blocked by rules

API:
- POST /inventory/conflicts/check (permission: inventory.read)
- GET /campaigns/{id}/inventory-conflicts

Tests: 18 unit (3 schema + 14 async conflict detection + 1 import)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1537,17 +1537,17 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>✅ Готово: S-077 schema/repo, S-078 availability, S-079 reservation + campaign integration. S-080+ запланировано.</t>
+          <t>✅ Готово: S-077/S-078/S-079/S-080. Conflict detection + rules MVP.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>S-076: architecture model. S-077: 3 tables + migration + repository. S-078: availability calculator + API. S-079: reserve/commit/release/expire lifecycle, auto-reserve at request_approval, commit at approve, release at reject. 24 unit tests. GET /campaigns/{id}/inventory-reservations.</t>
+          <t>S-076: model. S-077: schema. S-078: availability. S-079: reservation + campaign integration. S-080: 6 conflict types (SURFACE_INACTIVE, CAPACITY_OVERBOOKED, BLACKOUT_RULE, INTERNAL_BLOCK, MAX_SOV_RULE, SOV_OVER_100), rule engine with scope precedence, integration with reservation blocking, API endpoint.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>S-080 conflict detection engine. S-081 UI calendar. S-082 campaign integration hardening.</t>
+          <t>S-081 UI календарь инвентаря.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>✅ Готово: калькулятор + бронирование + интеграция с approval (S-079).</t>
+          <t>✅ Готово: availability + reservation + conflicts + rules (S-080)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -3732,20 +3732,18 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>✅ Inventory DB: слоты (surface × дата × час), бронирования (reserve/commit/release/expire).
-✅ Availability calculator: проверка свободных слотов.
-✅ Reservation lifecycle: автоматическое резервирование при запросе согласования, коммит при утверждении, освобождение при отклонении.
-✅ API: GET /campaigns/{id}/inventory-reservations.
-Что можно: размещения автоматически проверяются на доступность инвентаря. Нельзя согласовать кампанию, если инвентарь недоступен.</t>
+          <t>✅ Проверка доступности слотов.
+✅ Бронирование (reserve/commit/release/expire).
+✅ Авто-резервирование при запросе согласования.
+✅ Конфликт-детекция: неактивные поверхности, блэкаут-правила, внутренние блокировки, лимиты SOV, перебронирование.
+✅ Правила: blackout, internal_block, max_sov с приоритетами.</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>❌ Нет визуальной сетки/календаря инвентаря по магазинам.
-❌ Нет настройки правил (макс. нагрузка, prime-time, приоритеты).
+          <t>❌ Нет визуальной сетки/календаря инвентаря.
 ❌ Нет прогноза доступности.
-❌ Нет детекции конфликтов между кампаниями.
-Почему идём так: minimum inventory contract (availability + booking + campaign integration) готов. Дальше — конфликты (S-080) и календарь (S-081) перед KSO/player.</t>
+❌ Нет competitor separation (нет данных о категориях).</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -3755,7 +3753,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>S-080: conflict detection. S-081: UI календарь. S-082: campaign integration hardening.</t>
+          <t>S-081: UI календарь инвентаря.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add inventory availability calendar UI
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1547,12 +1547,12 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>S-081 UI календарь инвентаря.</t>
+          <t>✅ S-081 calendar UI done. Admin-web: 4 tabs (каталог/доступность/конфликты/правила). Availability checker + conflict checker + rules placeholder.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Minimum inventory contract: availability check ✅, booking/reservation ✅, campaign integration ✅. Player/KSO blocked until S-080/S-081 (conflicts + UI).</t>
+          <t>Minimum inventory contract: availability ✅, booking ✅, campaign integration ✅, conflicts ✅, UI calendar ✅. Ready for KSO preparation.</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>S-079 booking lifecycle + campaign integration. S-080 conflicts. S-081 UI calendar.</t>
+          <t>✅ S-081 UI calendar done.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3491,12 +3491,12 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Блокирован до минимального inventory-контракта (S-079). Без гарантии, что размещения не конфликтуют, плеер будет работать технически, но бизнес-правила будут неполными. Планируется на v0.9 после S-080/S-081.</t>
+          <t>Minimum inventory contract выполнен (S-081). KSO подготовку можно начинать на v0.9.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>После S-080/S-081 (конфликты + календарь инвентаря), затем v0.9.</t>
+          <t>Готово к началу подготовки (v0.9).</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Инвентарь рекламных мест</t>
+          <t>✅ Готово: availability + reservation + conflicts + rules + UI calendar (S-081)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -3736,7 +3736,8 @@
 ✅ Бронирование (reserve/commit/release/expire).
 ✅ Авто-резервирование при запросе согласования.
 ✅ Конфликт-детекция: неактивные поверхности, блэкаут-правила, внутренние блокировки, лимиты SOV, перебронирование.
-✅ Правила: blackout, internal_block, max_sov с приоритетами.</t>
+✅ Правила: blackout, internal_block, max_sov с приоритетами.
+✅ UI календарь инвентаря: 4 вкладки (каталог, доступность, конфликты, правила).</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -3753,7 +3754,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>S-081: UI календарь инвентаря.</t>
+          <t>✅ Minimum inventory contract complete. S-082: sold-out detection.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: review v0.7 inventory foundation readiness
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>✅ Готово: S-077/S-078/S-079/S-080. Conflict detection + rules MVP.</t>
+          <t>✅ Готово: S-077/S-078/S-079/S-080/S-081. Minimum inventory contract complete.</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1547,12 +1547,12 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>✅ S-081 calendar UI done. Admin-web: 4 tabs (каталог/доступность/конфликты/правила). Availability checker + conflict checker + rules placeholder.</t>
+          <t>✅ S-081 calendar UI done. S-082 readiness review done. v0.7-inventory-foundation release candidate.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Minimum inventory contract: availability ✅, booking ✅, campaign integration ✅, conflicts ✅, UI calendar ✅. Ready for KSO preparation.</t>
+          <t>Minimum inventory contract complete: availability ✅, reservation ✅, campaign integration ✅, conflicts ✅, UI calendar ✅. KSO prep can begin after v0.7.</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>✅ S-081 UI calendar done.</t>
+          <t>✅ S-081 UI calendar done. v0.7 release candidate.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1974,12 +1974,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Milestone: v0.6.2 опубликован (тег 90e91cb). v0.7 inventory foundation: S-076 design ✅, S-077 schema ✅, S-078 availability ✅. S-079 booking запланирован.</t>
+          <t>Milestone: v0.7-inventory-foundation release candidate. S-076–S-081 done: availability, reservation, conflicts, rules, UI calendar. KSO prep can begin.</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>develop HEAD = f993541. CI #29493671897 green 34/34.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Proposed tag: v0.7-inventory-foundation on f993541.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>S-046 plan: docs/product/v06-production-readiness-plan.md</t>
+          <t>Post-release: S-083 (sold-out), KSO architecture prep.</t>
         </is>
       </c>
     </row>
@@ -3468,35 +3478,37 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>⚪ Не начато (v0.7)</t>
+          <t>🟡 Готово к началу подготовки (v0.9)</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Кассы самообслуживания — первый физический канал показа рекламы в магазинах сети «Верный». Основной носитель для розничной рекламы.</t>
+          <t>Кассы самообслуживания — первый физический канал показа рекламы. Основной носитель для розничной рекламы.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>✅ Архитектура зафиксирована (ADR-013, ADR-016). Симулятор: 41 тест безопасности.
-✅ Device-gateway: GET /manifest/latest.
-✅ v0.5 Business Portal — блокер снят. KSO/player — v0.7 milestone.
-Почему ждём: без inventory (слоты + бронирование) плеер может получить конфликтующие размещения. Minimum inventory contract (availability + booking) должен быть готов до интеграции с реальным плеером.</t>
+          <t>✅ Minimum inventory contract выполнен — можно начинать архитектурную подготовку плеера.
+✅ Device-gateway: GET /manifest/latest работает.
+✅ Симулятор безопасности: 41 тест.
+Почему сейчас можно: минимальный inventory-контракт (availability + reservation + campaign integration + conflicts + UI) предотвращает конфликтующие размещения. Без него плеер получил бы слоты без гарантии эксклюзивности.</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Реального KSO плеера нет. Нет интеграции с железом КСО.</t>
+          <t>❌ Минимальный inventory контракт выполнен — блокер снят.
+Ограничение: rule management UI не готов (правила создаются через DB), но backend-движок работает.
+❌ Реального KSO плеера нет. Нет интеграции с железом.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Minimum inventory contract выполнен (S-081). KSO подготовку можно начинать на v0.9.</t>
+          <t>Минимальный inventory contract выполнен (S-081). Критическая зависимость (гарантия эксклюзивности слотов) закрыта. Подготовка архитектуры плеера теперь безопасна.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Готово к началу подготовки (v0.9).</t>
+          <t>Готово к началу подготовки (v0.9): архитектура устройства, верификация манифестов, рантайм плеера, rollout/rollback, диагностика.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: fix v0.7 readiness wording before publish
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Milestone: v0.7-inventory-foundation release candidate. S-076–S-081 done: availability, reservation, conflicts, rules, UI calendar. KSO prep can begin.</t>
+          <t>Milestone: v0.7-inventory-foundation release candidate (GO from S-082 review). Not yet published — ready for S-083 publish step.</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Proposed tag: v0.7-inventory-foundation on f993541.</t>
+          <t>Proposed tag: v0.7-inventory-foundation on f993541. Tag not created. Main not updated.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">

</xml_diff>

<commit_message>
docs: add business readiness gate before player
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -2931,7 +2931,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Самая первая функция — без входа нельзя построить ничего. Сделана в v0.1, улучшалась до v0.6 (реальный LDAPS).</t>
+          <t>MUST (✅ done): самая первая функция — без входа нельзя построить ничего. Сделана в v0.1. Self-service сброс пароля — CAN DEFER.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Основа безопасности. Сделано до campaign-логики, потому что все эндпоинты зависят от проверки прав.</t>
+          <t>MUST (✅ done): основа безопасности. Сделано до campaign-логики. UI для управления ролями — CAN DEFER.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Self-service снижает нагрузку на операторов. Сделано после RBAC и campaign API, потому что кабинет — это UI поверх готового backend.</t>
+          <t>MUST (✅ done): self-service снижает нагрузку на операторов. Рекламодатель не может сам утверждать — SHOULD before pilot (by design: admin must approve). Биллинг — CAN DEFER.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Ядро продукта. Сделано первым после аутентификации, потому что все остальные функции (креативы, отчёты) привязаны к кампании.</t>
+          <t>MUST (✅ done): ядро продукта. Календарь/drag-and-drop — CAN DEFER. UX/accessibility — SHOULD before pilot.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>После CRUD кампаний — чтобы цепочка «создал → отправил → проверили → запустили» работала полностью.</t>
+          <t>MUST (✅ done): цепочка «создал → отправил → проверили → запустили». Рекламодатель не утверждает сам — by design (security).</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>После базового CRUD кампаний, потому что креатив привязывается к кампании. До модерации — потому что загруженный файл нужно проверить.</t>
+          <t>MUST (✅ done): креатив привязывается к кампании. Malware scan/transcoding — CAN DEFER. Работает для пилота.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>После campaign и creative API — manifest собирает утверждённые кампании в плейлист. Это «выход» платформы на устройство.</t>
+          <t>MUST (✅ done): manifest собирает утверждённые кампании в плейлист. Signing verification — SHOULD before pilot.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Нужен сразу после manifest — устройству нужен способ безопасно получить плейлист.</t>
+          <t>MUST (✅ done): устройству нужен способ безопасно получить плейлист. mTLS — SHOULD before production.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>После device gateway — так как PoP-события приходят от устройств, получающих manifest.</t>
+          <t>MUST (✅ done): PoP-события от устройств. Реальный KSO плеер — вне backend-пилота. Интеграционный тест с реальным плеером — SHOULD before pilot.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>После PoP ingestion — данные сначала нужно принять и сохранить, потом показывать.</t>
+          <t>SHOULD (✅ done): данные сначала нужно принять, потом показывать. ClickHouse — CAN DEFER.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Минимальный inventory contract выполнен (S-081). Критическая зависимость (гарантия эксклюзивности слотов) закрыта. Подготовка архитектуры плеера теперь безопасна.</t>
+          <t>MUST (✅ done): минимальный inventory contract выполнен (S-081). Критическая зависимость (гарантия эксклюзивности слотов) закрыта. SHOULD before pilot: device health, rollout/rollback, operational dashboard, emergency-применение на устройствах.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>После пилота КСО — архитектура каналов позволяет подключать новые типы устройств без переписывания платформы.</t>
+          <t>CAN DEFER: второй канал после KSO pilot.</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Низкий приоритет. После КСО и Android TV.</t>
+          <t>CAN DEFER: низкий приоритет. После KSO + Android TV.</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Отдельный интеграционный проект. Зависит от доступности оборудования и API вендоров.</t>
+          <t>CAN DEFER: отдельный интеграционный проект.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Самый низкий приоритет среди каналов.</t>
+          <t>CAN DEFER: самый низкий приоритет.</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Критично до запуска плеера: без inventory плеер может получить конфликтующие размещения. Availability + reservation + campaign integration готовы (S-079). Дальше — конфликты (S-080) и календарь (S-081).</t>
+          <t>MUST (✅ done): критично до запуска плеера. Без inventory плеер получил бы конфликтующие размещения. Rule management UI — CAN DEFER. Прогноз — CAN DEFER.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -3804,7 +3804,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>После production PoP pipeline — нужны реальные данные о показах за несколько месяцев для обучения модели.</t>
+          <t>CAN DEFER: после production PoP pipeline. Статическая ёмкость достаточна для пилота.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Backend готов. Применение на устройствах ждёт KSO runtime (v0.9).</t>
+          <t>SHOULD: backend готов. Применение на устройствах ждёт KSO runtime (v0.9). Интеграция с KSO runtime — SHOULD before pilot.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>До production-развёртывания. PostgreSQL, MinIO, NATS — все три компонента покрыты (S-031, S-049, S-050).</t>
+          <t>MUST (✅ done): PostgreSQL, MinIO, NATS. Автоматическое расписание — SHOULD before production.</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>До масштабирования и до плееров — чтобы не строить runtime на непрозрачной платформе.</t>
+          <t>MUST (✅ done): до масштабирования и плееров. Инфраструктурный мониторинг — SHOULD before production.</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>После стабилизации основного портала (v0.5). Сейчас pilot-ready — работает для демо.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>После tenant model ADR (ADR-018) и PoP pipeline. Требует интеграции с данными чеков.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>После tenant model ADR. Без разделения рекламодателей нельзя определить «конкурента».</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>После tenant model ADR и inventory — нужно знать, на каких поверхностях в каких магазинах есть свободные слоты.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>После tenant model ADR и production pilot — биллинг имеет смысл когда есть реальные показы и рекламодатели.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>После production pilot — нужен работающий инвентарь и стабильные показы для подключения внешних площадок.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -4330,7 +4330,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>После стабильного KSO плеера — требует HTML5-рендеринга на устройстве.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>После KSO плеера — пока нет устройств в поле, нет потребности в полевых операциях.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>После production pilot — нужно иметь стабильный поток показов для аудита.</t>
+          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: add business functions completion gate before player
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -2931,7 +2931,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): самая первая функция — без входа нельзя построить ничего. Сделана в v0.1. Self-service сброс пароля — CAN DEFER.</t>
+          <t>SHOULD FIX (C): AD — stub, local основной. MFA отсутствует. Не блокирует плеер, но нужно до production.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): основа безопасности. Сделано до campaign-логики. UI для управления ролями — CAN DEFER.</t>
+          <t>✅ Готово. UI управления ролями — CAN DEFER. Не блокирует.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): self-service снижает нагрузку на операторов. Рекламодатель не может сам утверждать — SHOULD before pilot (by design: admin must approve). Биллинг — CAN DEFER.</t>
+          <t>✅ Готово для self-service создания кампаний. PDF/XLSX отчёты — BLOCKER BEFORE PILOT (B).</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -3107,12 +3107,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): ядро продукта. Календарь/drag-and-drop — CAN DEFER. UX/accessibility — SHOULD before pilot.</t>
+          <t>BLOCKER BEFORE PLAYER (A): прогноз доступности при создании кампании (A1). Календарь — CAN DEFER.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Advertiser self-service create/edit работает (S-023f).</t>
+          <t>S-086: интеграция availability checker в campaign create flow.</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): цепочка «создал → отправил → проверили → запустили». Рекламодатель не утверждает сам — by design (security).</t>
+          <t>✅ Готово. Цепочка работает. Advertiser не утверждает — by design.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): креатив привязывается к кампании. Malware scan/transcoding — CAN DEFER. Работает для пилота.</t>
+          <t>SHOULD FIX (C): загрузка работает. Антивирус — BLOCKER BEFORE PILOT (B). Превью/история версий — SHOULD FIX (C).</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): manifest собирает утверждённые кампании в плейлист. Signing verification — SHOULD before pilot.</t>
+          <t>✅ Готово. Signing verification — SHOULD FIX (C).</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): устройству нужен способ безопасно получить плейлист. mTLS — SHOULD before production.</t>
+          <t>✅ Готово. mTLS — SHOULD FIX (C).</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): PoP-события от устройств. Реальный KSO плеер — вне backend-пилота. Интеграционный тест с реальным плеером — SHOULD before pilot.</t>
+          <t>✅ Готово. Проверка с реальным плеером — BLOCKER BEFORE PILOT (B).</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -3418,12 +3418,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>SHOULD (✅ done): данные сначала нужно принять, потом показывать. ClickHouse — CAN DEFER.</t>
+          <t>BLOCKER BEFORE PLAYER (A): дашборд кампании с план/факт и причинами отклонений (A5). ClickHouse — CAN DEFER.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>После campaign UI стабилизации.</t>
+          <t>S-090: дашборд кампании с анализом отклонений.</t>
         </is>
       </c>
     </row>
@@ -3503,12 +3503,12 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): минимальный inventory contract выполнен (S-081). Критическая зависимость (гарантия эксклюзивности слотов) закрыта. SHOULD before pilot: device health, rollout/rollback, operational dashboard, emergency-применение на устройствах.</t>
+          <t>BLOCKER BEFORE PLAYER (A): нельзя начинать плеер пока A1–A6 не закрыты. S-086–S-091 сначала.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Готово к началу подготовки (v0.9): архитектура устройства, верификация манифестов, рантайм плеера, rollout/rollback, диагностика.</t>
+          <t>S-086–S-091: закрыть 6 BLOCKER BEFORE PLAYER. Потом player architecture.</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: низкий приоритет. После KSO + Android TV.</t>
+          <t>CAN DEFER.</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: отдельный интеграционный проект.</t>
+          <t>CAN DEFER.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: самый низкий приоритет.</t>
+          <t>CAN DEFER.</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -3761,12 +3761,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): критично до запуска плеера. Без inventory плеер получил бы конфликтующие размещения. Rule management UI — CAN DEFER. Прогноз — CAN DEFER.</t>
+          <t>BLOCKER BEFORE PLAYER (A): нет sold-out + альтернатив (A2), нет настройки правил в UI (A3). Прогноз — CAN DEFER.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>✅ Minimum inventory contract complete. S-082: sold-out detection.</t>
+          <t>S-087 sold-out alternatives + S-088 rules admin UI.</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: после production PoP pipeline. Статическая ёмкость достаточна для пилота.</t>
+          <t>CAN DEFER: статическая ёмкость достаточна для пилота.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -3889,12 +3889,12 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>SHOULD: backend готов. Применение на устройствах ждёт KSO runtime (v0.9). Интеграция с KSO runtime — SHOULD before pilot.</t>
+          <t>BLOCKER BEFORE PLAYER (A): emergency не применяется на устройствах (A6). MFA — SHOULD FIX (C).</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Интеграция с KSO runtime (v0.9).</t>
+          <t>S-091: emergency-применение на устройствах.</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): PostgreSQL, MinIO, NATS. Автоматическое расписание — SHOULD before production.</t>
+          <t>✅ Готово. Авто-расписание — SHOULD FIX (C).</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>MUST (✅ done): до масштабирования и плееров. Инфраструктурный мониторинг — SHOULD before production.</t>
+          <t>✅ Готово. Инфраструктурный мониторинг — SHOULD FIX (C).</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -4330,7 +4330,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER: v2.6 Next Branch. Не блокирует KSO pilot.</t>
+          <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: show inventory availability forecast during campaign creation
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2785,6 +2785,33 @@
       <c r="E88" t="inlineStr">
         <is>
           <t>P1 — first channel live. BLOCKED until v0.5 Business Portal Complete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>S-086</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>✅ A1 done: availability forecast during campaign creation. CampaignCreatePage + CampaignDetailPage placement tab.</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Admin-web: forecast section in create form (surface selector + check button). Detail page: "🔍 Доступность" button in placement form.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>S-087 sold-out alternatives (A2).</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>No backend changes. Uses existing POST /inventory/availability. 2 vitest tests.</t>
         </is>
       </c>
     </row>
@@ -3107,12 +3134,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>BLOCKER BEFORE PLAYER (A): прогноз доступности при создании кампании (A1). Календарь — CAN DEFER.</t>
+          <t>BLOCKER A1 ✅ done: прогноз доступности при создании кампании (S-086). A2–A6 остаются. Календарь — CAN DEFER.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>S-086: интеграция availability checker в campaign create flow.</t>
+          <t>S-087 sold-out alternatives (A2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(D2): align roadmap with PROJECT_STATE — honest C1/C2/H0/D1 statuses
Roadmap changes:
- R53 Creative Moderation: ✅→🟡 C1 fixed on develop, merge to main pending
- R55 Campaign Approval: ✅→🟡 C1 fixed on develop, merge pending after D2
- R60 Real LDAPS: ✅ S-048 done → ✅ C2 resolved (SHA 47e7d44, CI #29519917049)
- R82 Identity Hardening: ✅→✅ C2 resolved, cert validation fail-secure
- R84 Creative Moderation Manual: ⚪→🟡 C1 moderation queue on develop
- R4 Outbox: +H0 note (flaky fix, ADR-008 green, CI #29515994509)
- R78 Production Gaps: +D1 note (TZ table reattachment, SHA 9216a54)

Rules:
- roadmap-maintenance-rules.md: new section «Синхронизация с PROJECT_STATE»
  with behavioral proof alignment rule
- PROJECT_STATE.md: HEAD→9216a54, D1 resolved, D2 in progress

Workbook structure: 2 sheets, 91+38 rows — unchanged.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -637,7 +637,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Transactional outbox pattern.</t>
+          <t>Transactional outbox pattern. H0 resolved: flaky test_backoff_respected_on_second_run stabilised (SHA 39dc8bc, CI #29515994509). ADR-008 gate green.</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>✅ S-036 done</t>
+          <t>🟡 C1: fixed on develop (behavioural proof: 8 tests, NOBYPASSRLS). Merge to main pending after D2.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1849,12 +1849,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Malware scan deferred to v0.7.</t>
+          <t>Merge to main. ADR-008 gate green ✓ (H0 resolved, CI #29515994509).</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>v0.5 gate: manual moderation before displays show content.</t>
+          <t>C1 = Creative Moderation + Campaign Approval RLS. Bug fixed: AdvertiserOrganization.name→legal_name. Seed: creatives.moderate added.</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>✅ S-038 done</t>
+          <t>🟡 C1: fixed on develop. Merge to main pending after D2.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1903,12 +1903,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Advertiser resubmit after rejection (v0.6).</t>
+          <t>Merge to main. ADR-008 gate green (H0).</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>v0.5: full approval cycle (submit → review → reject → edit → resubmit).</t>
+          <t>C1: approval queue + moderation queue RLS on 4 endpoints. Cross-tenant 404 proven.</t>
         </is>
       </c>
     </row>
@@ -2028,22 +2028,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>✅ S-048 done</t>
+          <t>✅ C2 resolved (SHA 47e7d44, CI #29519917049. Real bug: two silent CERT_NONE paths.)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>RealLDAPAuthProvider with ldap3 bind+search. Safe filter escaping. Timeouts. No password logs. Stub preserved when AD_ENABLED=false.</t>
+          <t>SHA 47e7d44. CI #29519917049: 34/34 green. 10 TLS tests. Fail-secure else for unknown cert_val.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Production deploy: TLS cert validation + secrets management.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>P0 — blocks real admin access.</t>
+          <t>C2 Critical: ad_use_tls gate + unrecognised cert_val → tls=None → CERT_NONE. Fix: removed gate, else→CERT_REQUIRED.</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>No code changes. Docs-only triage.</t>
+          <t>No code changes. Docs-only triage. D1 resolved: extracted TZ table reattachment (SHA 9216a54). Section 14 now has security reqs, not device statuses.</t>
         </is>
       </c>
     </row>
@@ -2607,22 +2607,22 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>✅ Готово</t>
+          <t>✅ C2 resolved: LDAPS cert validation fail-secure (SHA 47e7d44, CI #29519917049)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>AD stub returns 503. No real LDAPS integration.</t>
+          <t>C2: RealLDAPAuthProvider._connect() always creates TLS with cert policy. CERT_REQUIRED enforced.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>real LDAPS bind+search via ldap3. Stub preserved for AD_ENABLED=false. local_advertiser + break_glass preserved.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>P1 — blocks real admin access.</t>
+          <t>C2 was a real bug — required silently degraded to CERT_NONE via two paths. Now fail-secure.</t>
         </is>
       </c>
     </row>
@@ -2661,22 +2661,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟡 C1: moderation queue + RLS on develop. Merge to main pending.</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CREATIVE_AUTO_APPROVE_UPLOADS=true. No human review.</t>
+          <t>C1: GET /creative-assets/moderation-queue, POST approve/reject (NOBYPASSRLS). 8 behavioural tests.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Admin-web moderation queue. Approve/reject with reason.</t>
+          <t>Merge to main after D2.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>P1 — quality control before live.</t>
+          <t>C1: manual moderation backend complete. Malware scan still deferred.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(D2 follow-up): dictionary statuses in roadmap, D2→RESOLVED
Roadmap status column now uses only dictionary values:
- R53 Creative Moderation: 🟡 Готово для пилота
- R55 Campaign Approval: 🟡 Готово для пилота
- R60 Real LDAPS: ✅ Готово
- R82 Identity Hardening: ✅ Готово
- R84 Creative Moderation Manual: 🟡 Готово для пилота

C1/C2/H0/D1 proof moved to Коммиты/Тесты/ADR and Заметки columns.
PROJECT_STATE.md: HEAD→df3b946, D2→RESOLVED, C1 next step→merge after D2 resolved.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1839,22 +1839,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>🟡 C1: fixed on develop (behavioural proof: 8 tests, NOBYPASSRLS). Merge to main pending after D2.</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Backend: GET moderation-queue, POST approve/reject with creatives.moderate permission. Admin-web: CreativeModerationPage. Advertiser-web: moderation status display. creative_auto_approve_uploads=False.</t>
+          <t>C1: 8 behavioural tests (NOBYPASSRLS). 4 RLS endpoints: moderation queue + approve/reject. Bug fixed: AdvertiserOrganization.name→legal_name.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Merge to main. ADR-008 gate green ✓ (H0 resolved, CI #29515994509).</t>
+          <t>Merge to main after D2. ADR-008 gate green ✓ (H0 resolved, CI #29515994509).</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>C1 = Creative Moderation + Campaign Approval RLS. Bug fixed: AdvertiserOrganization.name→legal_name. Seed: creatives.moderate added.</t>
+          <t>C1 blocks: seed — creatives.moderate added to system_admin/security_admin role_permissions.</t>
         </is>
       </c>
     </row>
@@ -1893,22 +1893,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>🟡 C1: fixed on develop. Merge to main pending after D2.</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Backend: GET /campaigns/approval-queue with readiness summary. Admin-web: ApprovalInboxPage — approve/reject with readiness checklist + creative moderation gate.</t>
+          <t>C1: GET /campaigns/approval-queue (NOBYPASSRLS). 8 behavioural tests pass. Cross-tenant 404 proven.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Merge to main. ADR-008 gate green (H0).</t>
+          <t>Merge to main after D2. ADR-008 gate green (H0).</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>C1: approval queue + moderation queue RLS on 4 endpoints. Cross-tenant 404 proven.</t>
+          <t>C1 = Creative Moderation + Campaign Approval RLS as a unit. Both fixed on develop.</t>
         </is>
       </c>
     </row>
@@ -2028,12 +2028,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>✅ C2 resolved (SHA 47e7d44, CI #29519917049. Real bug: two silent CERT_NONE paths.)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SHA 47e7d44. CI #29519917049: 34/34 green. 10 TLS tests. Fail-secure else for unknown cert_val.</t>
+          <t>SHA 47e7d44. CI #29519917049: 34/34 green. 10 TLS tests. Fail-secure else for unknown cert_val. ldap3 in requirements+CI.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>C2 Critical: ad_use_tls gate + unrecognised cert_val → tls=None → CERT_NONE. Fix: removed gate, else→CERT_REQUIRED.</t>
+          <t>C2 Critical resolved: ad_use_tls gate + unrecognised cert_val → tls=None → CERT_NONE. Fix: removed gate, else→CERT_REQUIRED.</t>
         </is>
       </c>
     </row>
@@ -2607,12 +2607,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>✅ C2 resolved: LDAPS cert validation fail-secure (SHA 47e7d44, CI #29519917049)</t>
+          <t>✅ Готово</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>C2: RealLDAPAuthProvider._connect() always creates TLS with cert policy. CERT_REQUIRED enforced.</t>
+          <t>C2: RealLDAPAuthProvider._connect() always creates TLS with cert policy. CERT_REQUIRED enforced. SHA 47e7d44, CI #29519917049.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2661,22 +2661,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>🟡 C1: moderation queue + RLS on develop. Merge to main pending.</t>
+          <t>🟡 Готово для пилота</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>C1: GET /creative-assets/moderation-queue, POST approve/reject (NOBYPASSRLS). 8 behavioural tests.</t>
+          <t>C1: GET /creative-assets/moderation-queue, POST approve/reject (NOBYPASSRLS). 8 behavioural tests pass.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Merge to main after D2.</t>
+          <t>Merge to main after D2. Malware scan still deferred.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>C1: manual moderation backend complete. Malware scan still deferred.</t>
+          <t>C1: manual moderation backend complete on develop. CREATIVE_AUTO_APPROVE_UPLOADS still default for dev convenience.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(D3): roadmap coverage audit — add 28 missing TZ requirement rows
Sheet 1 (Технический Roadmap): +16 rows (now 107)
Sheet 2 (Бизнес-функции): +12 rows (now 50)

Covers:
  §5/22.2 SLA/NFT — 99.5/99.9%, RTO 4ч, RPO 15м
  §14 SIEM/Wazuh, mTLS/cert rotation, HTML5 sandbox/CSP, PII, VPN-only
  §16.2 УКМ4 integration (Attribution v2.6)
  §22.3 Недопоказы / компенсации (make-good)
  §22.6 Device fleet health dashboard
  §22.7 Staged rollout / rollback
  §22.9 Feature flags
  §22.11 Data Governance / retention / partitioning
  §22.15 Нагрузочные профили / performance criteria
  §22.17 Timezone / calendar / holiday scheduling
  §24 Channel Orchestrator / Adapter Layer

Statuses: ⚪ Не начато (11), 🚫 Отложено (1: HTML5 sandbox),
🧭 Требует решения (2: Channel Orchestrator, Admin VPN-only)
No ✅ Готово — все требуют коммита/теста/proof.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2866,6 +2866,370 @@
       <c r="E91" t="inlineStr">
         <is>
           <t>13 backend + 124 vitest. Full CI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>SECTION</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ТЗ-покрытие (D3 audit)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Добавлено 2026-07-16 при D3 Roadmap coverage audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>§14 SIEM / Wazuh export</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>S-092</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Передача логов в SIEM/Wazuh согласно §14 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>§14 mTLS / device cert rotation</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>S-093</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Ротация сертификатов устройств, отзыв, mTLS согласно §14 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>§14 HTML5 sandbox / CSP enforcement</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>🚫 Отложено</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>После решения ИБ</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Sandbox + CSP для HTML5-креативов согласно §14 и §22.5 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>§14 PII minimisation</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>S-094</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Минимизация персональных данных, разграничение доступа согласно §14 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>§14 Admin VPN-only access</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>🧭 Требует решения</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Зависит от инфраструктуры</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Доступ к админке только из корп. сети/VPN согласно §4.3 и §14 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>§5 / §22.2 SLA 99.5/99.9% + RTO 4ч / RPO 15м</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>S-095</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Целевые SLA: Control Plane 99.5%, Device GW 99.9%, RTO 4ч, RPO 15м согласно §5 и §22.2 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>§16.2 УКМ4 integration (Attribution v2.6)</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>v2.6 Attribution</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Интеграция с чеками УКМ4 для оценки охвата. Пакетная загрузка → регулярная согласно §16.2 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>§22.3 Недопоказы / компенсации (make-good)</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>S-096</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Учёт недопоказов, классификация причин, предложение компенсаций согласно §22.3 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>§22.6 Device fleet health dashboard</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>S-097</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Операционный центр здоровья носителей: онлайн/офлайн/ошибки/detailed view согласно §22.6 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>§22.7 Staged rollout / rollback</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>S-098</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Поэтапный rollout: лаб→5→50→300→10%→50%→сеть. Auto-stop по метрикам согласно §22.7 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>§22.9 Feature flags</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>S-099</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Feature flags с аудитом и rollback для безопасного развития согласно §22.9 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>§22.11 Data Governance / retention / partitioning</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>S-100</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Правила хранения: PoP 12–18 мес, архив 3–5 лет, аудит 3+ лет, партиционирование согласно §22.11 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>§22.15 Нагрузочные профили и performance criteria</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>S-101</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Профили: 40K KSO + heartbeat/PoP/manifest/emergency + аналитика + админка согласно §22.15 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>§22.17 Timezone / calendar / holiday scheduling</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>S-102</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Часовые пояса (UTC+локальный), календарь, праздники, ночные интервалы согласно §22.17 ТЗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>§24 Channel Orchestrator / Adapter Layer</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>🧭 Требует решения</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ADR требуется</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Channel Orchestrator + Adapter SDK + adapter_payload в manifest согласно §24 ТЗ</t>
         </is>
       </c>
     </row>
@@ -2881,7 +3245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4504,6 +4868,431 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ТЗ-покрытие (D3 audit)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SLA/NFT: 99.5/99.9% доступность, RTO 4ч, RPO 15м</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>S-095</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Рекламодатели и бизнес видят гарантии качества услуги</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Инвентарь/кампании без привязки к SLA</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>SLA не утверждены с бизнесом</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Мониторинг недопоказов и компенсации</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>S-096</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Автоматический расчёт компенсаций при недовыполнении плана</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Ручной пересчёт недопоказа без классификации причин</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Нет автоматического предложения докрутки</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Операционный центр здоровья устройств</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>S-097</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ИТ-поддержка видит все устройства, их статус и ошибки</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Нет единой картины здоровья сети носителей</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Данные heartbeat есть, но нет операционного интерфейса</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Staged rollout и rollback</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>S-098</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Безопасное обновление плееров/manifest без массовых сбоев</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Любое изменение затрагивает всю сеть сразу</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Нет механизма поэтапного выкатывания</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Интеграция с УКМ4 / чековые данные</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Attribution v2.6</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Оценка охвата через чеки для Sales Lift</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Показы считаются без привязки к транзакциям</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Требуется согласование с владельцем УКМ4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Feature flags для безопасного развития</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>S-099</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Включение функций на пилотные магазины без риска для сети</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Все изменения применяются глобально</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Нет инфраструктуры feature flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Data Governance: retention, партиционирование</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>S-100</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Соответствие требованиям хранения данных и юр. нормам</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Данные хранятся без явных политик TTL</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Нет утверждённых сроков хранения с юристами</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Нагрузочное тестирование 40K устройств</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>S-101</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Подтверждение способности системы работать под расчётной нагрузкой</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Тесты только на малых объёмах данных</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Нет утверждённых профилей нагрузки</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Часовые пояса и календарь показов</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>S-102</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Корректное расписание во всех часовых поясах РФ с учётом праздников</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Только UTC/Moscow, без календаря исключений</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Требуется дизайн модели хранения tz-aware данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Channel Orchestrator / Adapter Layer</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>🧭 Требует решения</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ADR требуется</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Единый слой адаптеров для KSO/Android/ESL/LED</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>КСО-центричная архитектура</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Нет ADR, нет абстракции адаптеров</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SIEM/Wazuh + ИБ-мониторинг</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>⚪ Не начато</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>S-092</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Передача критичных событий в SIEM для ИБ</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Логи只在 локальных файлах</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Требуется согласование с ИБ-отделом</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: RM1 — roadmap sync after K1/K2
- Sheet 1 (Тех): R20C4 signature verification no longer deferred (K2)
- Sheet 1 (Тех): R45 emergency management reflects K1 resolved
- Sheet 1 (Тех): R24 simulator notes K2 verification
- Sheet 2 (Бизнес): R11/R12 signature verify resolved (K2)
- Sheet 2 (Бизнес): R25 emergency split: manifest-level K1 resolved,
  player-side still deferred
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1028,12 +1028,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Device-gateway signature verification (deferred)</t>
+          <t>K2 resolved: runtime simulator verifies manifest signature before apply/play. CI #29638045838.</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>HMAC-SHA256 signing implemented (S-021). Production config hardened (S-021a). compute_manifest_id + compute_campaign_version_hash.</t>
+          <t>HMAC-SHA256 signing implemented (S-021). Production config hardened (S-021a). compute_manifest_id + compute_campaign_version_hash. K2: manifest signing moved to contracts/manifest_signing.py. Simulator: real HMAC-SHA256 verification before apply.</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>ADR-013 headless simulator: manifest apply, kill-switch (4 levels, fail-closed), render slot (6 gates), PoP integrity, offline TTL. 41 tests.</t>
+          <t>ADR-013 headless simulator: manifest apply, kill-switch (4 levels, fail-closed), render slot (6 gates), PoP integrity, offline TTL. 41 tests. K2: manifest signature verification before apply (CI #29638045838, 27 tests).</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1628,7 +1628,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Emergency Management</t>
+          <t>Emergency Management (K1 resolved)</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>POST /emergency/activate|deactivate, GET /emergency/status. Admin-web EmergencyPage. Permissions emergency.read|manage. Outbox emergency.changed. Player-side enforcement deferred.</t>
+          <t>POST /emergency/activate|deactivate, GET /emergency/status. Admin-web EmergencyPage. Permissions emergency.read|manage. Outbox emergency.changed. Player-side enforcement deferred. K1: emergency override flows to device manifest (CI #29636889061, 4 behavioural tests).</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>No emergency API. No MFA for emergency users. No UI.</t>
+          <t>KSO player-side emergency enforcement (deferred). Manifest-level emergency propagation: K1 resolved.</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
@@ -3702,14 +3702,14 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Верификация подписи на device-gateway (signing есть, verify deferred).
+          <t>Верификация подписи манифеста: K2 resolved — runtime simulator проверяет подпись до apply/play (CI #29638045838).
 Nested per-surface playlist — Manifest v2.
 Манифест доставляется только в тестах (нет реального плеера).</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>✅ Готово. Signing verification — SHOULD FIX (C).</t>
+          <t>✅ Готово. K2 resolved: signing verification done. Real KSO player: deferred.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -3750,7 +3750,7 @@
       <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Только HTTP (не HTTPS/mTLS).
-Верификация подписи manifest на устройстве (backend signing есть, verify deferred).
+Верификация подписи manifest: K2 resolved — runtime simulator проверяет подпись до apply (CI #29638045838).
 Нет emergency-канала для срочных команд.
 Нет реального KSO плеера, принимающего manifest.</t>
         </is>
@@ -3762,8 +3762,8 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>mTLS после интеграции с KSO плеером.
-Production manifest signing.</t>
+          <t>K2 resolved: manifest signing verification. mTLS — deferred.
+Next: RM1/R1/T1 process hygiene -&gt; release v0.8.</t>
         </is>
       </c>
     </row>
@@ -4303,6 +4303,7 @@
       <c r="E25" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: POST /emergency/activate|deactivate, GET /emergency/status.
+K1 resolved: emergency состояние попадает в device manifest (emergency.active, activated_at, reason). CI #29636889061.
 ✅ Admin-web: EmergencyPage — активация/деактивация с причиной.
 ✅ Аудит всех emergency-действий.
 ✅ Outbox: emergency.changed события.</t>
@@ -4310,7 +4311,8 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>❌ Применение на устройствах — deferred (требуется KSO runtime).
+          <t>✅ Manifest-level emergency: K1 resolved (manifest содержит реальное emergency состояние: active, activated_at, reason). CI #29636889061.
+❌ Player-side enforcement на реальном KSO — deferred (требуется KSO runtime).
 ❌ Нет MFA для emergency-пользователей.
 Почему: backend готов. Применение на устройствах ждёт player/KSO (v0.9).</t>
         </is>
@@ -4322,7 +4324,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>S-091: emergency-применение на устройствах.</t>
+          <t>K1 resolved: emergency override -&gt; manifest. Player-side KSO enforcement: phase 1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RECONCILE-001: roadmap overclaims removed — 7 rows, honest statuses
- 7 business functions: «Готово» → «🟠 Бэкенд готов, UI-smoke нет»
- Rows: 3 (Вход), 4 (Роли), 5 (Кабинет), 7 (Кампании), 8 (Согласование), 9 (Креативы), 22 (Инвентарь)
- Limitations updated with blocked journey IDs (G1–G4, campaign.create, user.assign_roles, self.*, inventory.*)
- Workbook structure preserved: 2 sheets, 50×8
- Consistency audit: 0 violations
- Next: G1-FIX
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3334,7 +3334,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>🟡 Готово для пилота</t>
+          <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -3354,7 +3354,8 @@
         <is>
           <t>❌ Нет self-service сброса пароля.
 ❌ Нет инвайт-писем для новых рекламодателей.
-Почему: базовый вход работает. Self-service onboarding — v0.8.</t>
+Почему: базовый вход работает. Self-service onboarding — v0.8.
+❌ UI-TRUTH: blocked — campaign.create (G1), self.login, advertiser.create_org. UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3381,7 +3382,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>✅ Готово</t>
+          <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3399,7 +3400,8 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Нет UI для управления ролями и назначения прав (только API).</t>
+          <t>Нет UI для управления ролями и назначения прав (только API).
+❌ UI-TRUTH: blocked — user.assign_roles (G2), user.create_advertiser. UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3426,7 +3428,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>✅ Готово</t>
+          <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -3445,7 +3447,8 @@
           <t>❌ Рекламодатель не может сам утверждать кампании — только admin.
 ❌ Нет биллинга/атрибуции.
 ❌ Production UX audit отложен.
-Почему: self-service пилот работает. Полный production UX — после стабилизации backend.</t>
+Почему: self-service пилот работает. Полный production UX — после стабилизации backend.
+❌ UI-TRUTH: blocked — self.login, self.campaign_view, self.report_view. Advertiser-web не проходил UI-аудит.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3510,7 +3513,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>🟡 Готово для пилота</t>
+          <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -3530,7 +3533,8 @@
           <t>❌ Нет календаря планирования.
 ❌ Нет drag-and-drop.
 ❌ UX/accessibility не завершены.
-❌ Нет браузерных E2E-тестов.</t>
+❌ Нет браузерных E2E-тестов.
+❌ UI-TRUTH: blocked — campaign.create (G1), campaign.edit, campaign.submit, campaign.activate.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -3557,7 +3561,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>🟡 Готово для пилота</t>
+          <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -3575,7 +3579,8 @@
       <c r="F8" s="3" t="inlineStr">
         <is>
           <t>❌ Рекламодатель не может сам утверждать — только отправляет.
-Почему: это осознанное ограничение безопасности.</t>
+Почему: это осознанное ограничение безопасности.
+❌ UI-TRUTH: blocked — campaign.approve, campaign.reject. UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3602,7 +3607,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>🟡 Готово для пилота</t>
+          <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -3619,7 +3624,8 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Malware scan, transcoding, CDN — отложены.</t>
+          <t>Malware scan, transcoding, CDN — отложены.
+❌ UI-TRUTH: blocked — creative.upload, creative.moderate_approve, creative.moderate_reject.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -4162,7 +4168,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>✅ Готово: availability + reservation + conflicts + rules (S-080)</t>
+          <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -4184,7 +4190,8 @@
         <is>
           <t>❌ Нет визуальной сетки/календаря инвентаря.
 ❌ Нет прогноза доступности.
-❌ Нет competitor separation (нет данных о категориях).</t>
+❌ Нет competitor separation (нет данных о категориях).
+❌ UI-TRUTH: blocked — inventory.simulate, inventory.rule_create. UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: ROADMAP-DONE-GATE-001 — 4-column business roadmap, G1/G2 honestly ready
Business sheet: single «Статус» → 4 columns (Бэкенд, UI, Юзер-стори, Итог).
G1 (campaign.create): ✅/✅/✅ → Готово/Юзабельно.
G2 (user.assign_roles): ✅/✅/✅ → Готово/Юзабельно.
campaign.edit: ✅/⚪️/⚪️ → Частично (edit не reachable).
feature-registry: reachable 5→7.
AGENTS.md: Done Gate rule #7 — roadmap sync mandatory.
Next: ROADMAP-GUARD-002.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3228,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3254,30 +3254,45 @@
       </c>
       <c r="C1" s="9" t="inlineStr">
         <is>
-          <t>Статус</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
+          <t>Бэкенд</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Юзер-стори (journey)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Итог</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>Для чего нужна</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>Что уже можно использовать</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>Что ещё нельзя / ограничения</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>Почему сейчас / зависимость</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>Следующий шаг</t>
         </is>
@@ -3295,27 +3310,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F2" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3334,15 +3349,30 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Чтобы сотрудники офиса и рекламодатели могли войти в систему безопасно, каждый под своей учётной записью, без передачи паролей в открытом виде.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>✅ Вход через local_advertiser и local_break_glass (bcrypt).
 ✅ Admin-web: страница логина с выбором провайдера (Рекламодатель / Break-glass Admin / Сотрудник AD).
@@ -3350,7 +3380,7 @@
 ✅ Реальный LDAPS (S-048): ldap3 bind+search, safe filter escaping, таймауты. Stub preserved при AD_ENABLED=false.</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>❌ Нет self-service сброса пароля.
 ❌ Нет инвайт-писем для новых рекламодателей.
@@ -3358,12 +3388,12 @@
 ❌ UI-TRUTH: blocked — campaign.create (G1), self.login, advertiser.create_org. UI-smoke отсутствует.</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>SHOULD FIX (C): AD — stub, local основной. MFA отсутствует. Не блокирует плеер, но нужно до production.</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Готово (S-048). Self-service сброс пароля — v0.8.</t>
         </is>
@@ -3382,15 +3412,30 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>🟠 Бэкенд готов, UI-smoke нет</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>✅ user.assign_roles</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅ Готово/Юзабельно</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Чтобы разные роли (админ, оператор, аналитик) видели только то, что им положено. Безопасность данных рекламодателей.</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>4 системные роли (system_admin, security_admin, operator, analyst).
 16 permissions с backend-проверкой.
@@ -3398,18 +3443,18 @@
 Scoped-доступ: branch, cluster, store, advertiser.</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Нет UI для управления ролями и назначения прав (только API).
 ❌ UI-TRUTH: blocked — user.assign_roles (G2), user.create_advertiser. UI-smoke отсутствует.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. UI управления ролями — CAN DEFER. Не блокирует.</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3428,21 +3473,36 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Чтобы рекламодатель мог сам создавать кампании, загружать креативы и смотреть отчёты — без помощи администратора.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>✅ Advertiser-web (http://192.168.110.77:3001): вход, создание/редактирование кампаний, библиотека креативов, загрузка, прикрепление к кампании, отправка на согласование, PoP-отчёты + CSV экспорт, профиль/смена пароля.
 ✅ Admin-web: полное управление рекламодателями.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>❌ Рекламодатель не может сам утверждать кампании — только admin.
 ❌ Нет биллинга/атрибуции.
@@ -3451,12 +3511,12 @@
 ❌ UI-TRUTH: blocked — self.login, self.campaign_view, self.report_view. Advertiser-web не проходил UI-аудит.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>✅ Готово для self-service создания кампаний. PDF/XLSX отчёты — BLOCKER BEFORE PILOT (B).</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Production UX audit (deferred). Browser E2E (deferred).</t>
         </is>
@@ -3474,27 +3534,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3513,22 +3573,37 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>🟠 Бэкенд готов, UI-smoke нет</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>✅ (create) / ⚪️ (edit)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>✅ campaign.create / ⚪️ campaign.edit</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>🟠 Частично (edit не reachable)</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Основной рабочий инструмент: создание, настройка и управление рекламными кампаниями (бюджет, сроки, поверхности).</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: полный CRUD кампаний (7 endpoints), пролёты, размещения, креативы.
 ✅ Admin-web: список с фильтром, мастер создания, 5 вкладок (пролёты, размещения, креативы+upload, согласование, PoP-отчёты).
 ✅ Advertiser-web: создание/редактирование черновиков.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>❌ Нет календаря планирования.
 ❌ Нет drag-and-drop.
@@ -3537,12 +3612,12 @@
 ❌ UI-TRUTH: blocked — campaign.create (G1), campaign.edit, campaign.submit, campaign.activate.</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>BLOCKER A1 ✅ done: прогноз доступности при создании кампании (S-086). A2–A6 остаются. Календарь — CAN DEFER.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>A3 ✅ S-088 rules admin UI. A4–A6 remain.</t>
         </is>
@@ -3561,34 +3636,49 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Чтобы ни одна кампания не пошла в показ без проверки администратором: правильные ли креативы, не нарушен ли бюджет.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: request-approval → approve/reject с audit trail.
 ✅ Admin-web: очередь согласования, approve/reject с причиной.
 ✅ Advertiser-web: отправка на согласование, видимость статуса/причины отклонения.</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>❌ Рекламодатель не может сам утверждать — только отправляет.
 Почему: это осознанное ограничение безопасности.
 ❌ UI-TRUTH: blocked — campaign.approve, campaign.reject. UI-smoke отсутствует.</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Цепочка работает. Advertiser не утверждает — by design.</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>После campaign UI (S-009c).</t>
         </is>
@@ -3607,33 +3697,48 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Чтобы рекламодатели могли загружать изображения и видео для показа на экранах. Хранение — в защищённом MinIO (S3).</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Backend: presigned URL (MinIO/S3) + SHA-256.
 Admin-web UI: загрузка с прогресс-баром.
 Advertiser-web: библиотека + загрузка + привязка к кампании (S-023c, S-023g).</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Malware scan, transcoding, CDN — отложены.
 ❌ UI-TRUTH: blocked — creative.upload, creative.moderate_approve, creative.moderate_reject.</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>SHOULD FIX (C): загрузка работает. Антивирус — BLOCKER BEFORE PILOT (B). Превью/история версий — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>Malware scan, transcoding, manual moderation — отложены.
 Работает для пилота.</t>
@@ -3652,27 +3757,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3691,34 +3796,49 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Автоматически формирует плейлист для каждого устройства: какие креативы и в каком порядке показывать. Без этого плеер не знает, что играть.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Manifest JSON с полями: device_id, store_id, playlist[], media_files[], valid_from/to, offline_ttl_hours.
 ETag/304 — кэширование на устройстве.
 Автоматическая генерация при изменении кампании.</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Верификация подписи манифеста: K2 resolved — runtime simulator проверяет подпись до apply/play (CI #29638045838).
 Nested per-surface playlist — Manifest v2.
 Манифест доставляется только в тестах (нет реального плеера).</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. K2 resolved: signing verification done. Real KSO player: deferred.</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>Production manifest signing (отдельная задача).</t>
         </is>
@@ -3737,15 +3857,30 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Единая точка получения manifest для всех устройств. Кэширование (ETag), чтобы не грузить сеть повторными запросами.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>GET /api/v1/device/manifest/latest.
 Аутентификация: device JWT (sub=device_id, auth_provider=device).
@@ -3753,7 +3888,7 @@
 ETag/If-None-Match для кэширования.</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Только HTTP (не HTTPS/mTLS).
 Верификация подписи manifest: K2 resolved — runtime simulator проверяет подпись до apply (CI #29638045838).
@@ -3761,12 +3896,12 @@
 Нет реального KSO плеера, принимающего manifest.</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. mTLS — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>K2 resolved: manifest signing verification. mTLS — deferred.
 Next: RM1/R1/T1 process hygiene -&gt; release v0.8.</t>
@@ -3786,33 +3921,48 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Принимает подтверждения показов от устройств: что, когда и сколько раз показали. Это основа для отчётности перед рекламодателем.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>POST /api/v1/pop/batch — приём PoP-событий от устройств.
 11-шаговая валидация: schema, device, dedup, duration, playback, clock drift, cross-entity.
 Карантин 72h. Billing-grade accepted события.</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>PoP эмитится только симулятором (не реальным KSO плеером).
 Нет экспорта отчётов о показах.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Проверка с реальным плеером — BLOCKER BEFORE PILOT (B).</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>Реальный KSO плеер — вне backend-пилота.</t>
         </is>
@@ -3831,31 +3981,46 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Чтобы рекламодатель и администратор видели: сколько показов было, по каким поверхностям, в какой день. Это «доказательство» для рекламодателя.</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Backend: GET pop/{summary,by-day,by-surface}. Admin-web: вкладка PoP-отчёты. Advertiser-web: секция Отчётность в детали кампании.</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>Нет дашборда сети (ТЗ §15.1).
 Нет ClickHouse / materialized views.</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): дашборд кампании с план/факт и причинами отклонений (A5). ClickHouse — CAN DEFER.</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>S-090: дашборд кампании с анализом отклонений.</t>
         </is>
@@ -3873,27 +4038,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3912,15 +4077,30 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>⚪ Не начато (после ADR-018)</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Кассы самообслуживания — первый физический канал показа рекламы. Основной носитель для розничной рекламы.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>✅ Minimum inventory contract выполнен — можно начинать архитектурную подготовку плеера.
 ✅ Device-gateway: GET /manifest/latest работает.
@@ -3928,19 +4108,19 @@
 Почему сейчас можно: минимальный inventory-контракт (availability + reservation + campaign integration + conflicts + UI) предотвращает конфликтующие размещения. Без него плеер получил бы слоты без гарантии эксклюзивности.</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>❌ Минимальный inventory контракт выполнен — блокер снят.
 Ограничение: rule management UI не готов (правила создаются через DB), но backend-движок работает.
 ❌ Реального KSO плеера нет. Нет интеграции с железом.</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): нельзя начинать плеер пока A1–A6 не закрыты. S-086–S-091 сначала.</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>Фаза 1 (PLAN-001): один КСО. Onboarding → play → PoP. После ADR-018.</t>
         </is>
@@ -3959,32 +4139,47 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Второй по важности канал после КСО — ТВ-приставки в магазинах. Расширяет охват аудитории.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Архитектура заложена: capability profiles в БД, manifest поддерживает несколько device_types.</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Нет Android плеера.
 Нет WebView kiosk режима.
 Нет ТВ-приставок.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER: второй канал после KSO pilot.</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>Второй канал после KSO pilot.</t>
         </is>
@@ -4003,30 +4198,45 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Прайс-чекеры — дополнительные точки контакта с покупателем. Показ рекламы в режиме ожидания.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ (§6.8): показ рекламы только в idle/screen saver, без блокировки проверки цены.</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Нет реализации.</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER.</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>После KSO + Android TV.</t>
         </is>
@@ -4045,31 +4255,46 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Электронные ценники — потенциально тысячи мини-экранов в магазине. Требуют интеграции с оборудованием вендоров.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ (§6.8): интеграция через шлюзы и vendor API.</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Нет адаптеров к ESL-шлюзам.
 Нет поддержки протоколов вендоров.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER.</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>Отдельный проект интеграции.</t>
         </is>
@@ -4088,30 +4313,45 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>LED-панели на полках — дополнительный рекламный инвентарь. Схож с КСО по архитектуре.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ.</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Нет реализации.</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER.</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>Низкий приоритет.</t>
         </is>
@@ -4129,27 +4369,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4168,15 +4408,30 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Гарантирует, что два рекламодателя не получат один и тот же слот на одном экране в одно время. Управляет ёмкостью рекламных поверхностей.</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>✅ Проверка доступности слотов.
 ✅ Бронирование (reserve/commit/release/expire).
@@ -4186,7 +4441,7 @@
 ✅ UI календарь инвентаря: 4 вкладки (каталог, доступность, конфликты, правила).</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>❌ Нет визуальной сетки/календаря инвентаря.
 ❌ Нет прогноза доступности.
@@ -4194,12 +4449,12 @@
 ❌ UI-TRUTH: blocked — inventory.simulate, inventory.rule_create. UI-smoke отсутствует.</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): нет sold-out + альтернатив (A2), нет настройки правил в UI (A3). Прогноз — CAN DEFER.</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>A3 ✅ S-088 rules admin UI. A4–A6 remain.</t>
         </is>
@@ -4218,31 +4473,46 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Позволяет планировать рекламные кампании на будущие периоды, оценивать доступность слотов и загрузку поверхностей.</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Нет данных для прогноза — нужен работающий PoP pipeline + статистика за период.
 Нет ML/статистической модели.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER: статическая ёмкость достаточна для пилота.</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>После production PoP pipeline.</t>
         </is>
@@ -4260,27 +4530,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4299,15 +4569,30 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Возможность мгновенно остановить показ всей рекламы при чрезвычайной ситуации. Кнопка «стоп» для всей сети.</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: POST /emergency/activate|deactivate, GET /emergency/status.
 K1 resolved: emergency состояние попадает в device manifest (emergency.active, activated_at, reason). CI #29636889061.
@@ -4316,7 +4601,7 @@
 ✅ Outbox: emergency.changed события.</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>✅ Manifest-level emergency: K1 resolved (manifest содержит реальное emergency состояние: active, activated_at, reason). CI #29636889061.
 ❌ Player-side enforcement на реальном KSO — deferred (требуется KSO runtime).
@@ -4324,12 +4609,12 @@
 Почему: backend готов. Применение на устройствах ждёт player/KSO (v0.9).</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): emergency не применяется на устройствах (A6). MFA — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>K1 resolved: emergency override -&gt; manifest. Player-side KSO enforcement: phase 1.</t>
         </is>
@@ -4348,22 +4633,37 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>✅ Готово: PostgreSQL (S-031), MinIO (S-049), NATS (S-050)</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✅ Готово: PostgreSQL (S-031), MinIO (S-049), NATS </t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Защита от потери данных: база, медиафайлы, конфигурация. Возможность восстановления после сбоя.</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>✅ PostgreSQL: pg_dump backup + restore, drill test (5/5), runbook.
 ✅ MinIO: полный backup + manifest + SHA-256, restore с check/dry-run/confirm, runbook.
 ✅ NATS: outbox как source of truth, recovery через provisioning + relay replay (dedup-safe), runbook.</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>❌ Нет автоматического расписания бэкапов.
 ❌ Нет offsite-репликации.
@@ -4371,12 +4671,12 @@
 ❌ Нет нагрузочных тестов (ТЗ: 40 000 устройств).</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Авто-расписание — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>MinIO mirror + NATS policy — v0.6 (S-049/S-050).</t>
         </is>
@@ -4395,15 +4695,30 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Чтобы видеть состояние платформы в реальном времени: жива ли, сколько запросов, есть ли ошибки. Prometheus + Grafana.</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>✅ Prometheus метрики на control-api + device-gateway.
 ✅ Grafana дашборд «RMP Overview»: 4 секции, 10 панелей.
@@ -4412,19 +4727,19 @@
 ✅ Graceful shutdown (SIGTERM).</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>❌ Нет мониторинга инфраструктуры (CPU, RAM, диск).
 ❌ Grafana admin password не hardened для production.
 Почему: baseline observability готов. Инфраструктурный мониторинг — после production deploy.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Инфраструктурный мониторинг — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>v0.6: Prometheus metrics endpoint + Grafana dashboard.</t>
         </is>
@@ -4438,11 +4753,11 @@
       </c>
       <c r="B28" s="5" t="n"/>
       <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="n"/>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="10" t="inlineStr"/>
@@ -4456,27 +4771,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4495,30 +4810,45 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>🟡 Core pilot готов (PLAN-001: medium priority)</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Полноценный личный кабинет рекламодателя с самостоятельным управлением кампаниями, без участия оператора.</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>PLAN-001: self-service нужен, но не первым. Фаза 5.</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>После managed/core flow (фазы 1-4). Production UX, browser E2E.</t>
         </is>
@@ -4537,30 +4867,45 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>🚫 Отложено по решению бизнеса</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Измерение влияния рекламы на продажи: какие показы привели к покупкам. Ключевая метрика для рекламодателя.</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>PLAN-001: PoP достаточно. Attribution — осознанное бизнес-решение, не пробел.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>PLAN-001: решение владельца продукта.</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>Не начинать. Отложено по решению бизнеса.</t>
         </is>
@@ -4579,30 +4924,45 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Запрет показа рекламы конкурентов на одном экране. Защита интересов рекламодателей.</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>No competitive separation model.</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>After tenant model ADR.</t>
         </is>
@@ -4621,30 +4981,45 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Таргетинг рекламы на конкретные магазины или профили магазинов. Повышает релевантность показов.</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>No store profiles. No audience targeting.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>After tenant model ADR + inventory.</t>
         </is>
@@ -4663,30 +5038,45 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Финансовые документы: счета, акты, сверки. Интеграция с 1С / ERP для биллинга рекламодателей.</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>No 1C/ERP API. No invoicing.</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>After tenant model ADR.</t>
         </is>
@@ -4705,30 +5095,45 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Автоматизированная продажа рекламного инвентаря через внешние DSP/SSP платформы (OpenRTB).</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. OpenRTB stub.</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>No DSP/SSP integration.</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>
@@ -4747,30 +5152,45 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Креативы, которые меняются в реальном времени: цена, погода, остатки товара. Повышает вовлечённость.</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. HTML5 canvas/video templating.</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>No creative templating.</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="J36" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="K36" s="3" t="inlineStr">
         <is>
           <t>After KSO player stable.</t>
         </is>
@@ -4789,30 +5209,45 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Мобильное приложение для полевых операторов: проверка экранов, замена контента на месте.</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Mobile app.</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>No mobile client.</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>After KSO player stable.</t>
         </is>
@@ -4831,30 +5266,45 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Независимый аудит показов по стандартам DOOH (Digital Out-of-Home). Доверие крупных рекламодателей.</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Design stub only.</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>No external impression audit.</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="K38" s="3" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>
@@ -4885,25 +5335,40 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>S-095</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>Рекламодатели и бизнес видят гарантии качества услуги</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Инвентарь/кампании без привязки к SLA</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>SLA не утверждены с бизнесом</t>
         </is>
@@ -4922,25 +5387,40 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>S-096</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>Автоматический расчёт компенсаций при недовыполнении плана</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Ручной пересчёт недопоказа без классификации причин</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>Нет автоматического предложения докрутки</t>
         </is>
@@ -4959,25 +5439,40 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>S-097</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>ИТ-поддержка видит все устройства, их статус и ошибки</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Нет единой картины здоровья сети носителей</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>Данные heartbeat есть, но нет операционного интерфейса</t>
         </is>
@@ -4996,25 +5491,40 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>S-098</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>Безопасное обновление плееров/manifest без массовых сбоев</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Любое изменение затрагивает всю сеть сразу</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Нет механизма поэтапного выкатывания</t>
         </is>
@@ -5033,25 +5543,40 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
           <t>🚫 Отложено по решению бизнеса</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>Attribution v2.6</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>Оценка охвата через чеки для Sales Lift</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>PLAN-001: PoP достаточно. Интеграция с чеками отложена.</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>PLAN-001: решение владельца продукта.</t>
         </is>
@@ -5070,25 +5595,40 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>S-099</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>Включение функций на пилотные магазины без риска для сети</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>Все изменения применяются глобально</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>Нет инфраструктуры feature flags</t>
         </is>
@@ -5107,25 +5647,40 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>S-100</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>Соответствие требованиям хранения данных и юр. нормам</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>Данные хранятся без явных политик TTL</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>Нет утверждённых сроков хранения с юристами</t>
         </is>
@@ -5144,25 +5699,40 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>S-101</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>Подтверждение способности системы работать под расчётной нагрузкой</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>Тесты только на малых объёмах данных</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>Нет утверждённых профилей нагрузки</t>
         </is>
@@ -5181,30 +5751,45 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
+          <t>🧭</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>🧭 Требует решения (P0)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>S-102</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>Корректное расписание во всех часовых поясах РФ с учётом праздников</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>Только UTC/Moscow, без календаря исключений</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>PLAN-001: решение владельца продукта — время по местному.</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>ADR: store-local time. P0 после ADR-018.</t>
         </is>
@@ -5223,25 +5808,40 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>🧭</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
           <t>🧭 Требует решения</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>ADR требуется</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>Единый слой адаптеров для KSO/Android/ESL/LED</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>КСО-центричная архитектура</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>Нет ADR, нет абстракции адаптеров</t>
         </is>
@@ -5260,25 +5860,40 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>S-092</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>Передача критичных событий в SIEM для ИБ</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Логи只在 локальных файлах</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>Требуется согласование с ИБ-отделом</t>
         </is>

</xml_diff>

<commit_message>
docs: ROADMAP-DONE-GATE-001-FU — remove stale blocked claims, cross-reference superseded
R4 (RBAC): 'user.assign_roles blocked' → '✅ G2 green smoke / ❌ user.create_advertiser'
R7 (Campaigns): 'campaign.create blocked' → '✅ G1 green smoke / ❌ campaign.edit/submit/activate'
PROJECT_STATE: 3 stale refs strikethrough + RESOLVED (findings 7→5, reachable 5→7)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3445,8 +3445,9 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Нет UI для управления ролями и назначения прав (только API).
-❌ UI-TRUTH: blocked — user.assign_roles (G2), user.create_advertiser. UI-smoke отсутствует.</t>
+          <t>Нет UI для создания рекламодателей (user.create_advertiser) и сброса паролей.
+✅ user.assign_roles (G2) — зелёный UI-smoke.
+❌ user.create_advertiser, user.reset_password — UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -3609,7 +3610,8 @@
 ❌ Нет drag-and-drop.
 ❌ UX/accessibility не завершены.
 ❌ Нет браузерных E2E-тестов.
-❌ UI-TRUTH: blocked — campaign.create (G1), campaign.edit, campaign.submit, campaign.activate.</t>
+✅ campaign.create (G1) — зелёный UI-smoke.
+❌ campaign.edit, campaign.submit, campaign.activate — UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: G3-FIX — advertiser.create_org reachable (fix retailer_id default, smoke green)
- Fix retailer_id default: 00000000-4000-a000 → 00000000-0000-4000-a000
- Registry: advertiser.create_org → reachable
- Roadmap: add 'Управление рекламодателями' row
- Smoke: test_uismoke__advertiser__create_org green
- Guard: 0 findings, tamper 3/3
- PROJECT_STATE: G3-FIX section, Next: G4-FIX
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3228,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3524,87 +3524,144 @@
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>v0.1–v0.4</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Управление рекламодателями</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>✅ (create_org) / ⚪️ (view/apply/review)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>✅ advertiser.create_org / ⚪️ остальные</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>🟠 Частично (create_org reachable, остальное без smoke)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Создание и управление организациями рекламодателей (managed, не self-service). Системный администратор создаёт организацию, назначает роли.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>✅ Готово/Юзабельно частично: create_org работает, остальные journeys без UI-smoke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="10" t="inlineStr"/>
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Управление рекламными кампаниями</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>v0.1–v0.4</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Создание и редактирование кампаний</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>✅ (create) / ⚪️ (edit)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>✅ campaign.create / ⚪️ campaign.edit</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>🟠 Частично (edit не reachable)</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Основной рабочий инструмент: создание, настройка и управление рекламными кампаниями (бюджет, сроки, поверхности).</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: полный CRUD кампаний (7 endpoints), пролёты, размещения, креативы.
 ✅ Admin-web: список с фильтром, мастер создания, 5 вкладок (пролёты, размещения, креативы+upload, согласование, PoP-отчёты).
 ✅ Advertiser-web: создание/редактирование черновиков.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>❌ Нет календаря планирования.
 ❌ Нет drag-and-drop.
@@ -3614,275 +3671,275 @@
 ❌ campaign.edit, campaign.submit, campaign.activate — UI-smoke отсутствует.</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>BLOCKER A1 ✅ done: прогноз доступности при создании кампании (S-086). A2–A6 остаются. Календарь — CAN DEFER.</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>A3 ✅ S-088 rules admin UI. A4–A6 remain.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>v0.1–v0.4</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Согласование кампаний (Approval)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>🟠</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Чтобы ни одна кампания не пошла в показ без проверки администратором: правильные ли креативы, не нарушен ли бюджет.</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: request-approval → approve/reject с audit trail.
 ✅ Admin-web: очередь согласования, approve/reject с причиной.
 ✅ Advertiser-web: отправка на согласование, видимость статуса/причины отклонения.</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>❌ Рекламодатель не может сам утверждать — только отправляет.
 Почему: это осознанное ограничение безопасности.
 ❌ UI-TRUTH: blocked — campaign.approve, campaign.reject. UI-smoke отсутствует.</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Цепочка работает. Advertiser не утверждает — by design.</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>После campaign UI (S-009c).</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>v0.1–v0.4</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Загрузка креативов (медиафайлы)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>🟠</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Чтобы рекламодатели могли загружать изображения и видео для показа на экранах. Хранение — в защищённом MinIO (S3).</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Backend: presigned URL (MinIO/S3) + SHA-256.
 Admin-web UI: загрузка с прогресс-баром.
 Advertiser-web: библиотека + загрузка + привязка к кампании (S-023c, S-023g).</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Malware scan, transcoding, CDN — отложены.
 ❌ UI-TRUTH: blocked — creative.upload, creative.moderate_approve, creative.moderate_reject.</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>SHOULD FIX (C): загрузка работает. Антивирус — BLOCKER BEFORE PILOT (B). Превью/история версий — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>Malware scan, transcoding, manual moderation — отложены.
 Работает для пилота.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr">
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Доставка контента на устройства</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>v0.1–v0.4</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Формирование плейлистов (manifest)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Автоматически формирует плейлист для каждого устройства: какие креативы и в каком порядке показывать. Без этого плеер не знает, что играть.</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Manifest JSON с полями: device_id, store_id, playlist[], media_files[], valid_from/to, offline_ttl_hours.
 ETag/304 — кэширование на устройстве.
 Автоматическая генерация при изменении кампании.</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Верификация подписи манифеста: K2 resolved — runtime simulator проверяет подпись до apply/play (CI #29638045838).
 Nested per-surface playlist — Manifest v2.
 Манифест доставляется только в тестах (нет реального плеера).</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. K2 resolved: signing verification done. Real KSO player: deferred.</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>Production manifest signing (отдельная задача).</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>v0.1–v0.4</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Получение manifest устройством</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Единая точка получения manifest для всех устройств. Кэширование (ETag), чтобы не грузить сеть повторными запросами.</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>GET /api/v1/device/manifest/latest.
 Аутентификация: device JWT (sub=device_id, auth_provider=device).
@@ -3890,7 +3947,7 @@
 ETag/If-None-Match для кэширования.</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Только HTTP (не HTTPS/mTLS).
 Верификация подписи manifest: K2 resolved — runtime simulator проверяет подпись до apply (CI #29638045838).
@@ -3898,211 +3955,211 @@
 Нет реального KSO плеера, принимающего manifest.</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. mTLS — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>K2 resolved: manifest signing verification. mTLS — deferred.
 Next: RM1/R1/T1 process hygiene -&gt; release v0.8.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>v0.1–v0.4</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Proof-of-Play (подтверждение показов)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Принимает подтверждения показов от устройств: что, когда и сколько раз показали. Это основа для отчётности перед рекламодателем.</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>POST /api/v1/pop/batch — приём PoP-событий от устройств.
 11-шаговая валидация: schema, device, dedup, duration, playback, clock drift, cross-entity.
 Карантин 72h. Billing-grade accepted события.</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>PoP эмитится только симулятором (не реальным KSO плеером).
 Нет экспорта отчётов о показах.</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Проверка с реальным плеером — BLOCKER BEFORE PILOT (B).</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>Реальный KSO плеер — вне backend-пилота.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>v0.1–v0.4</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Отчёты по показам</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Чтобы рекламодатель и администратор видели: сколько показов было, по каким поверхностям, в какой день. Это «доказательство» для рекламодателя.</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Backend: GET pop/{summary,by-day,by-surface}. Admin-web: вкладка PoP-отчёты. Advertiser-web: секция Отчётность в детали кампании.</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Нет дашборда сети (ТЗ §15.1).
 Нет ClickHouse / materialized views.</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): дашборд кампании с план/факт и причинами отклонений (A5). ClickHouse — CAN DEFER.</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>S-090: дашборд кампании с анализом отклонений.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr">
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="10" t="inlineStr"/>
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Каналы и устройства</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>v0.9 (фаза 1)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>КСО (кассы самообслуживания)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>⚪ Не начато (после ADR-018)</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Кассы самообслуживания — первый физический канал показа рекламы. Основной носитель для розничной рекламы.</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>✅ Minimum inventory contract выполнен — можно начинать архитектурную подготовку плеера.
 ✅ Device-gateway: GET /manifest/latest работает.
@@ -4110,137 +4167,80 @@
 Почему сейчас можно: минимальный inventory-контракт (availability + reservation + campaign integration + conflicts + UI) предотвращает конфликтующие размещения. Без него плеер получил бы слоты без гарантии эксклюзивности.</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>❌ Минимальный inventory контракт выполнен — блокер снят.
 Ограничение: rule management UI не готов (правила создаются через DB), но backend-движок работает.
 ❌ Реального KSO плеера нет. Нет интеграции с железом.</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): нельзя начинать плеер пока A1–A6 не закрыты. S-086–S-091 сначала.</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>Фаза 1 (PLAN-001): один КСО. Onboarding → play → PoP. После ADR-018.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>v0.9+</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Android / Android TV</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>🚫</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Второй по важности канал после КСО — ТВ-приставки в магазинах. Расширяет охват аудитории.</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Архитектура заложена: capability profiles в БД, manifest поддерживает несколько device_types.</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Нет Android плеера.
 Нет WebView kiosk режима.
 Нет ТВ-приставок.</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER: второй канал после KSO pilot.</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Второй канал после KSO pilot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>v0.9+</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Price Checker (Android)</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>🚫</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>🚫 Отложено</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Прайс-чекеры — дополнительные точки контакта с покупателем. Показ рекламы в режиме ожидания.</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Архитектура в ТЗ (§6.8): показ рекламы только в idle/screen saver, без блокировки проверки цены.</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Нет реализации.</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>CAN DEFER.</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>После KSO + Android TV.</t>
         </is>
       </c>
     </row>
@@ -4252,188 +4252,245 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>Price Checker (Android)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>🚫 Отложено</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Прайс-чекеры — дополнительные точки контакта с покупателем. Показ рекламы в режиме ожидания.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Архитектура в ТЗ (§6.8): показ рекламы только в idle/screen saver, без блокировки проверки цены.</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Нет реализации.</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>CAN DEFER.</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>После KSO + Android TV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>ESL / Электронные ценники</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>🚫</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Электронные ценники — потенциально тысячи мини-экранов в магазине. Требуют интеграции с оборудованием вендоров.</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ (§6.8): интеграция через шлюзы и vendor API.</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Нет адаптеров к ESL-шлюзам.
 Нет поддержки протоколов вендоров.</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER.</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>Отдельный проект интеграции.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>v0.9+</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>LED Shelf Banners</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>🚫</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>LED-панели на полках — дополнительный рекламный инвентарь. Схож с КСО по архитектуре.</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Архитектура в ТЗ.</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Нет реализации.</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER.</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>Низкий приоритет.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="10" t="inlineStr"/>
-      <c r="B21" s="10" t="inlineStr">
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="10" t="inlineStr"/>
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>Инвентарь и прогноз</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K21" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>v0.7</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>✅ Готово: availability + reservation + conflicts + rules + UI calendar (S-081)</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>🟠</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>🟠 Бэкенд готов, UI-smoke нет</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Гарантирует, что два рекламодателя не получат один и тот же слот на одном экране в одно время. Управляет ёмкостью рекламных поверхностей.</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>✅ Проверка доступности слотов.
 ✅ Бронирование (reserve/commit/release/expire).
@@ -4443,7 +4500,7 @@
 ✅ UI календарь инвентаря: 4 вкладки (каталог, доступность, конфликты, правила).</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>❌ Нет визуальной сетки/календаря инвентаря.
 ❌ Нет прогноза доступности.
@@ -4451,150 +4508,150 @@
 ❌ UI-TRUTH: blocked — inventory.simulate, inventory.rule_create. UI-smoke отсутствует.</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): нет sold-out + альтернатив (A2), нет настройки правил в UI (A3). Прогноз — CAN DEFER.</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>A3 ✅ S-088 rules admin UI. A4–A6 remain.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>v0.7</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Прогноз показов</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Позволяет планировать рекламные кампании на будущие периоды, оценивать доступность слотов и загрузку поверхностей.</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>Нет данных для прогноза — нужен работающий PoP pipeline + статистика за период.
 Нет ML/статистической модели.</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER: статическая ёмкость достаточна для пилота.</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>После production PoP pipeline.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="10" t="inlineStr"/>
-      <c r="B24" s="10" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="10" t="inlineStr"/>
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Эксплуатация и безопасность</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K24" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>v0.6</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Emergency-управление</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Возможность мгновенно остановить показ всей рекламы при чрезвычайной ситуации. Кнопка «стоп» для всей сети.</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>✅ Backend: POST /emergency/activate|deactivate, GET /emergency/status.
 K1 resolved: emergency состояние попадает в device manifest (emergency.active, activated_at, reason). CI #29636889061.
@@ -4603,7 +4660,7 @@
 ✅ Outbox: emergency.changed события.</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>✅ Manifest-level emergency: K1 resolved (manifest содержит реальное emergency состояние: active, activated_at, reason). CI #29636889061.
 ❌ Player-side enforcement на реальном KSO — deferred (требуется KSO runtime).
@@ -4611,61 +4668,61 @@
 Почему: backend готов. Применение на устройствах ждёт player/KSO (v0.9).</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>BLOCKER BEFORE PLAYER (A): emergency не применяется на устройствах (A6). MFA — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>K1 resolved: emergency override -&gt; manifest. Player-side KSO enforcement: phase 1.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>v0.6</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Резервное копирование и DR</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t xml:space="preserve">✅ Готово: PostgreSQL (S-031), MinIO (S-049), NATS </t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Защита от потери данных: база, медиафайлы, конфигурация. Возможность восстановления после сбоя.</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>✅ PostgreSQL: pg_dump backup + restore, drill test (5/5), runbook.
 ✅ MinIO: полный backup + manifest + SHA-256, restore с check/dry-run/confirm, runbook.
 ✅ NATS: outbox как source of truth, recovery через provisioning + relay replay (dedup-safe), runbook.</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>❌ Нет автоматического расписания бэкапов.
 ❌ Нет offsite-репликации.
@@ -4673,54 +4730,54 @@
 ❌ Нет нагрузочных тестов (ТЗ: 40 000 устройств).</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Авто-расписание — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>MinIO mirror + NATS policy — v0.6 (S-049/S-050).</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>v0.6</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Мониторинг и observability</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>✅ Готово</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Чтобы видеть состояние платформы в реальном времени: жива ли, сколько запросов, есть ли ошибки. Prometheus + Grafana.</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>✅ Prometheus метрики на control-api + device-gateway.
 ✅ Grafana дашборд «RMP Overview»: 4 секции, 10 панелей.
@@ -4729,147 +4786,90 @@
 ✅ Graceful shutdown (SIGTERM).</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>❌ Нет мониторинга инфраструктуры (CPU, RAM, диск).
 ❌ Grafana admin password не hardened для production.
 Почему: baseline observability готов. Инфраструктурный мониторинг — после production deploy.</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>✅ Готово. Инфраструктурный мониторинг — SHOULD FIX (C).</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>v0.6: Prometheus metrics endpoint + Grafana dashboard.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="60" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>v0.5–v0.6</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="n"/>
-    </row>
-    <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="10" t="inlineStr"/>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="n"/>
+      <c r="J29" s="3" t="inlineStr"/>
+      <c r="K29" s="3" t="n"/>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="10" t="inlineStr"/>
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>v2.6 Next Branch</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K29" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="60" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>v2.0 (фаза 5)</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Self-service advertiser cabinet</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>🟡 Core pilot готов (PLAN-001: medium priority)</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Полноценный личный кабинет рекламодателя с самостоятельным управлением кампаниями, без участия оператора.</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>PLAN-001: self-service нужен, но не первым. Фаза 5.</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>После managed/core flow (фазы 1-4). Production UX, browser E2E.</t>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>v2.6</t>
+          <t>v2.0 (фаза 5)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Sales Lift / Attribution proof</t>
+          <t>Self-service advertiser cabinet</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4884,32 +4884,32 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>🚫 Отложено по решению бизнеса</t>
+          <t>🟡 Core pilot готов (PLAN-001: medium priority)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Измерение влияния рекламы на продажи: какие показы привели к покупкам. Ключевая метрика для рекламодателя.</t>
+          <t>Полноценный личный кабинет рекламодателя с самостоятельным управлением кампаниями, без участия оператора.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>PLAN-001: PoP достаточно. Attribution — осознанное бизнес-решение, не пробел.</t>
+          <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>PLAN-001: решение владельца продукта.</t>
+          <t>PLAN-001: self-service нужен, но не первым. Фаза 5.</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Не начинать. Отложено по решению бизнеса.</t>
+          <t>После managed/core flow (фазы 1-4). Production UX, browser E2E.</t>
         </is>
       </c>
     </row>
@@ -4921,19 +4921,19 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Competitor blocking</t>
+          <t>Sales Lift / Attribution proof</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>—</t>
@@ -4941,12 +4941,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🚫 Отложено по решению бизнеса</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Запрет показа рекламы конкурентов на одном экране. Защита интересов рекламодателей.</t>
+          <t>Измерение влияния рекламы на продажи: какие показы привели к покупкам. Ключевая метрика для рекламодателя.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -4956,17 +4956,17 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>No competitive separation model.</t>
+          <t>PLAN-001: PoP достаточно. Attribution — осознанное бизнес-решение, не пробел.</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER (D): v2.6.</t>
+          <t>PLAN-001: решение владельца продукта.</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>Не начинать. Отложено по решению бизнеса.</t>
         </is>
       </c>
     </row>
@@ -4978,7 +4978,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Store/audience targeting</t>
+          <t>Competitor blocking</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Таргетинг рекламы на конкретные магазины или профили магазинов. Повышает релевантность показов.</t>
+          <t>Запрет показа рекламы конкурентов на одном экране. Защита интересов рекламодателей.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>No store profiles. No audience targeting.</t>
+          <t>No competitive separation model.</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>After tenant model ADR + inventory.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Financial docs / reconciliation / integration</t>
+          <t>Store/audience targeting</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Финансовые документы: счета, акты, сверки. Интеграция с 1С / ERP для биллинга рекламодателей.</t>
+          <t>Таргетинг рекламы на конкретные магазины или профили магазинов. Повышает релевантность показов.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>No 1C/ERP API. No invoicing.</t>
+          <t>No store profiles. No audience targeting.</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>After tenant model ADR + inventory.</t>
         </is>
       </c>
     </row>
@@ -5092,12 +5092,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Programmatic inventory sales</t>
+          <t>Financial docs / reconciliation / integration</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>⚪️</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -5112,22 +5112,22 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>🚫 Отложено</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Автоматизированная продажа рекламного инвентаря через внешние DSP/SSP платформы (OpenRTB).</t>
+          <t>Финансовые документы: счета, акты, сверки. Интеграция с 1С / ERP для биллинга рекламодателей.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. OpenRTB stub.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>No DSP/SSP integration.</t>
+          <t>No 1C/ERP API. No invoicing.</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>After production pilot.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5149,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Dynamic creatives</t>
+          <t>Programmatic inventory sales</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -5174,17 +5174,17 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Креативы, которые меняются в реальном времени: цена, погода, остатки товара. Повышает вовлечённость.</t>
+          <t>Автоматизированная продажа рекламного инвентаря через внешние DSP/SSP платформы (OpenRTB).</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. HTML5 canvas/video templating.</t>
+          <t>TZ v2.6. OpenRTB stub.</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>No creative templating.</t>
+          <t>No DSP/SSP integration.</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -5194,7 +5194,7 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>After KSO player stable.</t>
+          <t>After production pilot.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Mobile field ops</t>
+          <t>Dynamic creatives</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -5231,17 +5231,17 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Мобильное приложение для полевых операторов: проверка экранов, замена контента на месте.</t>
+          <t>Креативы, которые меняются в реальном времени: цена, погода, остатки товара. Повышает вовлечённость.</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. Mobile app.</t>
+          <t>TZ v2.6. HTML5 canvas/video templating.</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>No mobile client.</t>
+          <t>No creative templating.</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -5263,116 +5263,121 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
+          <t>Mobile field ops</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>🚫 Отложено</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Мобильное приложение для полевых операторов: проверка экранов, замена контента на месте.</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Mobile app.</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>No mobile client.</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>CAN DEFER (D): v2.6.</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>After KSO player stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
           <t>Independent DOOH measurement</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>🚫</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>Независимый аудит показов по стандартам DOOH (Digital Out-of-Home). Доверие крупных рекламодателей.</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Design stub only.</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>No external impression audit.</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="K39" s="3" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" t="inlineStr">
+    <row r="40">
+      <c r="B40" t="inlineStr">
         <is>
           <t>ТЗ-покрытие (D3 audit)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>v0.9+</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>SLA/NFT: 99.5/99.9% доступность, RTO 4ч, RPO 15м</t>
-        </is>
-      </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>⚪️</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>⚪ Не начато</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>S-095</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Рекламодатели и бизнес видят гарантии качества услуги</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Инвентарь/кампании без привязки к SLA</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>SLA не утверждены с бизнесом</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5384,7 +5389,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Мониторинг недопоказов и компенсации</t>
+          <t>SLA/NFT: 99.5/99.9% доступность, RTO 4ч, RPO 15м</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -5409,22 +5414,22 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>S-096</t>
+          <t>S-095</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Автоматический расчёт компенсаций при недовыполнении плана</t>
+          <t>Рекламодатели и бизнес видят гарантии качества услуги</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Ручной пересчёт недопоказа без классификации причин</t>
+          <t>Инвентарь/кампании без привязки к SLA</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Нет автоматического предложения докрутки</t>
+          <t>SLA не утверждены с бизнесом</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5441,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Операционный центр здоровья устройств</t>
+          <t>Мониторинг недопоказов и компенсации</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5461,22 +5466,22 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>S-097</t>
+          <t>S-096</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>ИТ-поддержка видит все устройства, их статус и ошибки</t>
+          <t>Автоматический расчёт компенсаций при недовыполнении плана</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Нет единой картины здоровья сети носителей</t>
+          <t>Ручной пересчёт недопоказа без классификации причин</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Данные heartbeat есть, но нет операционного интерфейса</t>
+          <t>Нет автоматического предложения докрутки</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5493,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Staged rollout и rollback</t>
+          <t>Операционный центр здоровья устройств</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5513,39 +5518,39 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>S-098</t>
+          <t>S-097</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Безопасное обновление плееров/manifest без массовых сбоев</t>
+          <t>ИТ-поддержка видит все устройства, их статус и ошибки</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Любое изменение затрагивает всю сеть сразу</t>
+          <t>Нет единой картины здоровья сети носителей</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Нет механизма поэтапного выкатывания</t>
+          <t>Данные heartbeat есть, но нет операционного интерфейса</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>v2.6</t>
+          <t>v0.9+</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Интеграция с УКМ4 / чековые данные</t>
+          <t>Staged rollout и rollback</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>⚪️</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5560,51 +5565,51 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>🚫 Отложено по решению бизнеса</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Attribution v2.6</t>
+          <t>S-098</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Оценка охвата через чеки для Sales Lift</t>
+          <t>Безопасное обновление плееров/manifest без массовых сбоев</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>PLAN-001: PoP достаточно. Интеграция с чеками отложена.</t>
+          <t>Любое изменение затрагивает всю сеть сразу</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>PLAN-001: решение владельца продукта.</t>
+          <t>Нет механизма поэтапного выкатывания</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>v0.9+</t>
+          <t>v2.6</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Feature flags для безопасного развития</t>
+          <t>Интеграция с УКМ4 / чековые данные</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>—</t>
@@ -5612,27 +5617,27 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🚫 Отложено по решению бизнеса</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>S-099</t>
+          <t>Attribution v2.6</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Включение функций на пилотные магазины без риска для сети</t>
+          <t>Оценка охвата через чеки для Sales Lift</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Все изменения применяются глобально</t>
+          <t>PLAN-001: PoP достаточно. Интеграция с чеками отложена.</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Нет инфраструктуры feature flags</t>
+          <t>PLAN-001: решение владельца продукта.</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5649,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Data Governance: retention, партиционирование</t>
+          <t>Feature flags для безопасного развития</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5669,22 +5674,22 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>S-100</t>
+          <t>S-099</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Соответствие требованиям хранения данных и юр. нормам</t>
+          <t>Включение функций на пилотные магазины без риска для сети</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Данные хранятся без явных политик TTL</t>
+          <t>Все изменения применяются глобально</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Нет утверждённых сроков хранения с юристами</t>
+          <t>Нет инфраструктуры feature flags</t>
         </is>
       </c>
     </row>
@@ -5696,7 +5701,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Нагрузочное тестирование 40K устройств</t>
+          <t>Data Governance: retention, партиционирование</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5721,39 +5726,39 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>S-101</t>
+          <t>S-100</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Подтверждение способности системы работать под расчётной нагрузкой</t>
+          <t>Соответствие требованиям хранения данных и юр. нормам</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Тесты только на малых объёмах данных</t>
+          <t>Данные хранятся без явных политик TTL</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Нет утверждённых профилей нагрузки</t>
+          <t>Нет утверждённых сроков хранения с юристами</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>v0.8 (P0: PLAN-001)</t>
+          <t>v0.9+</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Часовые пояса и календарь показов</t>
+          <t>Нагрузочное тестирование 40K устройств</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>🧭</t>
+          <t>⚪️</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5768,44 +5773,39 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>🧭 Требует решения (P0)</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>S-102</t>
+          <t>S-101</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Корректное расписание во всех часовых поясах РФ с учётом праздников</t>
+          <t>Подтверждение способности системы работать под расчётной нагрузкой</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Только UTC/Moscow, без календаря исключений</t>
+          <t>Тесты только на малых объёмах данных</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>PLAN-001: решение владельца продукта — время по местному.</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>ADR: store-local time. P0 после ADR-018.</t>
+          <t>Нет утверждённых профилей нагрузки</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>v0.9+</t>
+          <t>v0.8 (P0: PLAN-001)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Channel Orchestrator / Adapter Layer</t>
+          <t>Часовые пояса и календарь показов</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5825,77 +5825,134 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>🧭 Требует решения</t>
+          <t>🧭 Требует решения (P0)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>ADR требуется</t>
+          <t>S-102</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Единый слой адаптеров для KSO/Android/ESL/LED</t>
+          <t>Корректное расписание во всех часовых поясах РФ с учётом праздников</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>КСО-центричная архитектура</t>
+          <t>Только UTC/Moscow, без календаря исключений</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Нет ADR, нет абстракции адаптеров</t>
+          <t>PLAN-001: решение владельца продукта — время по местному.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ADR: store-local time. P0 после ADR-018.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Channel Orchestrator / Adapter Layer</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>🧭</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>🧭 Требует решения</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>ADR требуется</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Единый слой адаптеров для KSO/Android/ESL/LED</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>КСО-центричная архитектура</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Нет ADR, нет абстракции адаптеров</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>v2.6</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>SIEM/Wazuh + ИБ-мониторинг</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>S-092</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>Передача критичных событий в SIEM для ИБ</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>Логи只在 локальных файлах</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>Требуется согласование с ИБ-отделом</t>
         </is>

</xml_diff>

<commit_message>
G4-FIX-FU: durable DB persistence + roadmap sync
DB persistence:
- ADSettings model (ad_settings table — singleton, id=1)
- Migration 027: create table + default row
- Repository: get_ad_settings(), save_ad_settings()
- GET/PUT endpoints read/write from DB (survives restart)
- Bind password remains env-only — never stored in DB

Tests:
- Backend 15/15 (durable_persistence, save/read, perm, validation, no-secret)
- Frontend 163/163

Roadmap:
- New row: «Настройки AD / LDAPS» (v0.6)
  Бэкенд ✅ / UI ✅ / journey ✅ / Итог 🟠 Частично
- adsettings.test without smoke — honest partial status
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3228,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4805,128 +4805,128 @@
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>v0.6</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Настройки AD / LDAPS</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>✅ (PUT save, durable DB)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>✅ (adsettings.configure)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>✅ (adsettings.configure — green smoke)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>🟠 Частично (adsettings.test без smoke)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Администрирование AD/LDAPS для входа сотрудников</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Сохранить настройки AD (PUT /auth/ad-settings), просмотр, проверка подключения</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>adsettings.test без зелёного UI-smoke | bind_password env-only (не редактируется через UI)</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>G4-FIX закрыл save/persist; adsettings.test требует отдельного smoke</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>adsettings.configure smoke test</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>v0.5–v0.6</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="n"/>
-    </row>
-    <row r="30" ht="60" customHeight="1">
-      <c r="A30" s="10" t="inlineStr"/>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="n"/>
+    </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="10" t="inlineStr"/>
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>v2.6 Next Branch</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>v2.0 (фаза 5)</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Self-service advertiser cabinet</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>🟡 Core pilot готов (PLAN-001: medium priority)</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Полноценный личный кабинет рекламодателя с самостоятельным управлением кампаниями, без участия оператора.</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>PLAN-001: self-service нужен, но не первым. Фаза 5.</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>После managed/core flow (фазы 1-4). Production UX, browser E2E.</t>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J31" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>v2.6</t>
+          <t>v2.0 (фаза 5)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Sales Lift / Attribution proof</t>
+          <t>Self-service advertiser cabinet</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4941,32 +4941,32 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>🚫 Отложено по решению бизнеса</t>
+          <t>🟡 Core pilot готов (PLAN-001: medium priority)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Измерение влияния рекламы на продажи: какие показы привели к покупкам. Ключевая метрика для рекламодателя.</t>
+          <t>Полноценный личный кабинет рекламодателя с самостоятельным управлением кампаниями, без участия оператора.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. Future v2.6.</t>
+          <t>S-023a-i: advertiser-web — login, campaign list/detail/create/edit, creative library/upload/attach, submit approval, PoP, profile/password, responsive layout. 66 vitest tests. CI #29166816518 green (33/33). Live LAN preview.</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>PLAN-001: PoP достаточно. Attribution — осознанное бизнес-решение, не пробел.</t>
+          <t>No advertiser approve/reject. No billing. No attribution. No production UX audit.</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>PLAN-001: решение владельца продукта.</t>
+          <t>PLAN-001: self-service нужен, но не первым. Фаза 5.</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Не начинать. Отложено по решению бизнеса.</t>
+          <t>После managed/core flow (фазы 1-4). Production UX, browser E2E.</t>
         </is>
       </c>
     </row>
@@ -4978,19 +4978,19 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Competitor blocking</t>
+          <t>Sales Lift / Attribution proof</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>—</t>
@@ -4998,12 +4998,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🚫 Отложено по решению бизнеса</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Запрет показа рекламы конкурентов на одном экране. Защита интересов рекламодателей.</t>
+          <t>Измерение влияния рекламы на продажи: какие показы привели к покупкам. Ключевая метрика для рекламодателя.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -5013,17 +5013,17 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>No competitive separation model.</t>
+          <t>PLAN-001: PoP достаточно. Attribution — осознанное бизнес-решение, не пробел.</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>CAN DEFER (D): v2.6.</t>
+          <t>PLAN-001: решение владельца продукта.</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>Не начинать. Отложено по решению бизнеса.</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Store/audience targeting</t>
+          <t>Competitor blocking</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Таргетинг рекламы на конкретные магазины или профили магазинов. Повышает релевантность показов.</t>
+          <t>Запрет показа рекламы конкурентов на одном экране. Защита интересов рекламодателей.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>No store profiles. No audience targeting.</t>
+          <t>No competitive separation model.</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>After tenant model ADR + inventory.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Financial docs / reconciliation / integration</t>
+          <t>Store/audience targeting</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Финансовые документы: счета, акты, сверки. Интеграция с 1С / ERP для биллинга рекламодателей.</t>
+          <t>Таргетинг рекламы на конкретные магазины или профили магазинов. Повышает релевантность показов.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>No 1C/ERP API. No invoicing.</t>
+          <t>No store profiles. No audience targeting.</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>After tenant model ADR.</t>
+          <t>After tenant model ADR + inventory.</t>
         </is>
       </c>
     </row>
@@ -5149,12 +5149,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Programmatic inventory sales</t>
+          <t>Financial docs / reconciliation / integration</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>⚪️</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5169,22 +5169,22 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>🚫 Отложено</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Автоматизированная продажа рекламного инвентаря через внешние DSP/SSP платформы (OpenRTB).</t>
+          <t>Финансовые документы: счета, акты, сверки. Интеграция с 1С / ERP для биллинга рекламодателей.</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. OpenRTB stub.</t>
+          <t>TZ v2.6. Future v2.6.</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>No DSP/SSP integration.</t>
+          <t>No 1C/ERP API. No invoicing.</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -5194,7 +5194,7 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>After production pilot.</t>
+          <t>After tenant model ADR.</t>
         </is>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Dynamic creatives</t>
+          <t>Programmatic inventory sales</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -5231,17 +5231,17 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Креативы, которые меняются в реальном времени: цена, погода, остатки товара. Повышает вовлечённость.</t>
+          <t>Автоматизированная продажа рекламного инвентаря через внешние DSP/SSP платформы (OpenRTB).</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. HTML5 canvas/video templating.</t>
+          <t>TZ v2.6. OpenRTB stub.</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>No creative templating.</t>
+          <t>No DSP/SSP integration.</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>After KSO player stable.</t>
+          <t>After production pilot.</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Mobile field ops</t>
+          <t>Dynamic creatives</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -5288,17 +5288,17 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Мобильное приложение для полевых операторов: проверка экранов, замена контента на месте.</t>
+          <t>Креативы, которые меняются в реальном времени: цена, погода, остатки товара. Повышает вовлечённость.</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>TZ v2.6. Mobile app.</t>
+          <t>TZ v2.6. HTML5 canvas/video templating.</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>No mobile client.</t>
+          <t>No creative templating.</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
@@ -5320,116 +5320,121 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
+          <t>Mobile field ops</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>🚫 Отложено</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Мобильное приложение для полевых операторов: проверка экранов, замена контента на месте.</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>TZ v2.6. Mobile app.</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>No mobile client.</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>CAN DEFER (D): v2.6.</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>After KSO player stable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>v2.6</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
           <t>Independent DOOH measurement</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>🚫</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
         <is>
           <t>🚫 Отложено</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>Независимый аудит показов по стандартам DOOH (Digital Out-of-Home). Доверие крупных рекламодателей.</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>TZ v2.6. Design stub only.</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>No external impression audit.</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr">
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>CAN DEFER (D): v2.6.</t>
         </is>
       </c>
-      <c r="K39" s="3" t="inlineStr">
+      <c r="K40" s="3" t="inlineStr">
         <is>
           <t>After production pilot.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" t="inlineStr">
+    <row r="41">
+      <c r="B41" t="inlineStr">
         <is>
           <t>ТЗ-покрытие (D3 audit)</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>v0.9+</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>SLA/NFT: 99.5/99.9% доступность, RTO 4ч, RPO 15м</t>
-        </is>
-      </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>⚪️</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>⚪ Не начато</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>S-095</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Рекламодатели и бизнес видят гарантии качества услуги</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Инвентарь/кампании без привязки к SLA</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>SLA не утверждены с бизнесом</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5446,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Мониторинг недопоказов и компенсации</t>
+          <t>SLA/NFT: 99.5/99.9% доступность, RTO 4ч, RPO 15м</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5466,22 +5471,22 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>S-096</t>
+          <t>S-095</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Автоматический расчёт компенсаций при недовыполнении плана</t>
+          <t>Рекламодатели и бизнес видят гарантии качества услуги</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Ручной пересчёт недопоказа без классификации причин</t>
+          <t>Инвентарь/кампании без привязки к SLA</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Нет автоматического предложения докрутки</t>
+          <t>SLA не утверждены с бизнесом</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5498,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Операционный центр здоровья устройств</t>
+          <t>Мониторинг недопоказов и компенсации</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5518,22 +5523,22 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>S-097</t>
+          <t>S-096</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>ИТ-поддержка видит все устройства, их статус и ошибки</t>
+          <t>Автоматический расчёт компенсаций при недовыполнении плана</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Нет единой картины здоровья сети носителей</t>
+          <t>Ручной пересчёт недопоказа без классификации причин</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Данные heartbeat есть, но нет операционного интерфейса</t>
+          <t>Нет автоматического предложения докрутки</t>
         </is>
       </c>
     </row>
@@ -5545,7 +5550,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Staged rollout и rollback</t>
+          <t>Операционный центр здоровья устройств</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5570,39 +5575,39 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>S-098</t>
+          <t>S-097</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Безопасное обновление плееров/manifest без массовых сбоев</t>
+          <t>ИТ-поддержка видит все устройства, их статус и ошибки</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Любое изменение затрагивает всю сеть сразу</t>
+          <t>Нет единой картины здоровья сети носителей</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Нет механизма поэтапного выкатывания</t>
+          <t>Данные heartbeat есть, но нет операционного интерфейса</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>v2.6</t>
+          <t>v0.9+</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Интеграция с УКМ4 / чековые данные</t>
+          <t>Staged rollout и rollback</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>🚫</t>
+          <t>⚪️</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5617,51 +5622,51 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>🚫 Отложено по решению бизнеса</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Attribution v2.6</t>
+          <t>S-098</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Оценка охвата через чеки для Sales Lift</t>
+          <t>Безопасное обновление плееров/manifest без массовых сбоев</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>PLAN-001: PoP достаточно. Интеграция с чеками отложена.</t>
+          <t>Любое изменение затрагивает всю сеть сразу</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>PLAN-001: решение владельца продукта.</t>
+          <t>Нет механизма поэтапного выкатывания</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>v0.9+</t>
+          <t>v2.6</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Feature flags для безопасного развития</t>
+          <t>Интеграция с УКМ4 / чековые данные</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
+          <t>🚫</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>⚪️</t>
-        </is>
-      </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>—</t>
@@ -5669,27 +5674,27 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🚫 Отложено по решению бизнеса</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>S-099</t>
+          <t>Attribution v2.6</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Включение функций на пилотные магазины без риска для сети</t>
+          <t>Оценка охвата через чеки для Sales Lift</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Все изменения применяются глобально</t>
+          <t>PLAN-001: PoP достаточно. Интеграция с чеками отложена.</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Нет инфраструктуры feature flags</t>
+          <t>PLAN-001: решение владельца продукта.</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5706,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Data Governance: retention, партиционирование</t>
+          <t>Feature flags для безопасного развития</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5726,22 +5731,22 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>S-100</t>
+          <t>S-099</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Соответствие требованиям хранения данных и юр. нормам</t>
+          <t>Включение функций на пилотные магазины без риска для сети</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Данные хранятся без явных политик TTL</t>
+          <t>Все изменения применяются глобально</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Нет утверждённых сроков хранения с юристами</t>
+          <t>Нет инфраструктуры feature flags</t>
         </is>
       </c>
     </row>
@@ -5753,7 +5758,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Нагрузочное тестирование 40K устройств</t>
+          <t>Data Governance: retention, партиционирование</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5778,39 +5783,39 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>S-101</t>
+          <t>S-100</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Подтверждение способности системы работать под расчётной нагрузкой</t>
+          <t>Соответствие требованиям хранения данных и юр. нормам</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Тесты только на малых объёмах данных</t>
+          <t>Данные хранятся без явных политик TTL</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Нет утверждённых профилей нагрузки</t>
+          <t>Нет утверждённых сроков хранения с юристами</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>v0.8 (P0: PLAN-001)</t>
+          <t>v0.9+</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Часовые пояса и календарь показов</t>
+          <t>Нагрузочное тестирование 40K устройств</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>🧭</t>
+          <t>⚪️</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5825,44 +5830,39 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>🧭 Требует решения (P0)</t>
+          <t>⚪ Не начато</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>S-102</t>
+          <t>S-101</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Корректное расписание во всех часовых поясах РФ с учётом праздников</t>
+          <t>Подтверждение способности системы работать под расчётной нагрузкой</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Только UTC/Moscow, без календаря исключений</t>
+          <t>Тесты только на малых объёмах данных</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>PLAN-001: решение владельца продукта — время по местному.</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>ADR: store-local time. P0 после ADR-018.</t>
+          <t>Нет утверждённых профилей нагрузки</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>v0.9+</t>
+          <t>v0.8 (P0: PLAN-001)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Channel Orchestrator / Adapter Layer</t>
+          <t>Часовые пояса и календарь показов</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5882,77 +5882,134 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>🧭 Требует решения</t>
+          <t>🧭 Требует решения (P0)</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>ADR требуется</t>
+          <t>S-102</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Единый слой адаптеров для KSO/Android/ESL/LED</t>
+          <t>Корректное расписание во всех часовых поясах РФ с учётом праздников</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>КСО-центричная архитектура</t>
+          <t>Только UTC/Moscow, без календаря исключений</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Нет ADR, нет абстракции адаптеров</t>
+          <t>PLAN-001: решение владельца продукта — время по местному.</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ADR: store-local time. P0 после ADR-018.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>v0.9+</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Channel Orchestrator / Adapter Layer</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>🧭</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>🧭 Требует решения</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>ADR требуется</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Единый слой адаптеров для KSO/Android/ESL/LED</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>КСО-центричная архитектура</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Нет ADR, нет абстракции адаптеров</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>v2.6</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>SIEM/Wazuh + ИБ-мониторинг</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>⚪️</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
         <is>
           <t>⚪ Не начато</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>S-092</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>Передача критичных событий в SIEM для ИБ</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>Логи只在 локальных файлах</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>Требуется согласование с ИБ-отделом</t>
         </is>

</xml_diff>

<commit_message>
G4-FIX-FU2: state/roadmap hygiene after durable AD settings
- PROJECT_STATE: Repository Checkpoint develop → 6144148 (G4-FIX-FU2)
- PROJECT_STATE: Next Active Workstream → G4-SERIES CLOSED
- PROJECT_STATE: residual note — durable proof is unit/mock-level
- PROJECT_STATE: NAS mirror expected → 6144148
- Roadmap technical row 52: removed stale 'honest stub'/'LDAPS deferred to v0.6+'
  → updated to reflect S-034 + C2 real LDAPS + G4 durable DB + bind_password env-only

Guard: 0 findings. No stale patterns remain.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -1812,22 +1812,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>✅ S-034 done (honest stub)</t>
+          <t>✅ S-034 + C2 real LDAPS + G4 PUT save (durable DB, migration 027)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Admin-web ADSettingsPage. GET/POST /auth/ad-settings with users.manage. Honest stub/disabled/configured status reporting. No secrets in responses.</t>
+          <t>Admin-web ADSettingsPage. PUT /auth/ad-settings (users.manage). Real LDAPS cert validation (C2, SHA 47e7d44). Durable DB persistence (migration 027, ADSettings model). bind_password env-only, never in API responses.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Real LDAPS wiring deferred to v0.6+.</t>
+          <t>adsettings.test UI-smoke (separate task). bind_password env-only (v2 feature).</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>v0.5: admin-facing AD status page. Real AD wiring deferred to v0.6+.</t>
+          <t>v0.6: admin AD settings save/persist/validate done — S-034 UI, C2 real LDAPS cert validation, G4 configure/save endpoint (durable DB). bind_password env-only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JOURNEY-001: advertiser.apply reachable + green UI-smoke
- Backend: audit FK fix — actor_user_id=str→str|None in create_audit_event
  (public endpoint can't provide valid user UUID)
- Migration 028: permissive INSERT RLS on advertiser_applications for public
- Admin-web: data-testid on PublicApplicationForm (8 fields + submit + consent)
- UI-smoke: test_uismoke__advertiser__apply green (public /become-advertiser → 201)
- Registry: advertiser.apply → reachable (9→10), blocked 31→30
- Roadmap: Управление рекламодателями row — advertiser.apply ✅
- PROJECT_STATE: JOURNEY-001 record, Next → advertiser.application_review

Backend: 18/18, Admin-web: 163/163, Smoke: 1/1
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3541,12 +3541,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>✅ (create_org) / ⚪️ (view/apply/review)</t>
+          <t>✅ (create_org / apply) / ⚪️ (view/review)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>✅ advertiser.create_org / ⚪️ остальные</t>
+          <t>✅ advertiser.create_org / ✅ advertiser.apply / ⚪️ остальные</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-002: advertiser.application_review reachable + green UI-smoke
- Admin-web: data-testid on advertiser applications table + review button
- UI-smoke: self-contained test (public submit → admin login → reviewing)
  Phase 1: /become-advertiser → submit public application
  Phase 2: login as break_glass_admin
  Phase 3: navigate /advertiser-applications → find app → Начать рассмотрение
  Phase 4: verify status «На рассмотрении»
- Registry: advertiser.application_review → reachable (10→11)
- Roadmap: Управление рекламодателями row — application_review ✅
- PROJECT_STATE: JOURNEY-002 record, Next → advertiser.invite
- NAS mirror: verified 53b3ad5

Backend BP-001: 18/18, Admin-web: 163/163, Smoke: 1/1, Guard: 0 findings
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3541,12 +3541,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>✅ (create_org / apply) / ⚪️ (view/review)</t>
+          <t>✅ (create_org / apply / application_review) / ⚪️ (view/review)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>✅ advertiser.create_org / ✅ advertiser.apply / ⚪️ остальные</t>
+          <t>✅ advertiser.create_org / ✅ advertiser.apply / ✅ advertiser.application_review / ⚪️ остальные</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-003: advertiser.invite reachable + green UI-smoke
- Frontend: data-testid on approve/invite-create buttons, invite status/token
- Admin-web tests: 11/11 (3 new invite tests: button visibility, token display, RBAC)
- UI-smoke: test_uismoke__advertiser__invite — self-contained public→review→approve→invite
- Registry: advertiser.invite → reachable, reachable 11→12, blocked 29→28
- Roadmap: Управление рекламодателями updated (invite ✅)
- PROJECT_STATE: JOURNEY-003, Next → self.login
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3541,17 +3541,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>✅ (create_org / apply / application_review) / ⚪️ (view/review)</t>
+          <t>✅ (create_org / apply / application_review / invite) / ⚪️ (view)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>✅ advertiser.create_org / ✅ advertiser.apply / ✅ advertiser.application_review / ⚪️ остальные</t>
+          <t>✅ advertiser.create_org / ✅ advertiser.apply / ✅ advertiser.application_review / ✅ advertiser.invite / ⚪️ остальные</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>🟠 Частично (create_org reachable, остальное без smoke)</t>
+          <t>🟠 Частично (create_org/apply/review/invite reachable, остальное без smoke)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-003-FU: state/roadmap hygiene after advertiser.invite
- PROJECT_STATE: JOURNEY-003 → ✅ RESOLVED, PS-001 checkpoint
- Next Active: self.login (unchanged)
- Roadmap row 3 (Вход сотрудников): убраны stale-claims
  campaign.create (G1) и advertiser.create_org (G3) — уже reachable
- guard: 0 findings
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3385,7 +3385,7 @@
           <t>❌ Нет self-service сброса пароля.
 ❌ Нет инвайт-писем для новых рекламодателей.
 Почему: базовый вход работает. Self-service onboarding — v0.8.
-❌ UI-TRUTH: blocked — campaign.create (G1), self.login, advertiser.create_org. UI-smoke отсутствует.</t>
+❌ UI-TRUTH: blocked — self.login (advertiser web login journey без UI-smoke). campaign.create (G1), advertiser.create_org (G3) — уже reachable.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Готово (S-048). Self-service сброс пароля — v0.8.</t>
+          <t>Готово (S-048). self.login — следующий journey из wave 1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JOURNEY-004: self.login reachable + green UI-smoke
- Advertiser-web: data-testid on AcceptInvitePage (password, submit, go-to-login)
- UI-smoke: test_uismoke__self__login — full cross-portal flow:
  public submit → admin review/approve → invite → accept → login → dashboard
- Registry: self.login → reachable, reachable 12→13, blocked 28→27
- Roadmap: Вход сотрудников (R3), Личный кабинет (R5) — self.login ✅
- PROJECT_STATE: JOURNEY-004, Next → user.create_advertiser
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3354,17 +3354,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ (self.login) / ⚪️ (reset-password)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ self.login / ⚪️ остальные</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>🟠 Бэкенд готов, UI-smoke нет</t>
+          <t>🟠 Частично (self.login reachable, self-service сброс пароля без smoke)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3479,12 +3479,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ (self.login) / ⚪️ (campaigns/reports)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ self.login / ⚪️ self.campaign_view / ⚪️ self.report_view</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-004-FU: state/roadmap hygiene + smoke URL portability
- PROJECT_STATE: JOURNEY-004 → ✅ RESOLVED, PS-001 checkpoint
- Roadmap R3/R5: убраны stale self.login blocked/next claims
- Smoke: UI_SMOKE_ADVERTISER_URL env override + fallback port+1
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3385,7 +3385,8 @@
           <t>❌ Нет self-service сброса пароля.
 ❌ Нет инвайт-писем для новых рекламодателей.
 Почему: базовый вход работает. Self-service onboarding — v0.8.
-❌ UI-TRUTH: blocked — self.login (advertiser web login journey без UI-smoke). campaign.create (G1), advertiser.create_org (G3) — уже reachable.</t>
+✅ self.login (JOURNEY-004) — рекламодатель принимает приглашение и входит в портал. UI-smoke зелёный, CI #29909590097.
+❌ self.campaign_view, self.report_view — без UI-smoke.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -3395,7 +3396,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Готово (S-048). self.login — следующий journey из wave 1.</t>
+          <t>Готово (S-048, JOURNEY-004). Self-service сброс пароля — v0.8.</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3490,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>🟠 Бэкенд готов, UI-smoke нет</t>
+          <t>🟠 Частично (self.login ✅, self.campaign_view/self.report_view без smoke)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-005: user.create_advertiser reachable + green UI-smoke
- UsersPage: data-testid on create form (username, display_name, org_id, submit, result); fix auto-close-on-success
- UI-smoke: test_uismoke__user__create_advertiser — login → Пользователи → Создать → fill → submit → verify OTP
- Vitest: 5 tests — hidden-without-perm, visible-with-perm, opens-form, success-result, error-state (admin-web 166→171)
- Registry: user.create_advertiser → reachable (13→14, blocked 27→26)
- Roadmap: R4 (Роли и права) updated
- Guard: roadmap-consistency-check → 0 findings
- Backend: no changes (POST /users/local-advertiser existed)
- Backend tests: 111/111
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3418,12 +3418,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ (user.create_advertiser / user.assign_roles)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>✅ user.assign_roles</t>
+          <t>✅ user.create_advertiser / ✅ user.assign_roles</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-006: advertiser.view reachable + green UI-smoke
- AdvertisersPage: data-testid on org rows, detail panel, overview fields, users tab
- UI-smoke: test_uismoke__advertiser__view — login → Рекламодатели → click ADV-001 → verify detail → users tab
- Vitest: 3 view tests (detail panel, users empty state, empty org list). admin-web 171→174
- Registry: advertiser.view → reachable (14→15, blocked 26→25)
- Roadmap: R6 updated — advertiser.view ✅
- Guard: roadmap-consistency-check → 0 findings
- Backend: no changes needed (endpoints existed)
- Smoke: 1 passed in 1.83s against real PostgreSQL
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3542,12 +3542,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>✅ (create_org / apply / application_review / invite) / ⚪️ (view)</t>
+          <t>✅ (create_org / apply / application_review / invite / view)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>✅ advertiser.create_org / ✅ advertiser.apply / ✅ advertiser.application_review / ✅ advertiser.invite / ⚪️ остальные</t>
+          <t>✅ advertiser.create_org / ✅ advertiser.apply / ✅ advertiser.application_review / ✅ advertiser.invite / ✅ advertiser.view</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-006-FU: wave 1 closure hygiene
PROJECT_STATE checkpoint fix: state/docs SHA 0346ea1 -> 12b34d9
NAS mirror: pending/7a6444f -> verified/12b34d9 (cron sync confirmed)
Roadmap R6: Итог -> ✅ Готово/Юзабельно (all 5 listed journeys green)
Roadmap R6 K11: stale 'остальные journeys без smoke' removed
Guard: 0 findings, 10 reachable UI features with smoke

docs-only — no product code changes.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3552,7 +3552,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>🟠 Частично (create_org/apply/review/invite reachable, остальное без smoke)</t>
+          <t>✅ Готово/Юзабельно</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ Все 5 listed journeys (create_org, apply, application_review, invite, view) reachable с зелёным UI-smoke.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>✅ Готово/Юзабельно частично: create_org работает, остальные journeys без UI-smoke.</t>
+          <t>Wave 1 complete. ✅ Все 5 listed journeys reachable с зелёным UI-smoke.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JOURNEY-007: self.apply_or_brief reachable + green UI-smoke
Backend: existed (BP-004 CampaignBrief — full CRUD + submit, scoped to advertiser org).
UI: data-testid on BriefCreatePage (9 fields + 2 buttons), BriefListPage (create btn),
     Layout nav-briefs sidebar link.
Smoke: test_uismoke__self__apply_or_brief — 1 passed 1.37s.
       Seed advertiser (advertiser_test) login → Заявки → Создать → fill → submit
       → detail page with title + status.
Vitest: 6 new tests (BriefListPage: empty/list/error, BriefCreatePage: form/render/
        validation/submit). advertiser-web 97→103 passed.
Registry: self.apply_or_brief → reachable (15→16 reachable, 25→24 blocked).
Roadmap: R5 'Личный кабинет' — UI/Юзер-стори updated, stale removed.
Guard: 0 findings, 11 reachable UI features.

No backend changes — endpoints existed and worked.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3480,12 +3480,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>✅ (self.login) / ⚪️ (campaigns/reports)</t>
+          <t>✅ (self.login / self.apply_or_brief) / ⚪️ (campaigns/reports)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>✅ self.login / ⚪️ self.campaign_view / ⚪️ self.report_view</t>
+          <t>✅ self.login / ✅ self.apply_or_brief / ⚪️ self.campaign_view / ⚪️ self.report_view</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -3506,11 +3506,9 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>❌ Рекламодатель не может сам утверждать кампании — только admin.
-❌ Нет биллинга/атрибуции.
-❌ Production UX audit отложен.
-Почему: self-service пилот работает. Полный production UX — после стабилизации backend.
-❌ UI-TRUTH: blocked — self.login, self.campaign_view, self.report_view. Advertiser-web не проходил UI-аудит.</t>
+          <t>✅ self.login (JOURNEY-004) + self.apply_or_brief (JOURNEY-007) reachable.
+❌ self.campaign_view, self.report_view — без UI-smoke.
+ℹ self.campaign_create — deferred по managed-first (План волн).</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -3520,7 +3518,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Production UX audit (deferred). Browser E2E (deferred).</t>
+          <t>JOURNEY-007 closed. Next: campaign.edit (Wave 2).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JOURNEY-008: campaign.edit reachable + green UI-smoke
Backend: existed (CampaignFlight/CampaignPlacement full CRUD + PATCH campaign).
UI: data-testid on tabs (tab-flights, tab-placements), flight form
    (flight-add-btn, flight-start, flight-end, flight-submit),
    placement form (placement-add-btn, placement-surface, placement-submit).
Smoke: test_uismoke__campaign__edit — 1 passed 2.33s.
       login → create campaign → flights tab → add flight → placements
       tab → add placement → verify both tables.
Registry: campaign.edit → reachable (16→17 reachable, 24→23 blocked).
Roadmap: R8 'Создание и редактирование' — UI/Юзер-стори updated.
Guard: 0 findings, 12 reachable UI features.

No backend changes — endpoints existed and worked.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3635,12 +3635,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>✅ (create) / ⚪️ (edit)</t>
+          <t>✅ (create / edit)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>✅ campaign.create / ⚪️ campaign.edit</t>
+          <t>✅ campaign.create / ✅ campaign.edit</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3662,12 +3662,8 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>❌ Нет календаря планирования.
-❌ Нет drag-and-drop.
-❌ UX/accessibility не завершены.
-❌ Нет браузерных E2E-тестов.
-✅ campaign.create (G1) — зелёный UI-smoke.
-❌ campaign.edit, campaign.submit, campaign.activate — UI-smoke отсутствует.</t>
+          <t>✅ campaign.create (G1) + campaign.edit (JOURNEY-008) — зелёный UI-smoke.
+❌ campaign.submit, campaign.activate — UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
docs: JOURNEY-008-FU — state/roadmap hygiene after campaign.edit
- PROJECT_STATE: Next Active Workstream JOURNEY-008 → JOURNEY-009 (creative.upload)
- PROJECT_STATE: Repository Checkpoint State/Docs SHA 9790904 → d2dddc8
- PROJECT_STATE: NAS mirror develop=da37ec3 → d2dddc8
- PROJECT_STATE: ROADMAP-DONE-GATE-001 historical entry annotated as superseded
- Roadmap R8 Итог: 'edit не reachable' → 'campaign.submit/activate без smoke'
- Roadmap R5 Следующий шаг: JOURNEY-007 → JOURNEY-008 closed, next creative.upload
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3518,7 +3518,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>JOURNEY-007 closed. Next: campaign.edit (Wave 2).</t>
+          <t>JOURNEY-008 closed. Next: creative.upload (Wave 2).</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>🟠 Частично (edit не reachable)</t>
+          <t>🟠 Частично (campaign.submit/activate без smoke)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-009: creative.upload reachable + green UI-smoke (12.59s)
Backend: existed (presigned URL → MinIO → complete-upload).
Admin-web: 7 data-testid, advertiser_organization_id fix in handleCreateAsset.
Smoke: test_uismoke__creative__upload → create campaign → add library → attach → upload file.
Vitest: admin-web 174/174, no regressions.
Registry: creative.upload → reachable (18 reachable, 22 blocked).
Roadmap: Row 10 creative.upload ✅, guard 0 findings.
Next: JOURNEY-010 — inventory.simulate.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3756,17 +3756,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ (upload) / ⚪️ (moderation)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ creative.upload / ⚪️ creative.moderate_approve / ⚪️ creative.moderate_reject</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>🟠 Бэкенд готов, UI-smoke нет</t>
+          <t>🟠 Частично (moderation approve/reject без smoke)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">

</xml_diff>

<commit_message>
WAVE3-CLOSURE-001: Wave 3 canon closure — plan, registry, roadmap, state
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3635,17 +3635,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>✅ (create / edit)</t>
+          <t>✅ (create / edit / submit)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>✅ campaign.create / ✅ campaign.edit</t>
+          <t>✅ campaign.create / ✅ campaign.edit / ✅ campaign.submit</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>🟠 Частично (campaign.submit/activate без smoke)</t>
+          <t>🟠 Частично (campaign.activate/pause без smoke)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3662,8 +3662,8 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>✅ campaign.create (G1) + campaign.edit (JOURNEY-008) — зелёный UI-smoke.
-❌ campaign.submit, campaign.activate — UI-smoke отсутствует.</t>
+          <t>✅ campaign.create (G1) + campaign.edit (JOURNEY-008) + campaign.submit (JOURNEY-012) — зелёный UI-smoke.
+❌ campaign.activate, campaign.pause — UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -3690,22 +3690,22 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>🟠</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ (approve / reject)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ campaign.approve / ✅ campaign.reject</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>🟠 Бэкенд готов, UI-smoke нет</t>
+          <t>✅ Готово/Юзабельно</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3722,9 +3722,10 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>❌ Рекламодатель не может сам утверждать — только отправляет.
-Почему: это осознанное ограничение безопасности.
-❌ UI-TRUTH: blocked — campaign.approve, campaign.reject. UI-smoke отсутствует.</t>
+          <t>✅ campaign.approve + campaign.reject (JOURNEY-013) — полный pipeline с зелёным UI-smoke.
+✅ Backend: S-079 inventory commit/release, audit+outbox.
+✅ Admin-web: approve/reject кнопки, rejection reason display.
+❌ Рекламодатель не может сам утверждать — осознанное ограничение безопасности.</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
@@ -3734,7 +3735,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>После campaign UI (S-009c).</t>
+          <t>JOURNEY-013 closed. Next: campaign.activate/pause (Wave 4).</t>
         </is>
       </c>
     </row>
@@ -3751,22 +3752,22 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>🟠</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>✅ (upload) / ⚪️ (moderation)</t>
+          <t>✅ (upload / moderate_approve / moderate_reject)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>✅ creative.upload / ⚪️ creative.moderate_approve / ⚪️ creative.moderate_reject</t>
+          <t>✅ creative.upload / ✅ creative.moderate_approve / ✅ creative.moderate_reject</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>🟠 Частично (moderation approve/reject без smoke)</t>
+          <t>✅ Готово/Юзабельно</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3783,8 +3784,9 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Malware scan, transcoding, CDN — отложены.
-❌ UI-TRUTH: blocked — creative.upload, creative.moderate_approve, creative.moderate_reject.</t>
+          <t>✅ creative.upload (JOURNEY-009) + creative.moderate_approve + creative.moderate_reject (JOURNEY-011) — все 3 journeys с зелёным UI-smoke.
+Malware scan, transcoding, CDN — отложены.
+✅ Backend: S-036 approve/reject endpoints, moderation queue, audit events, perm creatives.moderate.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -3794,8 +3796,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Malware scan, transcoding, manual moderation — отложены.
-Работает для пилота.</t>
+          <t>JOURNEY-009/JOURNEY-011 closed. Malware scan — deferred.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JOURNEY-014-DOCS: canon — registry 24→26 reachable, roadmap row 8 ✅, PROJECT_STATE
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3635,17 +3635,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>✅ (create / edit / submit)</t>
+          <t>✅ (create / edit / submit / activate / pause)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>✅ campaign.create / ✅ campaign.edit / ✅ campaign.submit</t>
+          <t>✅ campaign.create / ✅ campaign.edit / ✅ campaign.submit / ✅ campaign.activate / ✅ campaign.pause</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>🟠 Частично (campaign.activate/pause без smoke)</t>
+          <t>✅ Готово/Юзабельно</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3662,8 +3662,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>✅ campaign.create (G1) + campaign.edit (JOURNEY-008) + campaign.submit (JOURNEY-012) — зелёный UI-smoke.
-❌ campaign.activate, campaign.pause — UI-smoke отсутствует.</t>
+          <t>✅ Все 5 listed journeys (create, edit, submit, activate, pause) reachable с зелёным UI-smoke.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-014-FU: rollback — activate/pause → blocked (MinIO presigned URL), honest status
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3635,17 +3635,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>✅ (create / edit / submit / activate / pause)</t>
+          <t>✅ (create / edit / submit)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>✅ campaign.create / ✅ campaign.edit / ✅ campaign.submit / ✅ campaign.activate / ✅ campaign.pause</t>
+          <t>✅ campaign.create / ✅ campaign.edit / ✅ campaign.submit</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>✅ Готово/Юзабельно</t>
+          <t>🟠 Частично (campaign.activate/pause — smoke written but not proven, JOURNEY-014-FU)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3662,7 +3662,8 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>✅ Все 5 listed journeys (create, edit, submit, activate, pause) reachable с зелёным UI-smoke.</t>
+          <t>✅ campaign.create (G1) + campaign.edit (JOURNEY-008) + campaign.submit (JOURNEY-012) — зелёный UI-smoke.
+❌ campaign.activate, campaign.pause — backend/UI/vitest готовы, smoke написан но не прогнан (MinIO presigned URL, JOURNEY-014-FU).</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-014-FU2: campaign.activate/pause → reachable
Smoke proof: activate (13.0s) + pause (8.1s) green on real stack.
Pause test fix: non-overlapping inventory window (Jan 2027 vs Dec 2026).

Registry: 24→26 reachable, 16→14 blocked.
Roadmap row 8: 🟠 → ✅ Готово/Юзабельно.
Consistency guard: 0 findings (21 UI reachable, all smokes found).
PROJECT_STATE: JOURNEY-014 ✅ RESOLVED.
Next: emergency.activate/deactivate (Wave 4).
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3635,17 +3635,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>✅ (create / edit / submit)</t>
+          <t>✅ (create / edit / submit / activate / pause)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>✅ campaign.create / ✅ campaign.edit / ✅ campaign.submit</t>
+          <t>✅ campaign.create / ✅ campaign.edit / ✅ campaign.submit / ✅ campaign.activate / ✅ campaign.pause</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>🟠 Частично (campaign.activate/pause — smoke written but not proven, JOURNEY-014-FU)</t>
+          <t>✅ Готово/Юзабельно</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3662,8 +3662,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>✅ campaign.create (G1) + campaign.edit (JOURNEY-008) + campaign.submit (JOURNEY-012) — зелёный UI-smoke.
-❌ campaign.activate, campaign.pause — backend/UI/vitest готовы, smoke написан но не прогнан (MinIO presigned URL, JOURNEY-014-FU).</t>
+          <t>✅ campaign.create (G1) + campaign.edit (JOURNEY-008) + campaign.submit (JOURNEY-012) + campaign.activate + campaign.pause (JOURNEY-014-FU2) — зелёный UI-smoke.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-015: registry/roadmap/state — emergency → reachable
Registry: 26→28 reachable, 14→12 blocked.
Roadmap row 26: UI ✅ (activate/deactivate), Story ✅.
Consistency guard: 0 findings (23 UI reachable).
PROJECT_STATE: JOURNEY-015 ✅ RESOLVED.
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -4628,12 +4628,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ (activate / deactivate)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ emergency.activate / ✅ emergency.deactivate</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-016: self.campaign_view reachable + green smoke (1.99s) — canon sync (registry 29/11, plan 🟢, roadmap, user-journeys, PROJECT_STATE)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3485,12 +3485,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>✅ self.login / ✅ self.apply_or_brief / ⚪️ self.campaign_view / ⚪️ self.report_view</t>
+          <t>✅ self.login / ✅ self.apply_or_brief / ✅ self.campaign_view / ⚪️ self.report_view</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>🟠 Частично (self.login ✅, self.campaign_view/self.report_view без smoke)</t>
+          <t>🟠 Частично (self.login ✅, self.campaign_view ✅, self.report_view без smoke)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-017 — device.health_view reachable + green smoke
- Schema DeviceOut: +health_state/last_heartbeat_at/runtime_version/player_version
- Admin-web DeviceHealthPage: health columns + 10 data-testid + formatApiError
- Vitest: +9 tests (device-health.test.tsx), total 215/215
- Smoke: test_uismoke__device__health_view — 8.68s PASSED
- Canon: registry 30/10, roadmap row 44 updated, plan Wave 5, user-journeys Happy-path
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -5550,22 +5550,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ Бэкенд: EDGE-004 heartbeat + S-070 fleet list/summary</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ UI: DeviceHealthPage — health_state badge, heartbeat, версии (admin-web)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ device.health_view — зелёный UI-smoke + Happy-path 6 шагов</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>🟠 Частично: device.health_view ✅, audit.view / self.report_view — blocked</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-020: adsettings.test reachable + green UI-smoke
Backend: already existed (POST /auth/ad-settings/test, users.manage).
Admin-web ADSettingsPage:
  - Added data-testid on test result (adsettings-test-success/error/loading)
  - Loading indicator during test
  - Test button already existed (adsettings-test-btn)
Vitest: 9/9 (added 4 test connection flow tests: result/ok/no-secrets/loading)
Smoke: break_glass_admin → AD settings → test → controlled failure (1.41s)
Roadmap: Настройки AD/LDAPS → ✅ Готово/Юзабельно (configure + test green)
Next: Wave 6 — user.reset_password (JOURNEY-021 candidate)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -4822,12 +4822,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>✅ (adsettings.configure — green smoke)</t>
+          <t>✅ (adsettings.configure + adsettings.test — green smokes)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>🟠 Частично (adsettings.test без smoke)</t>
+          <t>✅ Готово/Юзабельно</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">

</xml_diff>

<commit_message>
JOURNEY-021: user.reset_password reachable + green UI-smoke
Backend: already existed (POST /users/{id}/reset-password, users.manage).
Admin-web UsersPage: data-testid on reset flow (open/confirm/success/error/otp).
Vitest: 7/7 (added 4 reset tests: RBAC visibility, modal, API call, error).
Smoke: create throwaway user → find row → reset → OTP via response (2.87s).
Does NOT mutate shared seed credentials (break_glass_admin, advertiser_test).
Roadmap: RBAC row updated (user.reset_password ✅).
Next: Wave 6 — user.deactivate (JOURNEY-022 candidate)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3423,7 +3423,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>✅ user.create_advertiser / ✅ user.assign_roles</t>
+          <t>✅ user.create_advertiser / ✅ user.assign_roles / ✅ user.reset_password</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -3448,7 +3448,8 @@
         <is>
           <t>Нет UI для создания рекламодателей (user.create_advertiser) и сброса паролей.
 ✅ user.assign_roles (G2) — зелёный UI-smoke.
-❌ user.create_advertiser, user.reset_password — UI-smoke отсутствует.</t>
+✅ user.reset_password (JOURNEY-021) — зелёный UI-smoke.
+❌ user.create_advertiser — UI-smoke отсутствует.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(REGISTRY-TRUTH-001): brand/contract smokes accounted + Direction C guard
Registry blind spot fixed:
- advertiser.brand_crud, advertiser.contract_crud, advertiser.legal_requisites
  now in feature-registry.yaml (48 features, 38 reachable).
- Roadmap 'Управление рекламодателями' updated — all 9 journeys accounted.

Direction C — every UI-smoke must have exactly one registry reference:
- SMOKE-ORPHAN: smoke with 0 registry refs
- SMOKE-DUPLICATE: smoke with >1 registry refs

Tamper proof: brand_crud smoke→NONEXISTENT → SMOKE-ORPHAN detected.

Verification:
- Guard --strict: 0 findings
- rg confirmation: both smokes in registry
- rg stale claims: 0 matches
- Product code untouched
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3541,12 +3541,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>✅ (create_org / apply / application_review / invite / view)</t>
+          <t>✅ (create_org / apply / application_review / invite / view / contact_crud / brand_crud / contract_crud / legal_requisites)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>✅ advertiser.create_org / ✅ advertiser.apply / ✅ advertiser.application_review / ✅ advertiser.invite / ✅ advertiser.view</t>
+          <t>✅ advertiser.create_org / ✅ advertiser.apply / ✅ advertiser.application_review / ✅ advertiser.invite / ✅ advertiser.view / ✅ advertiser.contact_crud / ✅ advertiser.brand_crud / ✅ advertiser.contract_crud / ✅ advertiser.legal_requisites</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>

<commit_message>
docs: ROADMAP-RELEASE-SYNC-002 — roadmap truth + owner release decision prep
- registry truth 58/49/9 + license.* gap corrections (enforce A1+A2 ready, A3/A4/Layer2 pending)
- pre-pilot plan: counts 58/49/9, workstreams after R3, reachable/pilot-ready/production-ready split
- roadmap.xlsx: commerce + theme + licensing rows, campaign.complete, inventory stale fix
- release delta main vs develop + production UNKNOWN/NOT TRACKED + decision matrix (A/B/C)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -3228,7 +3228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3658,7 +3658,8 @@
         <is>
           <t>✅ Backend: полный CRUD кампаний (7 endpoints), пролёты, размещения, креативы.
 ✅ Admin-web: список с фильтром, мастер создания, 5 вкладок (пролёты, размещения, креативы+upload, согласование, PoP-отчёты).
-✅ Advertiser-web: создание/редактирование черновиков.</t>
+✅ Advertiser-web: создание/редактирование черновиков.
+✅ campaign.complete — авто-завершение кампании по концу рейса (service, behavioral proof LIFECYCLE-COMPLETE-001-FU, без UI journey).</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -4501,7 +4502,7 @@
           <t>❌ Нет визуальной сетки/календаря инвентаря.
 ❌ Нет прогноза доступности.
 ❌ Нет competitor separation (нет данных о категориях).
-❌ UI-TRUTH: blocked — inventory.simulate, inventory.rule_create. UI-smoke отсутствует.</t>
+✅ inventory.simulate + inventory.rule_create — reachable, зелёный UI-smoke (JOURNEY-010, JOURNEY-023).</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
@@ -4528,22 +4529,22 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>✅ (simulate)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ inventory.simulate</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>⚪ Не начато</t>
+          <t>✅ Готово/Юзабельно</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -6011,6 +6012,297 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Коммерция (Commerce Contour 2)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>v0.10 (R3→R4)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Коммерция: тарифы и прайс-листы</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅ (tariff_manage / price_list_manage)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅ commerce.tariff_manage / ✅ commerce.price_list_manage</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>✅ Готово/Юзабельно</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Продажа рекламного инвентаря по тарифам: прайс-листы, версии, единицы цены. Основа коммерческих заказов.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>✅ CRUD тарифов + price items через UI; зелёный smoke (commerce__tariff_manage).</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>COMMERCE-CONTUR2-001A3a — MVP closed.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>v0.10 (R3→R4)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Коммерция: заказы и бронирование</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅ (order_create)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅ commerce.order_create / ✅ commerce.offer_generate / ✅ commerce.booking / ✅ commerce.payment_status / ✅ commerce.order_close</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>✅ Готово/Юзабельно</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Коммерческий цикл: заказ → коммерческое предложение → бронирование → оплата → закрытие.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅ order create + lines/total + статусные переходы (draft→offered→booked→confirmed→closed) через UI; зелёный smoke (commerce__order_create). Server-derived quantity_days (без нулевых цен).</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>COMMERCE-CONTUR2-001A3b/c — MVP closed.</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Интерфейс и доступность</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>v0.10 (R3→R4)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Переключение темы (light/dark)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>✅ (theme_switch)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>✅ system.theme_switch</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>✅ Готово/Юзабельно</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Доступный переключатель светлой/тёмной темы; выбор переживает reload.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>✅ Toggle light/dark через semantic tokens (tokens.css), aria-label, keyboard usable; зелёный smoke (system__theme_switch).</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>THEME-SWITCH-001B — доступность + переопределение semantic tokens.</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Лицензирование (EPIC-L)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>v0.10+ (EPIC-L)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Лицензирование (seat ledger)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>🟠</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>⚪️</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>🔒 Заблокировано (A3+A4 pending, Layer 2)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Ограничение числа устройств лицензией (seat ledger) и enforcement при enrollment.</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>✅ A1 (schema/migration + read model + dev-ingest) и A2 (enrollment choke-point + FOR UPDATE + reconciliation) — behavioral/concurrency/tamper proof зелёные.</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>❌ A3 (seat release при decommission), A4 (report/peak_seats_for_month), Layer 2 (signed-license upload/view + UI). license.* остаётся blocked в registry.</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>EPIC-L Layer 1 не закрыт — A1+A2 готовы, A3+A4 нет.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>EPIC-L-SEAT-LEDGER-001A3.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: EPIC-L-SEAT-LEDGER-001A4 closure — Layer 1 closed (registry 58/52/6)
</commit_message>
<xml_diff>
--- a/docs/product/roadmap-s020-2026-07-10.xlsx
+++ b/docs/product/roadmap-s020-2026-07-10.xlsx
@@ -6013,7 +6013,6 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
           <t>Коммерция (Commerce Contour 2)</t>
@@ -6024,14 +6023,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6148,7 +6139,6 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
           <t>Интерфейс и доступность</t>
@@ -6159,14 +6149,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6226,7 +6208,6 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
           <t>Лицензирование (EPIC-L)</t>
@@ -6237,14 +6218,6 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6259,22 +6232,22 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>🟠</t>
+          <t>✅ (Layer 1)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>⚪️</t>
+          <t>⚪️ (Layer 2 UI)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>✅ license.enforce / ✅ license.seat_release / ✅ license.report (service, behavioral proof)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>🔒 Заблокировано (A3+A4 pending, Layer 2)</t>
+          <t>🟠 Частично (Layer 1 reachable: enforce/seat_release/report; Layer 2 view/upload blocked)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -6284,22 +6257,22 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>✅ A1 (schema/migration + read model + dev-ingest) и A2 (enrollment choke-point + FOR UPDATE + reconciliation) — behavioral/concurrency/tamper proof зелёные.</t>
+          <t>✅ A1 ledger + A2 enrollment choke-point + A3 decommission release + A4 report API/reconciliation. license.enforce/seat_release/report reachable (service, behavioral proof). GET /licenses/report.</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>❌ A3 (seat release при decommission), A4 (report/peak_seats_for_month), Layer 2 (signed-license upload/view + UI). license.* остаётся blocked в registry.</t>
+          <t>❌ Layer 2: signed .lic upload, offline Ed25519 verify, kid/CRL, license UI. license.view/license.upload blocked.</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>EPIC-L Layer 1 не закрыт — A1+A2 готовы, A3+A4 нет.</t>
+          <t>EPIC-L Layer 1 closed. Layer 2 (signed-license) — next.</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>EPIC-L-SEAT-LEDGER-001A3.</t>
+          <t>EPIC-L-SIGNED-LICENSE-002 (Layer 2).</t>
         </is>
       </c>
     </row>

</xml_diff>